<commit_message>
Add round 4 (Glasgow + Edinburgh) to Oct–Nov Track B digest
Adds 8 events (GlasGLOW, Core., Pop Mutations x Tiny Changes, Edinburgh's
Christmas, Storytelling Festival, Edinburgh Short Film Festival, Skindred
Birmingham and Alexandra Palace dates) and updates coverage and gaps.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_10.15-11.15.xlsx
+++ b/data/UK_Events_TrackB_10.15-11.15.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1317,67 +1317,67 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>Reel Talk Club</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
+          <t>Edinburgh Short Film Festival（第 16 届）</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>Edinburgh（多个场地）</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
+          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐节)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>同步发伦敦6校</t>
+          <t>同步发爱丁堡2校</t>
         </is>
       </c>
       <c r="N12" s="2" t="n"/>
@@ -1400,12 +1400,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1415,17 +1415,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>年轻人娱乐(烟花/音乐节)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London); St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1435,27 +1435,27 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>同步发伦敦6校（RCA 优先）</t>
+          <t>同步发伦敦6校</t>
         </is>
       </c>
       <c r="N13" s="2" t="n"/>
@@ -1473,37 +1473,37 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Snack Finds &amp; Picks; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London); St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1513,27 +1513,27 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>同步发 Snack Finds &amp; Picks、伯明翰3校</t>
+          <t>同步发伦敦6校（RCA 优先）</t>
         </is>
       </c>
       <c r="N14" s="2" t="n"/>
@@ -1551,37 +1551,37 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Snack Finds &amp; Picks</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>31 Oct 2026（周六）18:30</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1591,27 +1591,27 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>同步发 UK Food Lovers</t>
+          <t>同步发伦敦6校</t>
         </is>
       </c>
       <c r="N15" s="2" t="n"/>
@@ -1629,17 +1629,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1649,17 +1649,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>年轻人娱乐(Live Music/金属)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Harper Adams Campus Life; Wolverhampton Freshers Hub 2026</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1669,27 +1669,27 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>同步发 Harper Adams、Wolverhampton</t>
+          <t>同步发格拉斯哥3校</t>
         </is>
       </c>
       <c r="N16" s="2" t="n"/>
@@ -1707,67 +1707,67 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>MCM Comic Con London（October 2026）</t>
+          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
+          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>23–25 Oct 2026</t>
+          <t>13–14 Nov 2026</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(游戏/动漫/流行文化)</t>
+          <t>年轻人娱乐(Live Music/独立音乐)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>The Gaming Corner</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
+          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
+          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
+          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第5名</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发格拉斯哥3校</t>
         </is>
       </c>
       <c r="N17" s="2" t="n"/>
@@ -1785,17 +1785,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
+          <t>Skindred "You Got This" 巡演 伯明翰站</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
+          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1805,47 +1805,47 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
+          <t>30 Oct 2026（周五）</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Reel Talk Club</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
+          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
+          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
+          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第6名</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发伯明翰3校</t>
         </is>
       </c>
       <c r="N18" s="2" t="n"/>
@@ -1863,17 +1863,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>UK Food Lovers</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Frieze London &amp; Frieze Masters 2026</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>The Regent's Park, London</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1883,17 +1883,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(艺术/展览)</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Snack Finds &amp; Picks; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1903,27 +1903,27 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>RCA 优先推</t>
+          <t>同步发 Snack Finds &amp; Picks、伯明翰3校</t>
         </is>
       </c>
       <c r="N19" s="2" t="n"/>
@@ -1941,37 +1941,37 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Snack Finds &amp; Picks</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐节)</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>UK Food Lovers; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1981,27 +1981,27 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发 UK Food Lovers</t>
         </is>
       </c>
       <c r="N20" s="2" t="n"/>
@@ -2019,67 +2019,67 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Day Trip Buddies</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>年轻人娱乐(烟花) + 一日游</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>Harper Adams Campus Life; Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>第5名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边</t>
+          <t>同步发 Harper Adams、Wolverhampton</t>
         </is>
       </c>
       <c r="N21" s="2" t="n"/>
@@ -2102,62 +2102,62 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
+          <t>MCM Comic Con London（October 2026）</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
+          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）11:00–15:30</t>
+          <t>23–25 Oct 2026</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(城市传统活动)</t>
+          <t>兴趣类(游戏/动漫/流行文化)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
+          <t>The Gaming Corner</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>第6名</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>免费</t>
         </is>
       </c>
       <c r="N22" s="2" t="n"/>
@@ -2175,17 +2175,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>英格兰 vs 澳大利亚（Nations Championship 橄榄球）</t>
+          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
+          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2195,17 +2195,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）</t>
+          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>运动户外(观赛)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Reel Talk Club</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2215,22 +2215,22 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>RFU 官方公布的国家队主场赛，是新赛事 Nations Championship 的首届</t>
+          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship ; https://allianzstadiumtwickenham.com/nations-championship</t>
+          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>St Mary's 是体育强校，球场就在家门口；⚠️国家队比赛票价偏高</t>
+          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -2253,32 +2253,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>英格兰 vs 日本（Nations Championship 橄榄球）</t>
+          <t>Frieze London &amp; Frieze Masters 2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
+          <t>The Regent's Park, London</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）</t>
+          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>运动户外(观赛)</t>
+          <t>兴趣类(艺术/展览)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2293,27 +2293,27 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>RFU 官方公布的国家队主场赛</t>
+          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship</t>
+          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>对日本这场的票通常比对新西兰、澳大利亚便宜，更适合学生；⚠️票价还是要看一下</t>
+          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RCA 优先推</t>
         </is>
       </c>
       <c r="N24" s="2" t="n"/>
@@ -2331,17 +2331,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2351,17 +2351,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>年轻人娱乐(烟花/音乐节)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew; 伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2371,22 +2371,22 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2409,17 +2409,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Richmond Family Fireworks</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Richmond Athletic Ground, Twickenham Road, Richmond TW9 2SF</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2429,47 +2429,47 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>⚠️待核实：一个来源写 1 Nov，另一个写 5–7 Nov 2026</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>年年举办的本地烟花会（Richmond Athletic Association 主办）；2026 年日期各来源说法不一，所以降级</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.rag-events.co.uk/major-public-events-at-the-rag/richmond-family-fireworks/ ; https://chiswicktoday.co.uk/chiswick-fireworks-bonfire-night/</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>离 St Mary's 很近；确认日期之后再推</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第5名</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>⚠️日期待核实</t>
+          <t>RCA Battersea 校区就在旁边</t>
         </is>
       </c>
       <c r="N26" s="2" t="n"/>
@@ -2487,17 +2487,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -2507,17 +2507,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>14 Nov 2026（周六）11:00–15:30</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>本地生活类(城市传统活动)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers; Snack Finds &amp; Picks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2527,27 +2527,27 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第6名</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>免费</t>
         </is>
       </c>
       <c r="N27" s="2" t="n"/>
@@ -2565,62 +2565,62 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Birmingham Big Wheel &amp; Ice Rink（Centenary Square）</t>
+          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Centenary Square, Birmingham</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>5 Nov 2026 – 3 Jan 2027，每天 10:00–22:00</t>
+          <t>31 Oct 2026（周六）18:30</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(滑冰/游乐)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>跟圣诞市集同期，市集官方配套项目，年年举办；没有售票数据</t>
+          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham-now.co.uk/news/26551457.birmingham-frankfurt-christmas-market-2026---need-know/</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>BCU 主校区附近，适合宿舍、群友组团去滑冰</t>
+          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第7名</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -2643,57 +2643,57 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Harper Adams Campus Life</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>英格兰 vs 澳大利亚（Nations Championship 橄榄球）</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>8 Nov 2026（周日）</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>运动户外(观赛)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies; Wolverhampton Freshers Hub 2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>RFU 官方公布的国家队主场赛，是新赛事 Nations Championship 的首届</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship ; https://allianzstadiumtwickenham.com/nations-championship</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>St Mary's 是体育强校，球场就在家门口；⚠️国家队比赛票价偏高</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2721,62 +2721,62 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Wolverhampton Freshers Hub 2026</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>英格兰 vs 日本（Nations Championship 橄榄球）</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>14 Nov 2026（周六）</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>运动户外(观赛)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies; Harper Adams Campus Life</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>RFU 官方公布的国家队主场赛</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>对日本这场的票通常比对新西兰、澳大利亚便宜，更适合学生；⚠️票价还是要看一下</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -2799,62 +2799,62 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>University of Lancaster</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Capernwray 湖泊公开水域游泳（Lake Swim）</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>运动户外(游泳)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Swim Wave Tribe</t>
+          <t>Live Music Crew; 伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>仅见于 Outdoor Swimmer 杂志活动日历；主办方未核实（疑为 T2 Events，他们在该场地办过比赛）；无报名数据</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://outdoorswimmer.com/events/ ; https://www.t2.events/our-events/capernwray-open-water-swim/</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>窗口内极少数的户外游泳活动，10 月底水温很低，只适合有冷水经验的人；离 Lancaster 大学约 10 公里</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -2877,17 +2877,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>The University of Manchester</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
+          <t>Richmond Family Fireworks</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Islington Mill, James Street, Salford</t>
+          <t>Richmond Athletic Ground, Twickenham Road, Richmond TW9 2SF</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2897,47 +2897,47 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:00–24:00</t>
+          <t>⚠️待核实：一个来源写 1 Nov，另一个写 5–7 Nov 2026</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体 + 社交类(女性)</t>
+          <t>年轻人娱乐(烟花)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner; Reel Talk Club</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
+          <t>年年举办的本地烟花会（Richmond Athletic Association 主办）；2026 年日期各来源说法不一，所以降级</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
+          <t>https://www.rag-events.co.uk/major-public-events-at-the-rag/richmond-family-fireworks/ ; https://chiswicktoday.co.uk/chiswick-fireworks-bonfire-night/</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
+          <t>离 St Mary's 很近；确认日期之后再推</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⚠️日期待核实</t>
         </is>
       </c>
       <c r="N32" s="2" t="n"/>
@@ -2955,62 +2955,62 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>The University of Manchester</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：Season of the Witch 系列活动</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Manchester 多个场地</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>社交类(女性) + 兴趣类(手工)</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner</t>
+          <t>UK Food Lovers; Snack Finds &amp; Picks</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Manchester's Finest 收录；系列里有 Craft &amp; Coven 手工夜、Pendle 女巫审判主题徒步等；没有单场售票数据</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://www.manchestersfinest.com/events/girl-gang-mcr-season-of-the-witch/ ; https://girlgangmcr.com/upcoming-events/</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>窗口内有多场可选；Pendle 徒步的具体日期没搜到，推之前要看官网确认单场日期</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -3033,62 +3033,62 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>The University of Manchester</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Lonely Girls Club Manchester 活动（10/27 场）</t>
+          <t>Birmingham Big Wheel &amp; Ice Rink（Centenary Square）</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Manchester（场地待公布）</t>
+          <t>Centenary Square, Birmingham</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>27 Oct 2026（周二）</t>
+          <t>5 Nov 2026 – 3 Jan 2027，每天 10:00–22:00</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>社交类(女性交友)</t>
+          <t>年轻人娱乐(滑冰/游乐)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>成熟的女性交友组织（有 Wikipedia 词条），London+Manchester 成员约 5.5 万（这是社群规模，不代表到场人数）；这场的具体内容官网写"即将公布"</t>
+          <t>跟圣诞市集同期，市集官方配套项目，年年举办；没有售票数据</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.llgc.co.uk/collections/manchester</t>
+          <t>https://www.birmingham-now.co.uk/news/26551457.birmingham-frankfurt-christmas-market-2026---need-know/</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>票价 £8.95，便宜，专为一个人来交朋友设计；活动内容没公布，推之前再看一眼</t>
+          <t>BCU 主校区附近，适合宿舍、群友组团去滑冰</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
@@ -3103,6 +3103,1098 @@
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Skindred "You Got This" 巡演 伯明翰站</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>30 Oct 2026（周五）</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="n"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Harper Adams Campus Life</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花) + 一日游</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Day Trip Buddies; Wolverhampton Freshers Hub 2026</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="n"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Wolverhampton Freshers Hub 2026</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花) + 一日游</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Day Trip Buddies; Harper Adams Campus Life</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="n"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>University of Lancaster</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Capernwray 湖泊公开水域游泳（Lake Swim）</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct 2026</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>运动户外(游泳)</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Swim Wave Tribe</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>仅见于 Outdoor Swimmer 杂志活动日历；主办方未核实（疑为 T2 Events，他们在该场地办过比赛）；无报名数据</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>https://outdoorswimmer.com/events/ ; https://www.t2.events/our-events/capernwray-open-water-swim/</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>窗口内极少数的户外游泳活动，10 月底水温很低，只适合有冷水经验的人；离 Lancaster 大学约 10 公里</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n"/>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>The University of Manchester</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Islington Mill, James Street, Salford</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct 2026（周六）18:00–24:00</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>电影/媒体 + 社交类(女性)</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Girls' Corner; Reel Talk Club</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="n"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>The University of Manchester</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Girl Gang MCR：Season of the Witch 系列活动</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Manchester 多个场地</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>city_only</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>社交类(女性) + 兴趣类(手工)</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Girls' Corner</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Manchester's Finest 收录；系列里有 Craft &amp; Coven 手工夜、Pendle 女巫审判主题徒步等；没有单场售票数据</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.manchestersfinest.com/events/girl-gang-mcr-season-of-the-witch/ ; https://girlgangmcr.com/upcoming-events/</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>窗口内有多场可选；Pendle 徒步的具体日期没搜到，推之前要看官网确认单场日期</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>The University of Manchester</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Lonely Girls Club Manchester 活动（10/27 场）</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Manchester（场地待公布）</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>city_only</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>27 Oct 2026（周二）</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>社交类(女性交友)</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Girls' Corner</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>成熟的女性交友组织（有 Wikipedia 词条），London+Manchester 成员约 5.5 万（这是社群规模，不代表到场人数）；这场的具体内容官网写"即将公布"</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.llgc.co.uk/collections/manchester</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>票价 £8.95，便宜，专为一个人来交朋友设计；活动内容没公布，推之前再看一眼</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="n"/>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>itison GlasGLOW 2026：Zombie Zoo 万圣节灯光夜游</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Glasgow Botanic Gardens, 730 Great Western Road, Glasgow G12 0UE</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>⚠️起始日两种说法：16 Oct 或 24 Oct 开始，1–2 Nov 结束（24 Oct–1 Nov 两种说法都覆盖）</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(沉浸式/万圣节)</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>第 8 年举办；自称英国最大的万圣节活动；往年曾因需求大加售数千张票（Scottish Daily Express 报道）</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.itison.com/glasglow ; https://www.glasgowworld.com/news/glasglow-botanic-gardens-dates-5290284 ; https://www.scottishdailyexpress.co.uk/news/scottish-news/glasglow-botanic-gardens-thousands-extra-30877210</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>格拉斯哥万圣节季最火的项目，60 分钟沉浸式僵尸主题路线；要分时段买票，热门时段会卖完</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/金属)</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="n"/>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>13–14 Nov 2026</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/独立音乐)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="n"/>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Edinburgh's Christmas 2026（开幕）</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>East &amp; West Princes Street Gardens / George Street, Edinburgh</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>14 Nov 2026 – 3 Jan 2027（窗口内只有 14–15 Nov 开幕周末）</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>本地生活类(集市/节庆)</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>爱丁堡官方冬季节庆，每年举办；免费入场、不用买票</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>https://edinburgh.org/festivals/edinburghs-christmas/ ; https://edwinterfest.com/edinburgh-christmas/whats-on/traditional-christmas-markets</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>开幕周末可以去；市集免费逛，每天 10:00–22:00</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="n"/>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>21–31 Oct 2026</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>兴趣类(文学/讲故事)</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Page Turners Club</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="n"/>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Edinburgh Short Film Festival（第 16 届）</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Edinburgh（多个场地）</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>city_only</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>电影/媒体</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Reel Talk Club</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="n"/>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Page Turners Club</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>21–31 Oct 2026</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>兴趣类(文学/讲故事)</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>同步发爱丁堡2校</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="n"/>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
         <is>
           <t>未完成</t>
         </is>
@@ -3394,11 +4486,11 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>只有烟花节里的 DJ 场，还没专门搜演出</t>
+          <t>都来自城市轮顺带（烟花节 DJ、Skindred 巡演、格拉斯哥音乐节）；还没专门做全国演出轮</t>
         </is>
       </c>
     </row>
@@ -3415,17 +4507,13 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>顺带匹配（没专门搜）</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>计划：第12轮起按兴趣分批</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3494,7 +4582,7 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
     </row>
@@ -3778,15 +4866,15 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第4轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>计划：第4轮 格拉斯哥+爱丁堡</t>
+          <t>格拉斯哥同城共用；Glasgow Green 烟花没收录：搜到的"Mon 5 Nov"是 2018 年的旧页面，而且当地媒体说篝火夜活动已暂停</t>
         </is>
       </c>
     </row>
@@ -3828,15 +4916,15 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第4轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>计划：第4轮 格拉斯哥+爱丁堡</t>
+          <t>格拉斯哥同城共用；Glasgow Green 烟花没收录：搜到的"Mon 5 Nov"是 2018 年的旧页面，而且当地媒体说篝火夜活动已暂停</t>
         </is>
       </c>
     </row>
@@ -3853,15 +4941,15 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第4轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>计划：第4轮 格拉斯哥+爱丁堡</t>
+          <t>爱丁堡同城共用；Samhuinn 火节（10/31）已售罄没收录；Meadowbank 烟花 2017 年起就停办了；Skerryvore 演出票价从 £115 起，太贵，没收录</t>
         </is>
       </c>
     </row>
@@ -3957,11 +5045,11 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>伯明翰同城共用；未达 3–5 条：BCLM 万圣节夜日期对不上（搜到的是 2021 年页面），Moseley 烟花已售罄</t>
+          <t>伯明翰同城共用；第4轮顺带补了 Skindred 伯明翰站；BCLM 万圣节夜日期对不上（搜到的是 2021 年页面），Moseley 烟花已售罄</t>
         </is>
       </c>
     </row>
@@ -3982,11 +5070,11 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>伯明翰同城共用；未达 3–5 条：BCLM 万圣节夜日期对不上（搜到的是 2021 年页面），Moseley 烟花已售罄</t>
+          <t>伯明翰同城共用；第4轮顺带补了 Skindred 伯明翰站；BCLM 万圣节夜日期对不上（搜到的是 2021 年页面），Moseley 烟花已售罄</t>
         </is>
       </c>
     </row>
@@ -4270,15 +5358,15 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第4轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>计划：第4轮 格拉斯哥+爱丁堡</t>
+          <t>格拉斯哥同城共用；Glasgow Green 烟花没收录：搜到的"Mon 5 Nov"是 2018 年的旧页面，而且当地媒体说篝火夜活动已暂停</t>
         </is>
       </c>
     </row>
@@ -4645,11 +5733,11 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>伯明翰同城共用；未达 3–5 条：BCLM 万圣节夜日期对不上（搜到的是 2021 年页面），Moseley 烟花已售罄</t>
+          <t>伯明翰同城共用；第4轮顺带补了 Skindred 伯明翰站；BCLM 万圣节夜日期对不上（搜到的是 2021 年页面），Moseley 烟花已售罄</t>
         </is>
       </c>
     </row>
@@ -4716,15 +5804,15 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第4轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>计划：第4轮 格拉斯哥+爱丁堡</t>
+          <t>爱丁堡同城共用；Samhuinn 火节（10/31）已售罄没收录；Meadowbank 烟花 2017 年起就停办了；Skerryvore 演出票价从 £115 起，太贵，没收录</t>
         </is>
       </c>
     </row>
@@ -4764,7 +5852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4918,10 +6006,58 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>没收录（售罄）</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Samhuinn Fire Festival（爱丁堡 Calton Hill，10/31）：官方票务页显示已售罄，只能排候补</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>日期对不上→没收录</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Glasgow Green 烟花：搜到的"Mon 5 Nov"是 2018 年的旧页面，而且当地媒体说篝火夜活动已暂停</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>日期待核实</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>GlasGLOW：起始日有 16 Oct 和 24 Oct 两种说法，表里已标出来</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>票价偏高→没收录</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Skerryvore @ Edinburgh Corn Exchange（11/6）：Ticketmaster 显示从 £115 起</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>窗口提醒</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>BFI 伦敦电影节只有 15–18 Oct 在窗口内；Frieze 在 15–18 Oct，要推得早</t>
         </is>

</xml_diff>

<commit_message>
Add round 5 (Newcastle + Durham) to Oct–Nov Track B digest
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_10.15-11.15.xlsx
+++ b/data/UK_Events_TrackB_10.15-11.15.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1634,52 +1634,52 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
+          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
+          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
+          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/金属)</t>
+          <t>年轻人娱乐(Club/电子)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
+          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
+          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
+          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>同步发格拉斯哥3校</t>
+          <t>同步发纽卡斯尔3群</t>
         </is>
       </c>
       <c r="N16" s="2" t="n"/>
@@ -1712,12 +1712,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
+          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
+          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1727,12 +1727,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>13–14 Nov 2026</t>
+          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立音乐)</t>
+          <t>年轻人娱乐(Live Music/金属)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1747,17 +1747,17 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
+          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
+          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
+          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1790,32 +1790,32 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Skindred "You Got This" 巡演 伯明翰站</t>
+          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
+          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>30 Oct 2026（周五）</t>
+          <t>13–14 Nov 2026</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>年轻人娱乐(Live Music/独立音乐)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1825,17 +1825,17 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
+          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
+          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
+          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>同步发伯明翰3校</t>
+          <t>同步发格拉斯哥3校</t>
         </is>
       </c>
       <c r="N18" s="2" t="n"/>
@@ -1863,67 +1863,67 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Skindred "You Got This" 巡演 伯明翰站</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>30 Oct 2026（周五）</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Snack Finds &amp; Picks; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第7名</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>同步发 Snack Finds &amp; Picks、伯明翰3校</t>
+          <t>同步发伯明翰3校</t>
         </is>
       </c>
       <c r="N19" s="2" t="n"/>
@@ -1941,67 +1941,67 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Snack Finds &amp; Picks</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Reverend and The Makers 演唱会</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>14 Nov 2026（周六）19:00 开门</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>年轻人娱乐(Live Music/独立摇滚)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>就在 Northumbria 学生会里，在校生走路就到</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第8名</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>同步发 UK Food Lovers</t>
+          <t>同步发纽卡斯尔3群</t>
         </is>
       </c>
       <c r="N20" s="2" t="n"/>
@@ -2019,17 +2019,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies</t>
+          <t>UK Food Lovers</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -2039,37 +2039,37 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Harper Adams Campus Life; Wolverhampton Freshers Hub 2026</t>
+          <t>Snack Finds &amp; Picks; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>同步发 Harper Adams、Wolverhampton</t>
+          <t>同步发 Snack Finds &amp; Picks、伯明翰3校</t>
         </is>
       </c>
       <c r="N21" s="2" t="n"/>
@@ -2097,37 +2097,37 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Snack Finds &amp; Picks</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>MCM Comic Con London（October 2026）</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>23–25 Oct 2026</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(游戏/动漫/流行文化)</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>The Gaming Corner</t>
+          <t>UK Food Lovers; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2137,17 +2137,17 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发 UK Food Lovers</t>
         </is>
       </c>
       <c r="N22" s="2" t="n"/>
@@ -2175,67 +2175,67 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Day Trip Buddies</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>年轻人娱乐(烟花) + 一日游</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Reel Talk Club</t>
+          <t>Harper Adams Campus Life; Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发 Harper Adams、Wolverhampton</t>
         </is>
       </c>
       <c r="N23" s="2" t="n"/>
@@ -2258,62 +2258,62 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Frieze London &amp; Frieze Masters 2026</t>
+          <t>MCM Comic Con London（October 2026）</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>The Regent's Park, London</t>
+          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
+          <t>23–25 Oct 2026</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(艺术/展览)</t>
+          <t>兴趣类(游戏/动漫/流行文化)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
+          <t>The Gaming Corner</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>第3名</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>RCA 优先推</t>
         </is>
       </c>
       <c r="N24" s="2" t="n"/>
@@ -2336,12 +2336,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
+          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2351,17 +2351,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
+          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐节)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>Reel Talk Club</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2371,22 +2371,22 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2414,32 +2414,32 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>Frieze London &amp; Frieze Masters 2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>The Regent's Park, London</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>兴趣类(艺术/展览)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2449,27 +2449,27 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>第5名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边</t>
+          <t>RCA 优先推</t>
         </is>
       </c>
       <c r="N26" s="2" t="n"/>
@@ -2492,62 +2492,62 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
+          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）11:00–15:30</t>
+          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(城市传统活动)</t>
+          <t>年轻人娱乐(烟花/音乐节)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>第4名</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>第6名</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>免费</t>
         </is>
       </c>
       <c r="N27" s="2" t="n"/>
@@ -2570,12 +2570,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2585,12 +2585,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:30</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2605,27 +2605,27 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>第7名</t>
+          <t>第5名</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RCA Battersea 校区就在旁边</t>
         </is>
       </c>
       <c r="N28" s="2" t="n"/>
@@ -2643,32 +2643,32 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>英格兰 vs 澳大利亚（Nations Championship 橄榄球）</t>
+          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
+          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）</t>
+          <t>14 Nov 2026（周六）11:00–15:30</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>运动户外(观赛)</t>
+          <t>本地生活类(城市传统活动)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2683,27 +2683,27 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>RFU 官方公布的国家队主场赛，是新赛事 Nations Championship 的首届</t>
+          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship ; https://allianzstadiumtwickenham.com/nations-championship</t>
+          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>St Mary's 是体育强校，球场就在家门口；⚠️国家队比赛票价偏高</t>
+          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第6名</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>免费</t>
         </is>
       </c>
       <c r="N29" s="2" t="n"/>
@@ -2721,17 +2721,17 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>英格兰 vs 日本（Nations Championship 橄榄球）</t>
+          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2741,17 +2741,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）</t>
+          <t>31 Oct 2026（周六）18:30</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>运动户外(观赛)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2761,22 +2761,22 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>RFU 官方公布的国家队主场赛</t>
+          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>对日本这场的票通常比对新西兰、澳大利亚便宜，更适合学生；⚠️票价还是要看一下</t>
+          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第7名</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -2804,12 +2804,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>英格兰 vs 澳大利亚（Nations Championship 橄榄球）</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2819,17 +2819,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>8 Nov 2026（周日）</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>运动户外(观赛)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew; 伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2839,22 +2839,22 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>RFU 官方公布的国家队主场赛，是新赛事 Nations Championship 的首届</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship ; https://allianzstadiumtwickenham.com/nations-championship</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>St Mary's 是体育强校，球场就在家门口；⚠️国家队比赛票价偏高</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -2882,12 +2882,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Richmond Family Fireworks</t>
+          <t>英格兰 vs 日本（Nations Championship 橄榄球）</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Richmond Athletic Ground, Twickenham Road, Richmond TW9 2SF</t>
+          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2897,12 +2897,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>⚠️待核实：一个来源写 1 Nov，另一个写 5–7 Nov 2026</t>
+          <t>14 Nov 2026（周六）</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花)</t>
+          <t>运动户外(观赛)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2912,32 +2912,32 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>年年举办的本地烟花会（Richmond Athletic Association 主办）；2026 年日期各来源说法不一，所以降级</t>
+          <t>RFU 官方公布的国家队主场赛</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.rag-events.co.uk/major-public-events-at-the-rag/richmond-family-fireworks/ ; https://chiswicktoday.co.uk/chiswick-fireworks-bonfire-night/</t>
+          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>离 St Mary's 很近；确认日期之后再推</t>
+          <t>对日本这场的票通常比对新西兰、澳大利亚便宜，更适合学生；⚠️票价还是要看一下</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>⚠️日期待核实</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N32" s="2" t="n"/>
@@ -2955,37 +2955,37 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers; Snack Finds &amp; Picks</t>
+          <t>Live Music Crew; 伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2995,22 +2995,22 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -3033,32 +3033,32 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Birmingham Big Wheel &amp; Ice Rink（Centenary Square）</t>
+          <t>Richmond Family Fireworks</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Centenary Square, Birmingham</t>
+          <t>Richmond Athletic Ground, Twickenham Road, Richmond TW9 2SF</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>5 Nov 2026 – 3 Jan 2027，每天 10:00–22:00</t>
+          <t>⚠️待核实：一个来源写 1 Nov，另一个写 5–7 Nov 2026</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(滑冰/游乐)</t>
+          <t>年轻人娱乐(烟花)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3068,32 +3068,32 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>跟圣诞市集同期，市集官方配套项目，年年举办；没有售票数据</t>
+          <t>年年举办的本地烟花会（Richmond Athletic Association 主办）；2026 年日期各来源说法不一，所以降级</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham-now.co.uk/news/26551457.birmingham-frankfurt-christmas-market-2026---need-know/</t>
+          <t>https://www.rag-events.co.uk/major-public-events-at-the-rag/richmond-family-fireworks/ ; https://chiswicktoday.co.uk/chiswick-fireworks-bonfire-night/</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>BCU 主校区附近，适合宿舍、群友组团去滑冰</t>
+          <t>离 St Mary's 很近；确认日期之后再推</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⚠️日期待核实</t>
         </is>
       </c>
       <c r="N34" s="2" t="n"/>
@@ -3116,57 +3116,57 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Skindred "You Got This" 巡演 伯明翰站</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>30 Oct 2026（周五）</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>UK Food Lovers; Snack Finds &amp; Picks</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
@@ -3189,17 +3189,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Harper Adams Campus Life</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>Birmingham Big Wheel &amp; Ice Rink（Centenary Square）</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Centenary Square, Birmingham</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -3209,17 +3209,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>5 Nov 2026 – 3 Jan 2027，每天 10:00–22:00</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>年轻人娱乐(滑冰/游乐)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies; Wolverhampton Freshers Hub 2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3229,22 +3229,22 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>跟圣诞市集同期，市集官方配套项目，年年举办；没有售票数据</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.birmingham-now.co.uk/news/26551457.birmingham-frankfurt-christmas-market-2026---need-know/</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>BCU 主校区附近，适合宿舍、群友组团去滑冰</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
@@ -3267,37 +3267,37 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Wolverhampton Freshers Hub 2026</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>Skindred "You Got This" 巡演 伯明翰站</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>30 Oct 2026（周五）</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies; Harper Adams Campus Life</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -3307,22 +3307,22 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
@@ -3345,17 +3345,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>University of Lancaster</t>
+          <t>Harper Adams Campus Life</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Capernwray 湖泊公开水域游泳（Lake Swim）</t>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -3365,37 +3365,37 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026</t>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>运动户外(游泳)</t>
+          <t>年轻人娱乐(烟花) + 一日游</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Swim Wave Tribe</t>
+          <t>Day Trip Buddies; Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>仅见于 Outdoor Swimmer 杂志活动日历；主办方未核实（疑为 T2 Events，他们在该场地办过比赛）；无报名数据</t>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://outdoorswimmer.com/events/ ; https://www.t2.events/our-events/capernwray-open-water-swim/</t>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>窗口内极少数的户外游泳活动，10 月底水温很低，只适合有冷水经验的人；离 Lancaster 大学约 10 公里</t>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -3423,37 +3423,37 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>The University of Manchester</t>
+          <t>Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Islington Mill, James Street, Salford</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:00–24:00</t>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体 + 社交类(女性)</t>
+          <t>年轻人娱乐(烟花) + 一日游</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner; Reel Talk Club</t>
+          <t>Day Trip Buddies; Harper Adams Campus Life</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3463,17 +3463,17 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -3501,37 +3501,37 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>The University of Manchester</t>
+          <t>University of Lancaster</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：Season of the Witch 系列活动</t>
+          <t>Capernwray 湖泊公开水域游泳（Lake Swim）</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Manchester 多个场地</t>
+          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
+          <t>31 Oct 2026</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>社交类(女性) + 兴趣类(手工)</t>
+          <t>运动户外(游泳)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner</t>
+          <t>Swim Wave Tribe</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3541,22 +3541,22 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Manchester's Finest 收录；系列里有 Craft &amp; Coven 手工夜、Pendle 女巫审判主题徒步等；没有单场售票数据</t>
+          <t>仅见于 Outdoor Swimmer 杂志活动日历；主办方未核实（疑为 T2 Events，他们在该场地办过比赛）；无报名数据</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://www.manchestersfinest.com/events/girl-gang-mcr-season-of-the-witch/ ; https://girlgangmcr.com/upcoming-events/</t>
+          <t>https://outdoorswimmer.com/events/ ; https://www.t2.events/our-events/capernwray-open-water-swim/</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>窗口内有多场可选；Pendle 徒步的具体日期没搜到，推之前要看官网确认单场日期</t>
+          <t>窗口内极少数的户外游泳活动，10 月底水温很低，只适合有冷水经验的人；离 Lancaster 大学约 10 公里</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
@@ -3584,57 +3584,57 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Lonely Girls Club Manchester 活动（10/27 场）</t>
+          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Manchester（场地待公布）</t>
+          <t>Islington Mill, James Street, Salford</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>27 Oct 2026（周二）</t>
+          <t>31 Oct 2026（周六）18:00–24:00</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>社交类(女性交友)</t>
+          <t>电影/媒体 + 社交类(女性)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner</t>
+          <t>Girls' Corner; Reel Talk Club</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>成熟的女性交友组织（有 Wikipedia 词条），London+Manchester 成员约 5.5 万（这是社群规模，不代表到场人数）；这场的具体内容官网写"即将公布"</t>
+          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>https://www.llgc.co.uk/collections/manchester</t>
+          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>票价 £8.95，便宜，专为一个人来交朋友设计；活动内容没公布，推之前再看一眼</t>
+          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
@@ -3657,62 +3657,62 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>itison GlasGLOW 2026：Zombie Zoo 万圣节灯光夜游</t>
+          <t>Girl Gang MCR：Season of the Witch 系列活动</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Glasgow Botanic Gardens, 730 Great Western Road, Glasgow G12 0UE</t>
+          <t>Manchester 多个场地</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>⚠️起始日两种说法：16 Oct 或 24 Oct 开始，1–2 Nov 结束（24 Oct–1 Nov 两种说法都覆盖）</t>
+          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(沉浸式/万圣节)</t>
+          <t>社交类(女性) + 兴趣类(手工)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Girls' Corner</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>第 8 年举办；自称英国最大的万圣节活动；往年曾因需求大加售数千张票（Scottish Daily Express 报道）</t>
+          <t>Manchester's Finest 收录；系列里有 Craft &amp; Coven 手工夜、Pendle 女巫审判主题徒步等；没有单场售票数据</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.itison.com/glasglow ; https://www.glasgowworld.com/news/glasglow-botanic-gardens-dates-5290284 ; https://www.scottishdailyexpress.co.uk/news/scottish-news/glasglow-botanic-gardens-thousands-extra-30877210</t>
+          <t>https://www.manchestersfinest.com/events/girl-gang-mcr-season-of-the-witch/ ; https://girlgangmcr.com/upcoming-events/</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥万圣节季最火的项目，60 分钟沉浸式僵尸主题路线；要分时段买票，热门时段会卖完</t>
+          <t>窗口内有多场可选；Pendle 徒步的具体日期没搜到，推之前要看官网确认单场日期</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
@@ -3735,62 +3735,62 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
+          <t>Lonely Girls Club Manchester 活动（10/27 场）</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
+          <t>Manchester（场地待公布）</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
+          <t>27 Oct 2026（周二）</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/金属)</t>
+          <t>社交类(女性交友)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>Girls' Corner</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
+          <t>成熟的女性交友组织（有 Wikipedia 词条），London+Manchester 成员约 5.5 万（这是社群规模，不代表到场人数）；这场的具体内容官网写"即将公布"</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
+          <t>https://www.llgc.co.uk/collections/manchester</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
+          <t>票价 £8.95，便宜，专为一个人来交朋友设计；活动内容没公布，推之前再看一眼</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
@@ -3818,57 +3818,57 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
+          <t>itison GlasGLOW 2026：Zombie Zoo 万圣节灯光夜游</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
+          <t>Glasgow Botanic Gardens, 730 Great Western Road, Glasgow G12 0UE</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>13–14 Nov 2026</t>
+          <t>⚠️起始日两种说法：16 Oct 或 24 Oct 开始，1–2 Nov 结束（24 Oct–1 Nov 两种说法都覆盖）</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立音乐)</t>
+          <t>年轻人娱乐(沉浸式/万圣节)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
+          <t>第 8 年举办；自称英国最大的万圣节活动；往年曾因需求大加售数千张票（Scottish Daily Express 报道）</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
+          <t>https://www.itison.com/glasglow ; https://www.glasgowworld.com/news/glasglow-botanic-gardens-dates-5290284 ; https://www.scottishdailyexpress.co.uk/news/scottish-news/glasglow-botanic-gardens-thousands-extra-30877210</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
+          <t>格拉斯哥万圣节季最火的项目，60 分钟沉浸式僵尸主题路线；要分时段买票，热门时段会卖完</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
@@ -3891,17 +3891,17 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh's Christmas 2026（开幕）</t>
+          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>East &amp; West Princes Street Gardens / George Street, Edinburgh</t>
+          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -3911,42 +3911,42 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026 – 3 Jan 2027（窗口内只有 14–15 Nov 开幕周末）</t>
+          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/节庆)</t>
+          <t>年轻人娱乐(Live Music/金属)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡官方冬季节庆，每年举办；免费入场、不用买票</t>
+          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>https://edinburgh.org/festivals/edinburghs-christmas/ ; https://edwinterfest.com/edinburgh-christmas/whats-on/traditional-christmas-markets</t>
+          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>开幕周末可以去；市集免费逛，每天 10:00–22:00</t>
+          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
@@ -3969,37 +3969,37 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>21–31 Oct 2026</t>
+          <t>13–14 Nov 2026</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(文学/讲故事)</t>
+          <t>年轻人娱乐(Live Music/独立音乐)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Page Turners Club</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -4009,22 +4009,22 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
+          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
+          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
+          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
@@ -4052,57 +4052,57 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh Short Film Festival（第 16 届）</t>
+          <t>Edinburgh's Christmas 2026（开幕）</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh（多个场地）</t>
+          <t>East &amp; West Princes Street Gardens / George Street, Edinburgh</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
+          <t>14 Nov 2026 – 3 Jan 2027（窗口内只有 14–15 Nov 开幕周末）</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>本地生活类(集市/节庆)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Reel Talk Club</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
+          <t>爱丁堡官方冬季节庆，每年举办；免费入场、不用买票</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
+          <t>https://edinburgh.org/festivals/edinburghs-christmas/ ; https://edwinterfest.com/edinburgh-christmas/whats-on/traditional-christmas-markets</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
+          <t>开幕周末可以去；市集免费逛，每天 10:00–22:00</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
@@ -4125,39 +4125,39 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>21–31 Oct 2026</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>兴趣类(文学/讲故事)</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
           <t>Page Turners Club</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>21–31 Oct 2026</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>兴趣类(文学/讲故事)</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
-        </is>
-      </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
           <t>中热度</t>
@@ -4180,12 +4180,12 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>同步发爱丁堡2校</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N48" s="2" t="n"/>
@@ -4195,6 +4195,630 @@
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Edinburgh Short Film Festival（第 16 届）</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Edinburgh（多个场地）</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>city_only</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>电影/媒体</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Reel Talk Club</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="n"/>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Page Turners Club</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>21–31 Oct 2026</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>兴趣类(文学/讲故事)</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>同步发爱丁堡2校</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="n"/>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Club/电子)</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="n"/>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Durham university</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>英国知名露天博物馆的年度万圣节夜场；只能网上提前买票，往年经常售罄</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.beamish.org.uk/events/halloween-evening-28-oct-2026/ ; https://www.beamish.org.uk/halloween-at-beamish/</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>在纽卡斯尔和杜伦中间，两边都能去；有吓人路线，也有不吓人的；年卡在夜场不能用</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>同步发 Durham university</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="n"/>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle Racecourse Bonfire Night（夜场赛马 + 烟花）</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle Racecourse, High Gosforth Park, Newcastle upon Tyne NE3 5HP</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>6 Nov 2026（周五）18:00 开门，约 20:30 放烟花</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花/赛马)</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>赛马场官方年年举办，号称"本地区最大的烟花"（主办方说法）；已开售</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.newcastle-racecourse.co.uk/popular-events/fireworks</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>早鸟票成人 £9，很便宜；赛马 + 游乐场 + 烟花，一晚玩全套</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="n"/>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Reverend and The Makers 演唱会</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>14 Nov 2026（周六）19:00 开门</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/独立摇滚)</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>就在 Northumbria 学生会里，在校生走路就到</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>第4名</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Northumbria 优先</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="n"/>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Durham university</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>英国知名露天博物馆的年度万圣节夜场；只能网上提前买票，往年经常售罄</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.beamish.org.uk/events/halloween-evening-28-oct-2026/ ; https://www.beamish.org.uk/halloween-at-beamish/</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>在纽卡斯尔和杜伦中间，两边都能去；有吓人路线，也有不吓人的；年卡在夜场不能用</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="n"/>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Durham university</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Durham Jazz Festival 2026</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Gala Theatre / Redhills (Durham Miners' Hall) / Sir Thomas Allen Assembly Rooms 等，Durham</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>23–25 Oct 2026</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/爵士)</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>新办的爵士节（Visit County Durham 报道"新创办"），UK Jazz News 有收录；还没有售票数据</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>https://durhamjazzfestival.co.uk/ ; https://ukjazznews.com/durham-jazz-festival-2026-23-to-26-october/</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>场地都在杜伦市中心，有酒吧快闪演出，也有剧院大场，门槛可高可低</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="n"/>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
         <is>
           <t>未完成</t>
         </is>
@@ -4486,7 +5110,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -5408,15 +6032,15 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第5轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>计划：第5轮 纽卡斯尔+杜伦</t>
+          <t>纽卡斯尔同城共用，两个群内容完全一样；圣诞市集 11/19 才开，不在窗口内</t>
         </is>
       </c>
     </row>
@@ -5433,15 +6057,15 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第5轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>计划：第5轮 纽卡斯尔+杜伦</t>
+          <t>纽卡斯尔同城共用，两个群内容完全一样；圣诞市集 11/19 才开，不在窗口内</t>
         </is>
       </c>
     </row>
@@ -5458,15 +6082,15 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第5轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>计划：第5轮 纽卡斯尔+杜伦</t>
+          <t>纽卡斯尔同城共用，两个群内容完全一样；圣诞市集 11/19 才开，不在窗口内</t>
         </is>
       </c>
     </row>
@@ -5483,15 +6107,15 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第5轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>计划：第5轮 纽卡斯尔+杜伦</t>
+          <t>未达 3–5 条：Lumiere 灯光节 2025 年已停办；Durham Book Festival 在 10/9–11，不在窗口内；Hardwick Hall 烟花的 2026 年日期没确认</t>
         </is>
       </c>
     </row>
@@ -5852,7 +6476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6054,10 +6678,46 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>已停办</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Durham Lumiere 灯光节：2025 年是最后一届，2026 年没有</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>日期对不上→没收录</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Hardwick Hall 烟花（Sedgefield）：搜到的"Sat 5 / Sun 6 Nov"是 2022 年的日期，2026 年日期没确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>日期待核实</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Beamish 万圣节夜场：官网确认有 28 Oct 那一场，整季场次各来源说法不一</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>窗口提醒</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>BFI 伦敦电影节只有 15–18 Oct 在窗口内；Frieze 在 15–18 Oct，要推得早</t>
         </is>

</xml_diff>

<commit_message>
Add round 6 (Leeds + Sheffield + Huddersfield) to Oct–Nov Track B digest
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_10.15-11.15.xlsx
+++ b/data/UK_Events_TrackB_10.15-11.15.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P56"/>
+  <dimension ref="A1:P67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1244,52 +1244,52 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
+          <t>Leeds International Film Festival（第 40 届）</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Islington Mill, James Street, Salford</t>
+          <t>Hyde Park Picture House, 73 Brudenell Road, Leeds LS6 1JD / Everyman Leeds 等多个影院</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:00–24:00</t>
+          <t>29 Oct – 15 Nov 2026（有来源写 5–22 Nov；主流来源和官方节目时间表都写 29 Oct 开始）</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体 + 社交类(女性)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner; The University of Manchester</t>
+          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
+          <t>第 40 届，英国历史最悠久的电影节之一；10/1 节目上线、10/8 单片开票（YEP 报道）</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
+          <t>https://www.leedsfilm.com/liff-2026-6ftb ; https://www.yorkshireeveningpost.co.uk/whats-on/arts-and-entertainment/leeds-international-film-festival-2026-opening-films-liff-40th-9021020</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
+          <t>Hyde Park Picture House 就在 Leeds 大学学生区旁边；几乎整个窗口期都有放映</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>同步发 Girls' Corner</t>
+          <t>同步发利兹2群</t>
         </is>
       </c>
       <c r="N11" s="2" t="n"/>
@@ -1322,52 +1322,52 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh Short Film Festival（第 16 届）</t>
+          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh（多个场地）</t>
+          <t>Islington Mill, James Street, Salford</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
+          <t>31 Oct 2026（周六）18:00–24:00</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>电影/媒体 + 社交类(女性)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+          <t>Girls' Corner; The University of Manchester</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
+          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
+          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
+          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>同步发爱丁堡2校</t>
+          <t>同步发 Girls' Corner</t>
         </is>
       </c>
       <c r="N12" s="2" t="n"/>
@@ -1395,67 +1395,67 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>Reel Talk Club</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
+          <t>Edinburgh Short Film Festival（第 16 届）</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>Edinburgh（多个场地）</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
+          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐节)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>同步发伦敦6校</t>
+          <t>同步发爱丁堡2校</t>
         </is>
       </c>
       <c r="N13" s="2" t="n"/>
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1493,17 +1493,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>年轻人娱乐(烟花/音乐节)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London); St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1513,27 +1513,27 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>同步发伦敦6校（RCA 优先）</t>
+          <t>同步发伦敦6校</t>
         </is>
       </c>
       <c r="N14" s="2" t="n"/>
@@ -1556,12 +1556,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1571,17 +1571,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:30</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London); St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1591,27 +1591,27 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>同步发伦敦6校</t>
+          <t>同步发伦敦6校（RCA 优先）</t>
         </is>
       </c>
       <c r="N15" s="2" t="n"/>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
+          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1649,17 +1649,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
+          <t>31 Oct 2026（周六）18:30</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Club/电子)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1669,27 +1669,27 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
+          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
+          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>同步发纽卡斯尔3群</t>
+          <t>同步发伦敦6校</t>
         </is>
       </c>
       <c r="N16" s="2" t="n"/>
@@ -1712,62 +1712,62 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
+          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
+          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
+          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/金属)</t>
+          <t>年轻人娱乐(Club/电子)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
+          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
+          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
+          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>第5名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>同步发格拉斯哥3校</t>
+          <t>同步发纽卡斯尔3群</t>
         </is>
       </c>
       <c r="N17" s="2" t="n"/>
@@ -1790,12 +1790,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
+          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
+          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1805,12 +1805,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>13–14 Nov 2026</t>
+          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立音乐)</t>
+          <t>年轻人娱乐(Live Music/金属)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1825,22 +1825,22 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
+          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
+          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
+          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>第6名</t>
+          <t>第5名</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1868,32 +1868,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Skindred "You Got This" 巡演 伯明翰站</t>
+          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
+          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>30 Oct 2026（周五）</t>
+          <t>13–14 Nov 2026</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>年轻人娱乐(Live Music/独立音乐)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1903,27 +1903,27 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
+          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
+          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
+          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>第7名</t>
+          <t>第6名</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>同步发伯明翰3校</t>
+          <t>同步发格拉斯哥3校</t>
         </is>
       </c>
       <c r="N19" s="2" t="n"/>
@@ -1946,12 +1946,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Reverend and The Makers 演唱会</t>
+          <t>Skindred "You Got This" 巡演 伯明翰站</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
+          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1961,17 +1961,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）19:00 开门</t>
+          <t>30 Oct 2026（周五）</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立摇滚)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1981,27 +1981,27 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
+          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
+          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>就在 Northumbria 学生会里，在校生走路就到</t>
+          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>第8名</t>
+          <t>第7名</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>同步发纽卡斯尔3群</t>
+          <t>同步发伯明翰3校</t>
         </is>
       </c>
       <c r="N20" s="2" t="n"/>
@@ -2019,67 +2019,67 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Reverend and The Makers 演唱会</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>14 Nov 2026（周六）19:00 开门</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>年轻人娱乐(Live Music/独立摇滚)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Snack Finds &amp; Picks; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>就在 Northumbria 学生会里，在校生走路就到</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第8名</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>同步发 Snack Finds &amp; Picks、伯明翰3校</t>
+          <t>同步发纽卡斯尔3群</t>
         </is>
       </c>
       <c r="N21" s="2" t="n"/>
@@ -2097,67 +2097,67 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Snack Finds &amp; Picks</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Embrace 30 周年巡演（嘉宾：The Rolling People / The Bunny Suit）</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>O2 Academy Leeds, 55 Cookridge Street, Leeds LS2 3AW</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>13 Nov 2026（周五）19:00</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>年轻人娱乐(Live Music/英伦摇滚)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>Live Nation / Academy Music Group 正式售票；乐队 30 周年新专辑巡演</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.academymusicgroup.com/o2academyleeds/events/embrace-tickets-ae136632 ; https://www.gigsandtours.com/event/embrace/o2-academy-leeds/3605026</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>票价约 £37.70；场馆离 Leeds 大学、Leeds Beckett 都近</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第9名</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>同步发 UK Food Lovers</t>
+          <t>同步发利兹2群</t>
         </is>
       </c>
       <c r="N22" s="2" t="n"/>
@@ -2175,17 +2175,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies</t>
+          <t>UK Food Lovers</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2195,37 +2195,37 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Harper Adams Campus Life; Wolverhampton Freshers Hub 2026</t>
+          <t>Snack Finds &amp; Picks; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>同步发 Harper Adams、Wolverhampton</t>
+          <t>同步发 Snack Finds &amp; Picks、伯明翰3校</t>
         </is>
       </c>
       <c r="N23" s="2" t="n"/>
@@ -2253,37 +2253,37 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Snack Finds &amp; Picks</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>MCM Comic Con London（October 2026）</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>23–25 Oct 2026</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(游戏/动漫/流行文化)</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>The Gaming Corner</t>
+          <t>UK Food Lovers; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2293,17 +2293,17 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发 UK Food Lovers</t>
         </is>
       </c>
       <c r="N24" s="2" t="n"/>
@@ -2331,67 +2331,67 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Day Trip Buddies</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>年轻人娱乐(烟花) + 一日游</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Reel Talk Club</t>
+          <t>Harper Adams Campus Life; Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发 Harper Adams、Wolverhampton</t>
         </is>
       </c>
       <c r="N25" s="2" t="n"/>
@@ -2414,62 +2414,62 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Frieze London &amp; Frieze Masters 2026</t>
+          <t>MCM Comic Con London（October 2026）</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>The Regent's Park, London</t>
+          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
+          <t>23–25 Oct 2026</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(艺术/展览)</t>
+          <t>兴趣类(游戏/动漫/流行文化)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
+          <t>The Gaming Corner</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>第3名</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>RCA 优先推</t>
         </is>
       </c>
       <c r="N26" s="2" t="n"/>
@@ -2492,12 +2492,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
+          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -2507,17 +2507,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
+          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐节)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>Reel Talk Club</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2527,22 +2527,22 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -2570,32 +2570,32 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>Frieze London &amp; Frieze Masters 2026</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>The Regent's Park, London</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>兴趣类(艺术/展览)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2605,27 +2605,27 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>第5名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边</t>
+          <t>RCA 优先推</t>
         </is>
       </c>
       <c r="N28" s="2" t="n"/>
@@ -2648,62 +2648,62 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
+          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）11:00–15:30</t>
+          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(城市传统活动)</t>
+          <t>年轻人娱乐(烟花/音乐节)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>第4名</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>第6名</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>免费</t>
         </is>
       </c>
       <c r="N29" s="2" t="n"/>
@@ -2726,12 +2726,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2741,12 +2741,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:30</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2761,27 +2761,27 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>第7名</t>
+          <t>第5名</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RCA Battersea 校区就在旁边</t>
         </is>
       </c>
       <c r="N30" s="2" t="n"/>
@@ -2799,32 +2799,32 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>英格兰 vs 澳大利亚（Nations Championship 橄榄球）</t>
+          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
+          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）</t>
+          <t>14 Nov 2026（周六）11:00–15:30</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>运动户外(观赛)</t>
+          <t>本地生活类(城市传统活动)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2839,27 +2839,27 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>RFU 官方公布的国家队主场赛，是新赛事 Nations Championship 的首届</t>
+          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship ; https://allianzstadiumtwickenham.com/nations-championship</t>
+          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>St Mary's 是体育强校，球场就在家门口；⚠️国家队比赛票价偏高</t>
+          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第6名</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>免费</t>
         </is>
       </c>
       <c r="N31" s="2" t="n"/>
@@ -2877,17 +2877,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>英格兰 vs 日本（Nations Championship 橄榄球）</t>
+          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2897,17 +2897,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）</t>
+          <t>31 Oct 2026（周六）18:30</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>运动户外(观赛)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2917,22 +2917,22 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>RFU 官方公布的国家队主场赛</t>
+          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>对日本这场的票通常比对新西兰、澳大利亚便宜，更适合学生；⚠️票价还是要看一下</t>
+          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第7名</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
@@ -2960,12 +2960,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>英格兰 vs 澳大利亚（Nations Championship 橄榄球）</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2975,17 +2975,17 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>8 Nov 2026（周日）</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>运动户外(观赛)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew; 伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2995,22 +2995,22 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>RFU 官方公布的国家队主场赛，是新赛事 Nations Championship 的首届</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship ; https://allianzstadiumtwickenham.com/nations-championship</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>St Mary's 是体育强校，球场就在家门口；⚠️国家队比赛票价偏高</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -3038,12 +3038,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Richmond Family Fireworks</t>
+          <t>英格兰 vs 日本（Nations Championship 橄榄球）</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Richmond Athletic Ground, Twickenham Road, Richmond TW9 2SF</t>
+          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3053,12 +3053,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>⚠️待核实：一个来源写 1 Nov，另一个写 5–7 Nov 2026</t>
+          <t>14 Nov 2026（周六）</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花)</t>
+          <t>运动户外(观赛)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3068,32 +3068,32 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>年年举办的本地烟花会（Richmond Athletic Association 主办）；2026 年日期各来源说法不一，所以降级</t>
+          <t>RFU 官方公布的国家队主场赛</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.rag-events.co.uk/major-public-events-at-the-rag/richmond-family-fireworks/ ; https://chiswicktoday.co.uk/chiswick-fireworks-bonfire-night/</t>
+          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>离 St Mary's 很近；确认日期之后再推</t>
+          <t>对日本这场的票通常比对新西兰、澳大利亚便宜，更适合学生；⚠️票价还是要看一下</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>⚠️日期待核实</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N34" s="2" t="n"/>
@@ -3111,37 +3111,37 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers; Snack Finds &amp; Picks</t>
+          <t>Live Music Crew; 伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -3151,22 +3151,22 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
@@ -3189,32 +3189,32 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Birmingham Big Wheel &amp; Ice Rink（Centenary Square）</t>
+          <t>Richmond Family Fireworks</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Centenary Square, Birmingham</t>
+          <t>Richmond Athletic Ground, Twickenham Road, Richmond TW9 2SF</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>5 Nov 2026 – 3 Jan 2027，每天 10:00–22:00</t>
+          <t>⚠️待核实：一个来源写 1 Nov，另一个写 5–7 Nov 2026</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(滑冰/游乐)</t>
+          <t>年轻人娱乐(烟花)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3224,32 +3224,32 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>跟圣诞市集同期，市集官方配套项目，年年举办；没有售票数据</t>
+          <t>年年举办的本地烟花会（Richmond Athletic Association 主办）；2026 年日期各来源说法不一，所以降级</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham-now.co.uk/news/26551457.birmingham-frankfurt-christmas-market-2026---need-know/</t>
+          <t>https://www.rag-events.co.uk/major-public-events-at-the-rag/richmond-family-fireworks/ ; https://chiswicktoday.co.uk/chiswick-fireworks-bonfire-night/</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>BCU 主校区附近，适合宿舍、群友组团去滑冰</t>
+          <t>离 St Mary's 很近；确认日期之后再推</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⚠️日期待核实</t>
         </is>
       </c>
       <c r="N36" s="2" t="n"/>
@@ -3272,57 +3272,57 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Skindred "You Got This" 巡演 伯明翰站</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>30 Oct 2026（周五）</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>UK Food Lovers; Snack Finds &amp; Picks</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
@@ -3345,17 +3345,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Harper Adams Campus Life</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>Birmingham Big Wheel &amp; Ice Rink（Centenary Square）</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Centenary Square, Birmingham</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -3365,17 +3365,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>5 Nov 2026 – 3 Jan 2027，每天 10:00–22:00</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>年轻人娱乐(滑冰/游乐)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies; Wolverhampton Freshers Hub 2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -3385,22 +3385,22 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>跟圣诞市集同期，市集官方配套项目，年年举办；没有售票数据</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.birmingham-now.co.uk/news/26551457.birmingham-frankfurt-christmas-market-2026---need-know/</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>BCU 主校区附近，适合宿舍、群友组团去滑冰</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
@@ -3423,37 +3423,37 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Wolverhampton Freshers Hub 2026</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>Skindred "You Got This" 巡演 伯明翰站</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>30 Oct 2026（周五）</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies; Harper Adams Campus Life</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3463,22 +3463,22 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
@@ -3501,17 +3501,17 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>University of Lancaster</t>
+          <t>Harper Adams Campus Life</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Capernwray 湖泊公开水域游泳（Lake Swim）</t>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -3521,37 +3521,37 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026</t>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>运动户外(游泳)</t>
+          <t>年轻人娱乐(烟花) + 一日游</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Swim Wave Tribe</t>
+          <t>Day Trip Buddies; Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>仅见于 Outdoor Swimmer 杂志活动日历；主办方未核实（疑为 T2 Events，他们在该场地办过比赛）；无报名数据</t>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://outdoorswimmer.com/events/ ; https://www.t2.events/our-events/capernwray-open-water-swim/</t>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>窗口内极少数的户外游泳活动，10 月底水温很低，只适合有冷水经验的人；离 Lancaster 大学约 10 公里</t>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -3579,37 +3579,37 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>The University of Manchester</t>
+          <t>Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Islington Mill, James Street, Salford</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:00–24:00</t>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体 + 社交类(女性)</t>
+          <t>年轻人娱乐(烟花) + 一日游</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner; Reel Talk Club</t>
+          <t>Day Trip Buddies; Harper Adams Campus Life</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -3619,17 +3619,17 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -3657,37 +3657,37 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>The University of Manchester</t>
+          <t>University of Lancaster</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：Season of the Witch 系列活动</t>
+          <t>Capernwray 湖泊公开水域游泳（Lake Swim）</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Manchester 多个场地</t>
+          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
+          <t>31 Oct 2026</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>社交类(女性) + 兴趣类(手工)</t>
+          <t>运动户外(游泳)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner</t>
+          <t>Swim Wave Tribe</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -3697,22 +3697,22 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Manchester's Finest 收录；系列里有 Craft &amp; Coven 手工夜、Pendle 女巫审判主题徒步等；没有单场售票数据</t>
+          <t>仅见于 Outdoor Swimmer 杂志活动日历；主办方未核实（疑为 T2 Events，他们在该场地办过比赛）；无报名数据</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://www.manchestersfinest.com/events/girl-gang-mcr-season-of-the-witch/ ; https://girlgangmcr.com/upcoming-events/</t>
+          <t>https://outdoorswimmer.com/events/ ; https://www.t2.events/our-events/capernwray-open-water-swim/</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>窗口内有多场可选；Pendle 徒步的具体日期没搜到，推之前要看官网确认单场日期</t>
+          <t>窗口内极少数的户外游泳活动，10 月底水温很低，只适合有冷水经验的人；离 Lancaster 大学约 10 公里</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
@@ -3740,57 +3740,57 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Lonely Girls Club Manchester 活动（10/27 场）</t>
+          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Manchester（场地待公布）</t>
+          <t>Islington Mill, James Street, Salford</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>27 Oct 2026（周二）</t>
+          <t>31 Oct 2026（周六）18:00–24:00</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>社交类(女性交友)</t>
+          <t>电影/媒体 + 社交类(女性)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner</t>
+          <t>Girls' Corner; Reel Talk Club</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>成熟的女性交友组织（有 Wikipedia 词条），London+Manchester 成员约 5.5 万（这是社群规模，不代表到场人数）；这场的具体内容官网写"即将公布"</t>
+          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>https://www.llgc.co.uk/collections/manchester</t>
+          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>票价 £8.95，便宜，专为一个人来交朋友设计；活动内容没公布，推之前再看一眼</t>
+          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
@@ -3813,62 +3813,62 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>itison GlasGLOW 2026：Zombie Zoo 万圣节灯光夜游</t>
+          <t>Girl Gang MCR：Season of the Witch 系列活动</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Glasgow Botanic Gardens, 730 Great Western Road, Glasgow G12 0UE</t>
+          <t>Manchester 多个场地</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>⚠️起始日两种说法：16 Oct 或 24 Oct 开始，1–2 Nov 结束（24 Oct–1 Nov 两种说法都覆盖）</t>
+          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(沉浸式/万圣节)</t>
+          <t>社交类(女性) + 兴趣类(手工)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Girls' Corner</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>第 8 年举办；自称英国最大的万圣节活动；往年曾因需求大加售数千张票（Scottish Daily Express 报道）</t>
+          <t>Manchester's Finest 收录；系列里有 Craft &amp; Coven 手工夜、Pendle 女巫审判主题徒步等；没有单场售票数据</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.itison.com/glasglow ; https://www.glasgowworld.com/news/glasglow-botanic-gardens-dates-5290284 ; https://www.scottishdailyexpress.co.uk/news/scottish-news/glasglow-botanic-gardens-thousands-extra-30877210</t>
+          <t>https://www.manchestersfinest.com/events/girl-gang-mcr-season-of-the-witch/ ; https://girlgangmcr.com/upcoming-events/</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥万圣节季最火的项目，60 分钟沉浸式僵尸主题路线；要分时段买票，热门时段会卖完</t>
+          <t>窗口内有多场可选；Pendle 徒步的具体日期没搜到，推之前要看官网确认单场日期</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
@@ -3891,62 +3891,62 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
+          <t>Lonely Girls Club Manchester 活动（10/27 场）</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
+          <t>Manchester（场地待公布）</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
+          <t>27 Oct 2026（周二）</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/金属)</t>
+          <t>社交类(女性交友)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>Girls' Corner</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
+          <t>成熟的女性交友组织（有 Wikipedia 词条），London+Manchester 成员约 5.5 万（这是社群规模，不代表到场人数）；这场的具体内容官网写"即将公布"</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
+          <t>https://www.llgc.co.uk/collections/manchester</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
+          <t>票价 £8.95，便宜，专为一个人来交朋友设计；活动内容没公布，推之前再看一眼</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
@@ -3974,57 +3974,57 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
+          <t>itison GlasGLOW 2026：Zombie Zoo 万圣节灯光夜游</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
+          <t>Glasgow Botanic Gardens, 730 Great Western Road, Glasgow G12 0UE</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>13–14 Nov 2026</t>
+          <t>⚠️起始日两种说法：16 Oct 或 24 Oct 开始，1–2 Nov 结束（24 Oct–1 Nov 两种说法都覆盖）</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立音乐)</t>
+          <t>年轻人娱乐(沉浸式/万圣节)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
+          <t>第 8 年举办；自称英国最大的万圣节活动；往年曾因需求大加售数千张票（Scottish Daily Express 报道）</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
+          <t>https://www.itison.com/glasglow ; https://www.glasgowworld.com/news/glasglow-botanic-gardens-dates-5290284 ; https://www.scottishdailyexpress.co.uk/news/scottish-news/glasglow-botanic-gardens-thousands-extra-30877210</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
+          <t>格拉斯哥万圣节季最火的项目，60 分钟沉浸式僵尸主题路线；要分时段买票，热门时段会卖完</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
@@ -4047,17 +4047,17 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh's Christmas 2026（开幕）</t>
+          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>East &amp; West Princes Street Gardens / George Street, Edinburgh</t>
+          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -4067,42 +4067,42 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026 – 3 Jan 2027（窗口内只有 14–15 Nov 开幕周末）</t>
+          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/节庆)</t>
+          <t>年轻人娱乐(Live Music/金属)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡官方冬季节庆，每年举办；免费入场、不用买票</t>
+          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>https://edinburgh.org/festivals/edinburghs-christmas/ ; https://edwinterfest.com/edinburgh-christmas/whats-on/traditional-christmas-markets</t>
+          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>开幕周末可以去；市集免费逛，每天 10:00–22:00</t>
+          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
@@ -4125,37 +4125,37 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>21–31 Oct 2026</t>
+          <t>13–14 Nov 2026</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(文学/讲故事)</t>
+          <t>年轻人娱乐(Live Music/独立音乐)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Page Turners Club</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -4165,22 +4165,22 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
+          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
+          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
+          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
@@ -4208,57 +4208,57 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh Short Film Festival（第 16 届）</t>
+          <t>Edinburgh's Christmas 2026（开幕）</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh（多个场地）</t>
+          <t>East &amp; West Princes Street Gardens / George Street, Edinburgh</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
+          <t>14 Nov 2026 – 3 Jan 2027（窗口内只有 14–15 Nov 开幕周末）</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>本地生活类(集市/节庆)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Reel Talk Club</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
+          <t>爱丁堡官方冬季节庆，每年举办；免费入场、不用买票</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
+          <t>https://edinburgh.org/festivals/edinburghs-christmas/ ; https://edwinterfest.com/edinburgh-christmas/whats-on/traditional-christmas-markets</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
+          <t>开幕周末可以去；市集免费逛，每天 10:00–22:00</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
@@ -4281,39 +4281,39 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>21–31 Oct 2026</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>兴趣类(文学/讲故事)</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
           <t>Page Turners Club</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>21–31 Oct 2026</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>兴趣类(文学/讲故事)</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
-        </is>
-      </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
           <t>中热度</t>
@@ -4336,12 +4336,12 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>同步发爱丁堡2校</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N50" s="2" t="n"/>
@@ -4359,62 +4359,62 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
+          <t>Edinburgh Short Film Festival（第 16 届）</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
+          <t>Edinburgh（多个场地）</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
+          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Club/电子)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>Reel Talk Club</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
+          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
+          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
+          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -4437,17 +4437,17 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>Page Turners Club</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
+          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
+          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -4457,47 +4457,47 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
+          <t>21–31 Oct 2026</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
+          <t>兴趣类(文学/讲故事)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Durham university</t>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>英国知名露天博物馆的年度万圣节夜场；只能网上提前买票，往年经常售罄</t>
+          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.beamish.org.uk/events/halloween-evening-28-oct-2026/ ; https://www.beamish.org.uk/halloween-at-beamish/</t>
+          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>在纽卡斯尔和杜伦中间，两边都能去；有吓人路线，也有不吓人的；年卡在夜场不能用</t>
+          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>同步发 Durham university</t>
+          <t>同步发爱丁堡2校</t>
         </is>
       </c>
       <c r="N52" s="2" t="n"/>
@@ -4515,37 +4515,37 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>Page Turners Club</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Newcastle Racecourse Bonfire Night（夜场赛马 + 烟花）</t>
+          <t>Off the Shelf Festival of Words 2026</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Newcastle Racecourse, High Gosforth Park, Newcastle upon Tyne NE3 5HP</t>
+          <t>Sheffield（市内多个场地）</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>6 Nov 2026（周五）18:00 开门，约 20:30 放烟花</t>
+          <t>9–25 Oct 2026（窗口内为 15–25 Oct）</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/赛马)</t>
+          <t>兴趣类(文学/讲座)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -4555,27 +4555,27 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>赛马场官方年年举办，号称"本地区最大的烟花"（主办方说法）；已开售</t>
+          <t>谢菲尔德官方旅游网站列为"headline event"；年年举办的大型文学节，有数百场活动</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>https://www.newcastle-racecourse.co.uk/popular-events/fireworks</t>
+          <t>https://www.welcometosheffield.co.uk/content/events/off-the-shelf-festival-of-words-2026/</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>早鸟票成人 £9，很便宜；赛马 + 游乐场 + 烟花，一晚玩全套</t>
+          <t>有讲座、朗读、放映，很多场次免费或便宜；由谢菲尔德大学参与主办</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发谢菲尔德2校</t>
         </is>
       </c>
       <c r="N53" s="2" t="n"/>
@@ -4598,12 +4598,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Reverend and The Makers 演唱会</t>
+          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
+          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -4613,12 +4613,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）19:00 开门</t>
+          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立摇滚)</t>
+          <t>年轻人娱乐(Club/电子)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -4628,32 +4628,32 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
+          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
+          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>就在 Northumbria 学生会里，在校生走路就到</t>
+          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Northumbria 优先</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N54" s="2" t="n"/>
@@ -4671,39 +4671,39 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
           <t>Durham university</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
-        </is>
-      </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
           <t>高热度</t>
@@ -4726,12 +4726,12 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发 Durham university</t>
         </is>
       </c>
       <c r="N55" s="2" t="n"/>
@@ -4749,62 +4749,62 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Durham university</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Durham Jazz Festival 2026</t>
+          <t>Newcastle Racecourse Bonfire Night（夜场赛马 + 烟花）</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Gala Theatre / Redhills (Durham Miners' Hall) / Sir Thomas Allen Assembly Rooms 等，Durham</t>
+          <t>Newcastle Racecourse, High Gosforth Park, Newcastle upon Tyne NE3 5HP</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>23–25 Oct 2026</t>
+          <t>6 Nov 2026（周五）18:00 开门，约 20:30 放烟花</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/爵士)</t>
+          <t>年轻人娱乐(烟花/赛马)</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>新办的爵士节（Visit County Durham 报道"新创办"），UK Jazz News 有收录；还没有售票数据</t>
+          <t>赛马场官方年年举办，号称"本地区最大的烟花"（主办方说法）；已开售</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://durhamjazzfestival.co.uk/ ; https://ukjazznews.com/durham-jazz-festival-2026-23-to-26-october/</t>
+          <t>https://www.newcastle-racecourse.co.uk/popular-events/fireworks</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>场地都在杜伦市中心，有酒吧快闪演出，也有剧院大场，门槛可高可低</t>
+          <t>早鸟票成人 £9，很便宜；赛马 + 游乐场 + 烟花，一晚玩全套</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
@@ -4819,6 +4819,864 @@
         </is>
       </c>
       <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Reverend and The Makers 演唱会</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>14 Nov 2026（周六）19:00 开门</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/独立摇滚)</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>就在 Northumbria 学生会里，在校生走路就到</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>第4名</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>Northumbria 优先</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="n"/>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Durham university</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>英国知名露天博物馆的年度万圣节夜场；只能网上提前买票，往年经常售罄</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.beamish.org.uk/events/halloween-evening-28-oct-2026/ ; https://www.beamish.org.uk/halloween-at-beamish/</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>在纽卡斯尔和杜伦中间，两边都能去；有吓人路线，也有不吓人的；年卡在夜场不能用</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="n"/>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Durham university</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Durham Jazz Festival 2026</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Gala Theatre / Redhills (Durham Miners' Hall) / Sir Thomas Allen Assembly Rooms 等，Durham</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>23–25 Oct 2026</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/爵士)</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>新办的爵士节（Visit County Durham 报道"新创办"），UK Jazz News 有收录；还没有售票数据</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>https://durhamjazzfestival.co.uk/ ; https://ukjazznews.com/durham-jazz-festival-2026-23-to-26-october/</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>场地都在杜伦市中心，有酒吧快闪演出，也有剧院大场，门槛可高可低</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="n"/>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Light Night Leeds 2026（主题：A City Speaks）</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Leeds city centre（40 多处装置，Briggate 等）</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>city_only</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>28–29 Oct 2026（周三、周四）18:00–21:30</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>本地生活类(灯光艺术节)</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Leeds 市议会官方确认；号称英国最大的年度灯光艺术节；今年是 Leeds 400 周年的一部分；Yorkshire Evening Post 多次报道</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>https://news.leeds.gov.uk/news/return-of-citys-light-night-will-be-talk-of-the-town-as-it-moves-into-half-term ; https://www.yorkshireeveningpost.co.uk/whats-on/light-night-leeds-2026-briggate-projection-british-library-october-9208998</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>全部免费，40 多个互动装置遍布市中心，下课后顺路就能逛</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="n"/>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Leeds International Film Festival（第 40 届）</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Hyde Park Picture House, 73 Brudenell Road, Leeds LS6 1JD / Everyman Leeds 等多个影院</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>29 Oct – 15 Nov 2026（有来源写 5–22 Nov；主流来源和官方节目时间表都写 29 Oct 开始）</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>电影/媒体</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Reel Talk Club</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>第 40 届，英国历史最悠久的电影节之一；10/1 节目上线、10/8 单片开票（YEP 报道）</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.leedsfilm.com/liff-2026-6ftb ; https://www.yorkshireeveningpost.co.uk/whats-on/arts-and-entertainment/leeds-international-film-festival-2026-opening-films-liff-40th-9021020</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Hyde Park Picture House 就在 Leeds 大学学生区旁边；几乎整个窗口期都有放映</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="n"/>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Embrace 30 周年巡演（嘉宾：The Rolling People / The Bunny Suit）</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>O2 Academy Leeds, 55 Cookridge Street, Leeds LS2 3AW</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>13 Nov 2026（周五）19:00</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Live Music/英伦摇滚)</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Live Music Crew</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Live Nation / Academy Music Group 正式售票；乐队 30 周年新专辑巡演</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.academymusicgroup.com/o2academyleeds/events/embrace-tickets-ae136632 ; https://www.gigsandtours.com/event/embrace/o2-academy-leeds/3605026</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>票价约 £37.70；场馆离 Leeds 大学、Leeds Beckett 都近</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="n"/>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Off the Shelf Festival of Words 2026</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Sheffield（市内多个场地）</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>city_only</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>9–25 Oct 2026（窗口内为 15–25 Oct）</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>兴趣类(文学/讲座)</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Page Turners Club</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德官方旅游网站列为"headline event"；年年举办的大型文学节，有数百场活动</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.welcometosheffield.co.uk/content/events/off-the-shelf-festival-of-words-2026/</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>有讲座、朗读、放映，很多场次免费或便宜；由谢菲尔德大学参与主办</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="n"/>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>ArcNight 2026：谢菲尔德篝火夜烟花</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Don Valley Bowl, Coleridge Road, Sheffield S9 2DF</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>5 Nov 2026（周四）16:00–21:00</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花)</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>新办的活动，由 Illuminate the Gardens 团队主办；Exposed Magazine、Yorkshire Live 报道；票价还没公布</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>https://arcnight.com/ ; https://www.exposedmagazine.co.uk/whats-new/brand-new-bonfire-night-spectacular-to-bring-sheffield-steel-to-the-sky-at-don-valley/</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德唯一的大型烟花，篝火夜正日子；有电车可以到</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="n"/>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Leadmill Fridays 万圣节特别场 @ The Foundry</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>The Foundry, Sheffield Students' Union, Western Bank, Sheffield S10 2TG</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>⚠️万圣节前的周五（推定 30 Oct 2026），活动页没写年份，待核实</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Club/学生夜)</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Study Break Crew</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Leadmill 是谢菲尔德老牌学生夜品牌，主办方说"经常售罄"；在 Skiddle 售票</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>https://leadmill.co.uk/event/leadmill-fridays-halloween-special-at-the-foundry/ ; https://www.skiddle.com/whats-on/Sheffield/halloween-events/</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>专门办给学生的万圣节夜，就在 UoS 学生会里；日期确认后再推</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>UoS 优先；⚠️日期待核实</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="n"/>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Huddersfield Uni Student Hub</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Huddersfield &amp; District Round Table 慈善篝火烟花夜</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>DRAM Centre, Dalton, Huddersfield（与 Moldgreen ARLFC 合办）</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>7 Nov 2026（周六）17:00 开门</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花)</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Yorkshire Live 列入约克郡篝火夜推荐；本地慈善机构年年办；没有售票数据</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>成人 £5，很便宜，离市中心近</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="n"/>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Huddersfield Uni Student Hub</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Mirfield Bonfire &amp; Firework Extravaganza</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Mirfield Showground, Mirfield, West Yorkshire</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>7 Nov 2026（周六）16:00 开门，约 19:30 放烟花</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花/音乐)</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Yorkshire Live 列入约克郡最大篝火夜之一；有音乐舞台和游乐场；没有售票数据</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>离 Huddersfield 约 10 公里，比市内的活动规模大</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="n"/>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P67" s="2" t="inlineStr">
         <is>
           <t>未完成</t>
         </is>
@@ -5110,7 +5968,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -5135,7 +5993,7 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
     </row>
@@ -5206,7 +6064,7 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
     </row>
@@ -5761,15 +6619,15 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第6轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>计划：第6轮 利兹+谢菲尔德+哈德斯菲尔德</t>
+          <t>谢菲尔德同城共用；DocFest 在 6 月，不在窗口内</t>
         </is>
       </c>
     </row>
@@ -5786,15 +6644,15 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第6轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>计划：第6轮 利兹+谢菲尔德+哈德斯菲尔德</t>
+          <t>谢菲尔德同城共用；DocFest 在 6 月，不在窗口内</t>
         </is>
       </c>
     </row>
@@ -6157,15 +7015,15 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第6轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>计划：第6轮 利兹+谢菲尔德+哈德斯菲尔德</t>
+          <t>利兹同城共用，两个群内容完全一样；Roundhay Park 等 6 个市政篝火已被市议会决定停办</t>
         </is>
       </c>
     </row>
@@ -6182,15 +7040,15 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第6轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>计划：第6轮 利兹+谢菲尔德+哈德斯菲尔德</t>
+          <t>利兹同城共用，两个群内容完全一样；Roundhay Park 等 6 个市政篝火已被市议会决定停办</t>
         </is>
       </c>
     </row>
@@ -6207,15 +7065,15 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第6轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>计划：第6轮 利兹+谢菲尔德+哈德斯菲尔德</t>
+          <t>未达 3–5 条：hcmf// 当代音乐节在 11/20–29，不在窗口内；学生会官网只能看到 9 月的活动</t>
         </is>
       </c>
     </row>
@@ -6476,7 +7334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6714,10 +7572,46 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>已停办</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Leeds Roundhay Park 等 6 个市政篝火：市议会已决定停办（Leeds Castle 烟花在肯特郡，跟利兹无关，没收录）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>日期待核实</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Leadmill Fridays 万圣节特别场：活动页没写年份，推定 30 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>日期冲突</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>LIFF：有来源写 5–22 Nov，主流来源写 29 Oct–15 Nov；两种说法都在窗口内</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>窗口提醒</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>BFI 伦敦电影节只有 15–18 Oct 在窗口内；Frieze 在 15–18 Oct，要推得早</t>
         </is>

</xml_diff>

<commit_message>
Add round 7 (Manchester, Lancaster, Lancashire, Chester) to Oct–Nov digest
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_10.15-11.15.xlsx
+++ b/data/UK_Events_TrackB_10.15-11.15.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P67"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2253,17 +2253,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Snack Finds &amp; Picks</t>
+          <t>UK Food Lovers</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Manchester Christmas Markets 2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>Albert Square / Cathedral Gardens / Exchange Square 等，Manchester city centre</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>6 Nov – 22 Dec 2026（Albert Square、Cathedral Gardens 开到 3 Jan 2027；窗口内为 6–15 Nov）</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2293,27 +2293,27 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>年年举办的全英知名圣诞市集，The Manc 报道了 2026 年开市日期和新增点位</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://themanc.com/news/manchester-christmas-markets-2026-opening-date-announced-including-new-spots/ ; https://www.visitmanchester.com/whats-on/whats-on-this-christmas-in-manchester/</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>免费入场，市中心多个点位，逛吃一条龙</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>同步发 UK Food Lovers</t>
+          <t>同步发 The University of Manchester</t>
         </is>
       </c>
       <c r="N24" s="2" t="n"/>
@@ -2331,17 +2331,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies</t>
+          <t>Snack Finds &amp; Picks</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2351,37 +2351,37 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Harper Adams Campus Life; Wolverhampton Freshers Hub 2026</t>
+          <t>UK Food Lovers; 伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>同步发 Harper Adams、Wolverhampton</t>
+          <t>同步发 UK Food Lovers</t>
         </is>
       </c>
       <c r="N25" s="2" t="n"/>
@@ -2409,57 +2409,57 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>Day Trip Buddies</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>MCM Comic Con London（October 2026）</t>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>23–25 Oct 2026</t>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(游戏/动漫/流行文化)</t>
+          <t>年轻人娱乐(烟花) + 一日游</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>The Gaming Corner</t>
+          <t>Harper Adams Campus Life; Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发 Harper Adams、Wolverhampton</t>
         </is>
       </c>
       <c r="N26" s="2" t="n"/>
@@ -2492,12 +2492,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
+          <t>MCM Comic Con London（October 2026）</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
+          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -2507,17 +2507,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
+          <t>23–25 Oct 2026</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>兴趣类(游戏/动漫/流行文化)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Reel Talk Club</t>
+          <t>The Gaming Corner</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2527,22 +2527,22 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
+          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
+          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
+          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -2570,62 +2570,62 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Frieze London &amp; Frieze Masters 2026</t>
+          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>The Regent's Park, London</t>
+          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
+          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(艺术/展览)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
+          <t>Reel Talk Club</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>第3名</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>RCA 优先推</t>
         </is>
       </c>
       <c r="N28" s="2" t="n"/>
@@ -2648,32 +2648,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
+          <t>Frieze London &amp; Frieze Masters 2026</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>The Regent's Park, London</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
+          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐节)</t>
+          <t>兴趣类(艺术/展览)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2683,27 +2683,27 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RCA 优先推</t>
         </is>
       </c>
       <c r="N29" s="2" t="n"/>
@@ -2726,12 +2726,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2741,12 +2741,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>年轻人娱乐(烟花/音乐节)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2761,27 +2761,27 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>第5名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N30" s="2" t="n"/>
@@ -2804,32 +2804,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）11:00–15:30</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(城市传统活动)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2839,27 +2839,27 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>第6名</t>
+          <t>第5名</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>免费</t>
+          <t>RCA Battersea 校区就在旁边</t>
         </is>
       </c>
       <c r="N31" s="2" t="n"/>
@@ -2882,32 +2882,32 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
+          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:30</t>
+          <t>14 Nov 2026（周六）11:00–15:30</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>本地生活类(城市传统活动)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2917,27 +2917,27 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
+          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
+          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
+          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>第7名</t>
+          <t>第6名</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>免费</t>
         </is>
       </c>
       <c r="N32" s="2" t="n"/>
@@ -2955,17 +2955,17 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>St Mary's University, Twickenham</t>
+          <t>伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>英格兰 vs 澳大利亚（Nations Championship 橄榄球）</t>
+          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2975,17 +2975,17 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）</t>
+          <t>31 Oct 2026（周六）18:30</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>运动户外(观赛)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2995,22 +2995,22 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>RFU 官方公布的国家队主场赛，是新赛事 Nations Championship 的首届</t>
+          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship ; https://allianzstadiumtwickenham.com/nations-championship</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>St Mary's 是体育强校，球场就在家门口；⚠️国家队比赛票价偏高</t>
+          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第7名</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>英格兰 vs 日本（Nations Championship 橄榄球）</t>
+          <t>英格兰 vs 澳大利亚（Nations Championship 橄榄球）</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）</t>
+          <t>8 Nov 2026（周日）</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -3073,22 +3073,22 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>RFU 官方公布的国家队主场赛</t>
+          <t>RFU 官方公布的国家队主场赛，是新赛事 Nations Championship 的首届</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship</t>
+          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship ; https://allianzstadiumtwickenham.com/nations-championship</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>对日本这场的票通常比对新西兰、澳大利亚便宜，更适合学生；⚠️票价还是要看一下</t>
+          <t>St Mary's 是体育强校，球场就在家门口；⚠️国家队比赛票价偏高</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
@@ -3116,12 +3116,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>英格兰 vs 日本（Nations Championship 橄榄球）</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>Allianz Stadium Twickenham, 200 Whitton Road, Twickenham TW2 7BA</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -3131,17 +3131,17 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>14 Nov 2026（周六）</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>运动户外(观赛)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew; 伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -3151,22 +3151,22 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>RFU 官方公布的国家队主场赛</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.englandrugby.com/follow/news-and-media/england-fixtures-confirmed-inaugural-nations-championship</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>对日本这场的票通常比对新西兰、澳大利亚便宜，更适合学生；⚠️票价还是要看一下</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Richmond Family Fireworks</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Richmond Athletic Ground, Twickenham Road, Richmond TW9 2SF</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -3209,47 +3209,47 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>⚠️待核实：一个来源写 1 Nov，另一个写 5–7 Nov 2026</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
+          <t>Live Music Crew; 伦敦6校 (UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London)</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>潜在价值</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>年年举办的本地烟花会（Richmond Athletic Association 主办）；2026 年日期各来源说法不一，所以降级</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rag-events.co.uk/major-public-events-at-the-rag/richmond-family-fireworks/ ; https://chiswicktoday.co.uk/chiswick-fireworks-bonfire-night/</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>离 St Mary's 很近；确认日期之后再推</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>第4名</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
-        <is>
-          <t>⚠️日期待核实</t>
         </is>
       </c>
       <c r="N36" s="2" t="n"/>
@@ -3267,67 +3267,67 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Richmond Family Fireworks</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>Richmond Athletic Ground, Twickenham Road, Richmond TW9 2SF</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>⚠️待核实：一个来源写 1 Nov，另一个写 5–7 Nov 2026</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/美食)</t>
+          <t>年轻人娱乐(烟花)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>UK Food Lovers; Snack Finds &amp; Picks</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>年年举办的本地烟花会（Richmond Athletic Association 主办）；2026 年日期各来源说法不一，所以降级</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://www.rag-events.co.uk/major-public-events-at-the-rag/richmond-family-fireworks/ ; https://chiswicktoday.co.uk/chiswick-fireworks-bonfire-night/</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>离 St Mary's 很近；确认日期之后再推</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⚠️日期待核实</t>
         </is>
       </c>
       <c r="N37" s="2" t="n"/>
@@ -3350,12 +3350,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Birmingham Big Wheel &amp; Ice Rink（Centenary Square）</t>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Centenary Square, Birmingham</t>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -3365,42 +3365,42 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>5 Nov 2026 – 3 Jan 2027，每天 10:00–22:00</t>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(滑冰/游乐)</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>UK Food Lovers; Snack Finds &amp; Picks</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>跟圣诞市集同期，市集官方配套项目，年年举办；没有售票数据</t>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>https://www.birmingham-now.co.uk/news/26551457.birmingham-frankfurt-christmas-market-2026---need-know/</t>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>BCU 主校区附近，适合宿舍、群友组团去滑冰</t>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
@@ -3428,32 +3428,32 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Skindred "You Got This" 巡演 伯明翰站</t>
+          <t>Birmingham Big Wheel &amp; Ice Rink（Centenary Square）</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
+          <t>Centenary Square, Birmingham</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>30 Oct 2026（周五）</t>
+          <t>5 Nov 2026 – 3 Jan 2027，每天 10:00–22:00</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>年轻人娱乐(滑冰/游乐)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3463,22 +3463,22 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
+          <t>跟圣诞市集同期，市集官方配套项目，年年举办；没有售票数据</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
+          <t>https://www.birmingham-now.co.uk/news/26551457.birmingham-frankfurt-christmas-market-2026---need-know/</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
+          <t>BCU 主校区附近，适合宿舍、群友组团去滑冰</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
@@ -3501,37 +3501,37 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Harper Adams Campus Life</t>
+          <t>伯明翰3校 (BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life)</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
+          <t>Skindred "You Got This" 巡演 伯明翰站</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
+          <t>30 Oct 2026（周五）</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花) + 一日游</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies; Wolverhampton Freshers Hub 2026</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3541,22 +3541,22 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
+          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
+          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
+          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
@@ -3579,7 +3579,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Wolverhampton Freshers Hub 2026</t>
+          <t>Harper Adams Campus Life</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Day Trip Buddies; Harper Adams Campus Life</t>
+          <t>Day Trip Buddies; Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -3657,17 +3657,17 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>University of Lancaster</t>
+          <t>Wolverhampton Freshers Hub 2026</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Capernwray 湖泊公开水域游泳（Lake Swim）</t>
+          <t>Weston Park Bonfire &amp; Fireworks Night 2026</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -3677,37 +3677,37 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026</t>
+          <t>8 Nov 2026（周日）15:00 开门，17:00 点篝火，18:00 和 19:30 两场烟花</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>运动户外(游泳)</t>
+          <t>年轻人娱乐(烟花) + 一日游</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Swim Wave Tribe</t>
+          <t>Day Trip Buddies; Harper Adams Campus Life</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>仅见于 Outdoor Swimmer 杂志活动日历；主办方未核实（疑为 T2 Events，他们在该场地办过比赛）；无报名数据</t>
+          <t>年年举办的庄园篝火夜，在 See Tickets / Ents24 正规售票，Visit Telford 有收录</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>https://outdoorswimmer.com/events/ ; https://www.t2.events/our-events/capernwray-open-water-swim/</t>
+          <t>https://weston-park.com/bonfire-fireworks-night/ ; https://www.seetickets.com/event/bonfire-fireworks-night-2026/weston-park/3697208</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>窗口内极少数的户外游泳活动，10 月底水温很低，只适合有冷水经验的人；离 Lancaster 大学约 10 公里</t>
+          <t>离 Harper Adams 和 Wolverhampton 都不远；乡村庄园 + 游乐场 + 两场烟花，适合当一日游</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -3735,37 +3735,37 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>The University of Manchester</t>
+          <t>University of Lancaster</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
+          <t>Light Up Lancaster 2026（主题：No Boundaries）</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Islington Mill, James Street, Salford</t>
+          <t>Lancaster city centre（历史建筑和街区）</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:00–24:00</t>
+          <t>5–7 Nov 2026（周四到周六）17:00–22:00</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体 + 社交类(女性)</t>
+          <t>本地生活类(灯光艺术节)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner; Reel Talk Club</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3775,17 +3775,17 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
+          <t>Light Up the North 联盟成员，年年举办；Lancaster BID、Visit Lancashire、Lancaster Guardian、Beyond Radio 都有报道</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
+          <t>https://www.lightuplancaster.co.uk/ ; https://www.beyond.radio/news/local-news/light-up-lancaster-promises-to-illuminate-city-with-no-boundaries/ ; https://www.facebook.com/lightuplancaster/</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
+          <t>免费的灯光艺术路线，连着三晚，下课后去逛正合适</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3813,37 +3813,37 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>The University of Manchester</t>
+          <t>University of Lancaster</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：Season of the Witch 系列活动</t>
+          <t>Capernwray 湖泊公开水域游泳（Lake Swim）</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Manchester 多个场地</t>
+          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
+          <t>31 Oct 2026</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>社交类(女性) + 兴趣类(手工)</t>
+          <t>运动户外(游泳)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner</t>
+          <t>Swim Wave Tribe</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -3853,17 +3853,17 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Manchester's Finest 收录；系列里有 Craft &amp; Coven 手工夜、Pendle 女巫审判主题徒步等；没有单场售票数据</t>
+          <t>仅见于 Outdoor Swimmer 杂志活动日历；主办方未核实（疑为 T2 Events，他们在该场地办过比赛）；无报名数据</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>https://www.manchestersfinest.com/events/girl-gang-mcr-season-of-the-witch/ ; https://girlgangmcr.com/upcoming-events/</t>
+          <t>https://outdoorswimmer.com/events/ ; https://www.t2.events/our-events/capernwray-open-water-swim/</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>窗口内有多场可选；Pendle 徒步的具体日期没搜到，推之前要看官网确认单场日期</t>
+          <t>窗口内极少数的户外游泳活动，10 月底水温很低，只适合有冷水经验的人；离 Lancaster 大学约 10 公里</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -3896,62 +3896,62 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Lonely Girls Club Manchester 活动（10/27 场）</t>
+          <t>Manchester 市政免费烟花夜（Platt Fields / Heaton Park / Wythenshawe Park）</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Manchester（场地待公布）</t>
+          <t>Platt Fields Park, Wilmslow Road, Fallowfield, Manchester M14 6LA（另有 Heaton Park、Wythenshawe Park 两个点）</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>27 Oct 2026（周二）</t>
+          <t>7 Nov 2026（周六）17:00 低噪音场，20:00 主场烟花，之前有灯笼游行</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>社交类(女性交友)</t>
+          <t>年轻人娱乐(烟花)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Girls' Corner</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>成熟的女性交友组织（有 Wikipedia 词条），London+Manchester 成员约 5.5 万（这是社群规模，不代表到场人数）；这场的具体内容官网写"即将公布"</t>
+          <t>Manchester 市议会官方公布：市政烟花 2019 年后首次恢复；三个公园同时办</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>https://www.llgc.co.uk/collections/manchester</t>
+          <t>https://www.manchester.gov.uk/news-stories/2026/free-fireworks-night-events-to-make-spectacular-return-in-manchester</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>票价 £8.95，便宜，专为一个人来交朋友设计；活动内容没公布，推之前再看一眼</t>
+          <t>完全免费；Platt Fields 就在 Fallowfield 学生区，UoM 学生走路就到</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Platt Fields 就在 Fallowfield</t>
         </is>
       </c>
       <c r="N45" s="2" t="n"/>
@@ -3969,17 +3969,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>itison GlasGLOW 2026：Zombie Zoo 万圣节灯光夜游</t>
+          <t>The Warehouse Project 万圣节场：NeXup（Luke Dean、Omar+、Locky 等）</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Glasgow Botanic Gardens, 730 Great Western Road, Glasgow G12 0UE</t>
+          <t>Depot Mayfield, 11 Baring Street, Manchester M1 2PY</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -3989,17 +3989,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>⚠️起始日两种说法：16 Oct 或 24 Oct 开始，1–2 Nov 结束（24 Oct–1 Nov 两种说法都覆盖）</t>
+          <t>31 Oct 2026（周六）20:00–04:00</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(沉浸式/万圣节)</t>
+          <t>年轻人娱乐(Club/House)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -4009,22 +4009,22 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>第 8 年举办；自称英国最大的万圣节活动；往年曾因需求大加售数千张票（Scottish Daily Express 报道）</t>
+          <t>WHP 是 Manchester 办了 20 年的旗舰俱乐部季，场地可容纳 10,000 人；这场在 Ticketmaster 和官网正规售票</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>https://www.itison.com/glasglow ; https://www.glasgowworld.com/news/glasglow-botanic-gardens-dates-5290284 ; https://www.scottishdailyexpress.co.uk/news/scottish-news/glasglow-botanic-gardens-thousands-extra-30877210</t>
+          <t>https://thewarehouseproject.com/calendar/ ; https://www.skiddle.com/news/all/The-Warehouse-Project-2026-everything-you-need-to-know/61707/</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥万圣节季最火的项目，60 分钟沉浸式僵尸主题路线；要分时段买票，热门时段会卖完</t>
+          <t>万圣节夜 Manchester 最有代表性的 club 活动；⚠️WHP 票价通常不低，限 18 岁以上</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
@@ -4047,17 +4047,17 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
+          <t>Manchester Christmas Markets 2026</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
+          <t>Albert Square / Cathedral Gardens / Exchange Square 等，Manchester city centre</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -4067,42 +4067,42 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
+          <t>6 Nov – 22 Dec 2026（Albert Square、Cathedral Gardens 开到 3 Jan 2027；窗口内为 6–15 Nov）</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/金属)</t>
+          <t>本地生活类(集市/美食)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>UK Food Lovers</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
+          <t>年年举办的全英知名圣诞市集，The Manc 报道了 2026 年开市日期和新增点位</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
+          <t>https://themanc.com/news/manchester-christmas-markets-2026-opening-date-announced-including-new-spots/ ; https://www.visitmanchester.com/whats-on/whats-on-this-christmas-in-manchester/</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
+          <t>免费入场，市中心多个点位，逛吃一条龙</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
@@ -4125,37 +4125,37 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
+          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
+          <t>Islington Mill, James Street, Salford</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>13–14 Nov 2026</t>
+          <t>31 Oct 2026（周六）18:00–24:00</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立音乐)</t>
+          <t>电影/媒体 + 社交类(女性)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>Girls' Corner; Reel Talk Club</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -4165,22 +4165,22 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
+          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
+          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
+          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
@@ -4203,62 +4203,62 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh's Christmas 2026（开幕）</t>
+          <t>Girl Gang MCR：Season of the Witch 系列活动</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>East &amp; West Princes Street Gardens / George Street, Edinburgh</t>
+          <t>Manchester 多个场地</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026 – 3 Jan 2027（窗口内只有 14–15 Nov 开幕周末）</t>
+          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(集市/节庆)</t>
+          <t>社交类(女性) + 兴趣类(手工)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Girls' Corner</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡官方冬季节庆，每年举办；免费入场、不用买票</t>
+          <t>Manchester's Finest 收录；系列里有 Craft &amp; Coven 手工夜、Pendle 女巫审判主题徒步等；没有单场售票数据</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>https://edinburgh.org/festivals/edinburghs-christmas/ ; https://edwinterfest.com/edinburgh-christmas/whats-on/traditional-christmas-markets</t>
+          <t>https://www.manchestersfinest.com/events/girl-gang-mcr-season-of-the-witch/ ; https://girlgangmcr.com/upcoming-events/</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>开幕周末可以去；市集免费逛，每天 10:00–22:00</t>
+          <t>窗口内有多场可选；Pendle 徒步的具体日期没搜到，推之前要看官网确认单场日期</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第5名</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
@@ -4281,62 +4281,62 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+          <t>Lonely Girls Club Manchester 活动（10/27 场）</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+          <t>Manchester（场地待公布）</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>21–31 Oct 2026</t>
+          <t>27 Oct 2026（周二）</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(文学/讲故事)</t>
+          <t>社交类(女性交友)</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Page Turners Club</t>
+          <t>Girls' Corner</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
+          <t>成熟的女性交友组织（有 Wikipedia 词条），London+Manchester 成员约 5.5 万（这是社群规模，不代表到场人数）；这场的具体内容官网写"即将公布"</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
+          <t>https://www.llgc.co.uk/collections/manchester</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
+          <t>票价 £8.95，便宜，专为一个人来交朋友设计；活动内容没公布，推之前再看一眼</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第6名</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -4359,62 +4359,62 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh Short Film Festival（第 16 届）</t>
+          <t>itison GlasGLOW 2026：Zombie Zoo 万圣节灯光夜游</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Edinburgh（多个场地）</t>
+          <t>Glasgow Botanic Gardens, 730 Great Western Road, Glasgow G12 0UE</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
+          <t>⚠️起始日两种说法：16 Oct 或 24 Oct 开始，1–2 Nov 结束（24 Oct–1 Nov 两种说法都覆盖）</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>年轻人娱乐(沉浸式/万圣节)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Reel Talk Club</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
+          <t>第 8 年举办；自称英国最大的万圣节活动；往年曾因需求大加售数千张票（Scottish Daily Express 报道）</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
+          <t>https://www.itison.com/glasglow ; https://www.glasgowworld.com/news/glasglow-botanic-gardens-dates-5290284 ; https://www.scottishdailyexpress.co.uk/news/scottish-news/glasglow-botanic-gardens-thousands-extra-30877210</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
+          <t>格拉斯哥万圣节季最火的项目，60 分钟沉浸式僵尸主题路线；要分时段买票，热门时段会卖完</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -4437,37 +4437,37 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Page Turners Club</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>21–31 Oct 2026</t>
+          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(文学/讲故事)</t>
+          <t>年轻人娱乐(Live Music/金属)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -4477,27 +4477,27 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
+          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
+          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
+          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>同步发爱丁堡2校</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N52" s="2" t="n"/>
@@ -4515,37 +4515,37 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Page Turners Club</t>
+          <t>格拉斯哥3校 (Glasgow City College / Glasgow Caledonian University / University of Strathclyde)</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Off the Shelf Festival of Words 2026</t>
+          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Sheffield（市内多个场地）</t>
+          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>9–25 Oct 2026（窗口内为 15–25 Oct）</t>
+          <t>13–14 Nov 2026</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(文学/讲座)</t>
+          <t>年轻人娱乐(Live Music/独立音乐)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -4555,27 +4555,27 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>谢菲尔德官方旅游网站列为"headline event"；年年举办的大型文学节，有数百场活动</t>
+          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>https://www.welcometosheffield.co.uk/content/events/off-the-shelf-festival-of-words-2026/</t>
+          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>有讲座、朗读、放映，很多场次免费或便宜；由谢菲尔德大学参与主办</t>
+          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>同步发谢菲尔德2校</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N53" s="2" t="n"/>
@@ -4593,37 +4593,37 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
+          <t>Edinburgh's Christmas 2026（开幕）</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
+          <t>East &amp; West Princes Street Gardens / George Street, Edinburgh</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
+          <t>14 Nov 2026 – 3 Jan 2027（窗口内只有 14–15 Nov 开幕周末）</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Club/电子)</t>
+          <t>本地生活类(集市/节庆)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -4633,17 +4633,17 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
+          <t>爱丁堡官方冬季节庆，每年举办；免费入场、不用买票</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
+          <t>https://edinburgh.org/festivals/edinburghs-christmas/ ; https://edwinterfest.com/edinburgh-christmas/whats-on/traditional-christmas-markets</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
+          <t>开幕周末可以去；市集免费逛，每天 10:00–22:00</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
@@ -4671,17 +4671,17 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
+          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
+          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -4691,37 +4691,37 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
+          <t>21–31 Oct 2026</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
+          <t>兴趣类(文学/讲故事)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Durham university</t>
+          <t>Page Turners Club</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>英国知名露天博物馆的年度万圣节夜场；只能网上提前买票，往年经常售罄</t>
+          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>https://www.beamish.org.uk/events/halloween-evening-28-oct-2026/ ; https://www.beamish.org.uk/halloween-at-beamish/</t>
+          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>在纽卡斯尔和杜伦中间，两边都能去；有吓人路线，也有不吓人的；年卡在夜场不能用</t>
+          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>同步发 Durham university</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N55" s="2" t="n"/>
@@ -4749,57 +4749,57 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Newcastle Racecourse Bonfire Night（夜场赛马 + 烟花）</t>
+          <t>Edinburgh Short Film Festival（第 16 届）</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Newcastle Racecourse, High Gosforth Park, Newcastle upon Tyne NE3 5HP</t>
+          <t>Edinburgh（多个场地）</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>6 Nov 2026（周五）18:00 开门，约 20:30 放烟花</t>
+          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/赛马)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Reel Talk Club</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>赛马场官方年年举办，号称"本地区最大的烟花"（主办方说法）；已开售</t>
+          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>https://www.newcastle-racecourse.co.uk/popular-events/fireworks</t>
+          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>早鸟票成人 £9，很便宜；赛马 + 游乐场 + 烟花，一晚玩全套</t>
+          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
@@ -4827,17 +4827,17 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>Page Turners Club</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Reverend and The Makers 演唱会</t>
+          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
+          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -4847,17 +4847,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）19:00 开门</t>
+          <t>21–31 Oct 2026</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立摇滚)</t>
+          <t>兴趣类(文学/讲故事)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>爱丁堡2校 (Heriot-Watt University / University of Edinburgh Freshers 2026)</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4867,27 +4867,27 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
+          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
+          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>就在 Northumbria 学生会里，在校生走路就到</t>
+          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>第4名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>Northumbria 优先</t>
+          <t>同步发爱丁堡2校</t>
         </is>
       </c>
       <c r="N57" s="2" t="n"/>
@@ -4905,67 +4905,67 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Durham university</t>
+          <t>Page Turners Club</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
+          <t>Off the Shelf Festival of Words 2026</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
+          <t>Sheffield（市内多个场地）</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
+          <t>9–25 Oct 2026（窗口内为 15–25 Oct）</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
+          <t>兴趣类(文学/讲座)</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
+          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>英国知名露天博物馆的年度万圣节夜场；只能网上提前买票，往年经常售罄</t>
+          <t>谢菲尔德官方旅游网站列为"headline event"；年年举办的大型文学节，有数百场活动</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>https://www.beamish.org.uk/events/halloween-evening-28-oct-2026/ ; https://www.beamish.org.uk/halloween-at-beamish/</t>
+          <t>https://www.welcometosheffield.co.uk/content/events/off-the-shelf-festival-of-words-2026/</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>在纽卡斯尔和杜伦中间，两边都能去；有吓人路线，也有不吓人的；年卡在夜场不能用</t>
+          <t>有讲座、朗读、放映，很多场次免费或便宜；由谢菲尔德大学参与主办</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发谢菲尔德2校</t>
         </is>
       </c>
       <c r="N58" s="2" t="n"/>
@@ -4983,32 +4983,32 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Durham university</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Durham Jazz Festival 2026</t>
+          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Gala Theatre / Redhills (Durham Miners' Hall) / Sir Thomas Allen Assembly Rooms 等，Durham</t>
+          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>23–25 Oct 2026</t>
+          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/爵士)</t>
+          <t>年轻人娱乐(Club/电子)</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -5018,27 +5018,27 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>新办的爵士节（Visit County Durham 报道"新创办"），UK Jazz News 有收录；还没有售票数据</t>
+          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>https://durhamjazzfestival.co.uk/ ; https://ukjazznews.com/durham-jazz-festival-2026-23-to-26-october/</t>
+          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>场地都在杜伦市中心，有酒吧快闪演出，也有剧院大场，门槛可高可低</t>
+          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
@@ -5061,37 +5061,37 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Light Night Leeds 2026（主题：A City Speaks）</t>
+          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Leeds city centre（40 多处装置，Briggate 等）</t>
+          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>28–29 Oct 2026（周三、周四）18:00–21:30</t>
+          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>本地生活类(灯光艺术节)</t>
+          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Durham university</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -5101,27 +5101,27 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Leeds 市议会官方确认；号称英国最大的年度灯光艺术节；今年是 Leeds 400 周年的一部分；Yorkshire Evening Post 多次报道</t>
+          <t>英国知名露天博物馆的年度万圣节夜场；只能网上提前买票，往年经常售罄</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>https://news.leeds.gov.uk/news/return-of-citys-light-night-will-be-talk-of-the-town-as-it-moves-into-half-term ; https://www.yorkshireeveningpost.co.uk/whats-on/light-night-leeds-2026-briggate-projection-british-library-october-9208998</t>
+          <t>https://www.beamish.org.uk/events/halloween-evening-28-oct-2026/ ; https://www.beamish.org.uk/halloween-at-beamish/</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>全部免费，40 多个互动装置遍布市中心，下课后顺路就能逛</t>
+          <t>在纽卡斯尔和杜伦中间，两边都能去；有吓人路线，也有不吓人的；年卡在夜场不能用</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>同步发 Durham university</t>
         </is>
       </c>
       <c r="N60" s="2" t="n"/>
@@ -5139,62 +5139,62 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Leeds International Film Festival（第 40 届）</t>
+          <t>Newcastle Racecourse Bonfire Night（夜场赛马 + 烟花）</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Hyde Park Picture House, 73 Brudenell Road, Leeds LS6 1JD / Everyman Leeds 等多个影院</t>
+          <t>Newcastle Racecourse, High Gosforth Park, Newcastle upon Tyne NE3 5HP</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>29 Oct – 15 Nov 2026（有来源写 5–22 Nov；主流来源和官方节目时间表都写 29 Oct 开始）</t>
+          <t>6 Nov 2026（周五）18:00 开门，约 20:30 放烟花</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>年轻人娱乐(烟花/赛马)</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Reel Talk Club</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>高热度</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>第 40 届，英国历史最悠久的电影节之一；10/1 节目上线、10/8 单片开票（YEP 报道）</t>
+          <t>赛马场官方年年举办，号称"本地区最大的烟花"（主办方说法）；已开售</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>https://www.leedsfilm.com/liff-2026-6ftb ; https://www.yorkshireeveningpost.co.uk/whats-on/arts-and-entertainment/leeds-international-film-festival-2026-opening-films-liff-40th-9021020</t>
+          <t>https://www.newcastle-racecourse.co.uk/popular-events/fireworks</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Hyde Park Picture House 就在 Leeds 大学学生区旁边；几乎整个窗口期都有放映</t>
+          <t>早鸟票成人 £9，很便宜；赛马 + 游乐场 + 烟花，一晚玩全套</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
@@ -5217,17 +5217,17 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Embrace 30 周年巡演（嘉宾：The Rolling People / The Bunny Suit）</t>
+          <t>Reverend and The Makers 演唱会</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>O2 Academy Leeds, 55 Cookridge Street, Leeds LS2 3AW</t>
+          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -5237,12 +5237,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>13 Nov 2026（周五）19:00</t>
+          <t>14 Nov 2026（周六）19:00 开门</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/英伦摇滚)</t>
+          <t>年轻人娱乐(Live Music/独立摇滚)</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -5257,27 +5257,27 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Live Nation / Academy Music Group 正式售票；乐队 30 周年新专辑巡演</t>
+          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>https://www.academymusicgroup.com/o2academyleeds/events/embrace-tickets-ae136632 ; https://www.gigsandtours.com/event/embrace/o2-academy-leeds/3605026</t>
+          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>票价约 £37.70；场馆离 Leeds 大学、Leeds Beckett 都近</t>
+          <t>就在 Northumbria 学生会里，在校生走路就到</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第4名</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Northumbria 优先</t>
         </is>
       </c>
       <c r="N62" s="2" t="n"/>
@@ -5295,57 +5295,57 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+          <t>Durham university</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Off the Shelf Festival of Words 2026</t>
+          <t>Beamish Halloween Evenings："The Un-living Museum of the North"</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Sheffield（市内多个场地）</t>
+          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>9–25 Oct 2026（窗口内为 15–25 Oct）</t>
+          <t>⚠️整季场次说法不一；官网确认有 28 Oct 2026 这一场，其余场次看官网</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>兴趣类(文学/讲座)</t>
+          <t>年轻人娱乐(沉浸式/万圣节) + 一日游</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Page Turners Club</t>
+          <t>纽卡斯尔3群 (Newcastle university / Newcastle university 2 / Northumbria university)</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>谢菲尔德官方旅游网站列为"headline event"；年年举办的大型文学节，有数百场活动</t>
+          <t>英国知名露天博物馆的年度万圣节夜场；只能网上提前买票，往年经常售罄</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>https://www.welcometosheffield.co.uk/content/events/off-the-shelf-festival-of-words-2026/</t>
+          <t>https://www.beamish.org.uk/events/halloween-evening-28-oct-2026/ ; https://www.beamish.org.uk/halloween-at-beamish/</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>有讲座、朗读、放映，很多场次免费或便宜；由谢菲尔德大学参与主办</t>
+          <t>在纽卡斯尔和杜伦中间，两边都能去；有吓人路线，也有不吓人的；年卡在夜场不能用</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
@@ -5373,57 +5373,57 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+          <t>Durham university</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>ArcNight 2026：谢菲尔德篝火夜烟花</t>
+          <t>Durham Jazz Festival 2026</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Don Valley Bowl, Coleridge Road, Sheffield S9 2DF</t>
+          <t>Gala Theatre / Redhills (Durham Miners' Hall) / Sir Thomas Allen Assembly Rooms 等，Durham</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>5 Nov 2026（周四）16:00–21:00</t>
+          <t>23–25 Oct 2026</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花)</t>
+          <t>年轻人娱乐(Live Music/爵士)</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>新办的活动，由 Illuminate the Gardens 团队主办；Exposed Magazine、Yorkshire Live 报道；票价还没公布</t>
+          <t>新办的爵士节（Visit County Durham 报道"新创办"），UK Jazz News 有收录；还没有售票数据</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>https://arcnight.com/ ; https://www.exposedmagazine.co.uk/whats-new/brand-new-bonfire-night-spectacular-to-bring-sheffield-steel-to-the-sky-at-don-valley/</t>
+          <t>https://durhamjazzfestival.co.uk/ ; https://ukjazznews.com/durham-jazz-festival-2026-23-to-26-october/</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>谢菲尔德唯一的大型烟花，篝火夜正日子；有电车可以到</t>
+          <t>场地都在杜伦市中心，有酒吧快闪演出，也有剧院大场，门槛可高可低</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
@@ -5451,67 +5451,67 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Leadmill Fridays 万圣节特别场 @ The Foundry</t>
+          <t>Light Night Leeds 2026（主题：A City Speaks）</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>The Foundry, Sheffield Students' Union, Western Bank, Sheffield S10 2TG</t>
+          <t>Leeds city centre（40 多处装置，Briggate 等）</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>⚠️万圣节前的周五（推定 30 Oct 2026），活动页没写年份，待核实</t>
+          <t>28–29 Oct 2026（周三、周四）18:00–21:30</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Club/学生夜)</t>
+          <t>本地生活类(灯光艺术节)</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Study Break Crew</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>中热度</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Leadmill 是谢菲尔德老牌学生夜品牌，主办方说"经常售罄"；在 Skiddle 售票</t>
+          <t>Leeds 市议会官方确认；号称英国最大的年度灯光艺术节；今年是 Leeds 400 周年的一部分；Yorkshire Evening Post 多次报道</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>https://leadmill.co.uk/event/leadmill-fridays-halloween-special-at-the-foundry/ ; https://www.skiddle.com/whats-on/Sheffield/halloween-events/</t>
+          <t>https://news.leeds.gov.uk/news/return-of-citys-light-night-will-be-talk-of-the-town-as-it-moves-into-half-term ; https://www.yorkshireeveningpost.co.uk/whats-on/light-night-leeds-2026-briggate-projection-british-library-october-9208998</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>专门办给学生的万圣节夜，就在 UoS 学生会里；日期确认后再推</t>
+          <t>全部免费，40 多个互动装置遍布市中心，下课后顺路就能逛</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>第3名</t>
+          <t>第1名</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>UoS 优先；⚠️日期待核实</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N65" s="2" t="n"/>
@@ -5529,17 +5529,17 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Huddersfield Uni Student Hub</t>
+          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Huddersfield &amp; District Round Table 慈善篝火烟花夜</t>
+          <t>Leeds International Film Festival（第 40 届）</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>DRAM Centre, Dalton, Huddersfield（与 Moldgreen ARLFC 合办）</t>
+          <t>Hyde Park Picture House, 73 Brudenell Road, Leeds LS6 1JD / Everyman Leeds 等多个影院</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -5549,42 +5549,42 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>7 Nov 2026（周六）17:00 开门</t>
+          <t>29 Oct – 15 Nov 2026（有来源写 5–22 Nov；主流来源和官方节目时间表都写 29 Oct 开始）</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Reel Talk Club</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>高热度</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Yorkshire Live 列入约克郡篝火夜推荐；本地慈善机构年年办；没有售票数据</t>
+          <t>第 40 届，英国历史最悠久的电影节之一；10/1 节目上线、10/8 单片开票（YEP 报道）</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
+          <t>https://www.leedsfilm.com/liff-2026-6ftb ; https://www.yorkshireeveningpost.co.uk/whats-on/arts-and-entertainment/leeds-international-film-festival-2026-opening-films-liff-40th-9021020</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>成人 £5，很便宜，离市中心近</t>
+          <t>Hyde Park Picture House 就在 Leeds 大学学生区旁边；几乎整个窗口期都有放映</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>第1名</t>
+          <t>第2名</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
@@ -5607,62 +5607,62 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Huddersfield Uni Student Hub</t>
+          <t>利兹2群 (Leeds Uni Student Hub / Leeds University group 2)</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Mirfield Bonfire &amp; Firework Extravaganza</t>
+          <t>Embrace 30 周年巡演（嘉宾：The Rolling People / The Bunny Suit）</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Mirfield Showground, Mirfield, West Yorkshire</t>
+          <t>O2 Academy Leeds, 55 Cookridge Street, Leeds LS2 3AW</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>7 Nov 2026（周六）16:00 开门，约 19:30 放烟花</t>
+          <t>13 Nov 2026（周五）19:00</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>年轻人娱乐(Live Music/英伦摇滚)</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>潜在价值</t>
+          <t>中热度</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Yorkshire Live 列入约克郡最大篝火夜之一；有音乐舞台和游乐场；没有售票数据</t>
+          <t>Live Nation / Academy Music Group 正式售票；乐队 30 周年新专辑巡演</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
+          <t>https://www.academymusicgroup.com/o2academyleeds/events/embrace-tickets-ae136632 ; https://www.gigsandtours.com/event/embrace/o2-academy-leeds/3605026</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>离 Huddersfield 约 10 公里，比市内的活动规模大</t>
+          <t>票价约 £37.70；场馆离 Leeds 大学、Leeds Beckett 都近</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>第2名</t>
+          <t>第3名</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
@@ -5677,6 +5677,474 @@
         </is>
       </c>
       <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Off the Shelf Festival of Words 2026</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Sheffield（市内多个场地）</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>city_only</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>9–25 Oct 2026（窗口内为 15–25 Oct）</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>兴趣类(文学/讲座)</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Page Turners Club</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德官方旅游网站列为"headline event"；年年举办的大型文学节，有数百场活动</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.welcometosheffield.co.uk/content/events/off-the-shelf-festival-of-words-2026/</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>有讲座、朗读、放映，很多场次免费或便宜；由谢菲尔德大学参与主办</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="n"/>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>ArcNight 2026：谢菲尔德篝火夜烟花</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Don Valley Bowl, Coleridge Road, Sheffield S9 2DF</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>5 Nov 2026（周四）16:00–21:00</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花)</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>新办的活动，由 Illuminate the Gardens 团队主办；Exposed Magazine、Yorkshire Live 报道；票价还没公布</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>https://arcnight.com/ ; https://www.exposedmagazine.co.uk/whats-new/brand-new-bonfire-night-spectacular-to-bring-sheffield-steel-to-the-sky-at-don-valley/</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德唯一的大型烟花，篝火夜正日子；有电车可以到</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="n"/>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>谢菲尔德2校 (Sheffield Hallam University / University of Sheffield)</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Leadmill Fridays 万圣节特别场 @ The Foundry</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>The Foundry, Sheffield Students' Union, Western Bank, Sheffield S10 2TG</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>⚠️万圣节前的周五（推定 30 Oct 2026），活动页没写年份，待核实</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(Club/学生夜)</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Study Break Crew</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Leadmill 是谢菲尔德老牌学生夜品牌，主办方说"经常售罄"；在 Skiddle 售票</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>https://leadmill.co.uk/event/leadmill-fridays-halloween-special-at-the-foundry/ ; https://www.skiddle.com/whats-on/Sheffield/halloween-events/</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>专门办给学生的万圣节夜，就在 UoS 学生会里；日期确认后再推</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>第3名</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>UoS 优先；⚠️日期待核实</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="n"/>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Huddersfield Uni Student Hub</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Huddersfield &amp; District Round Table 慈善篝火烟花夜</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>DRAM Centre, Dalton, Huddersfield（与 Moldgreen ARLFC 合办）</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>7 Nov 2026（周六）17:00 开门</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花)</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Yorkshire Live 列入约克郡篝火夜推荐；本地慈善机构年年办；没有售票数据</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>成人 £5，很便宜，离市中心近</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="n"/>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P71" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Huddersfield Uni Student Hub</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Mirfield Bonfire &amp; Firework Extravaganza</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Mirfield Showground, Mirfield, West Yorkshire</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>7 Nov 2026（周六）16:00 开门，约 19:30 放烟花</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花/音乐)</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Yorkshire Live 列入约克郡最大篝火夜之一；有音乐舞台和游乐场；没有售票数据</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.examinerlive.co.uk/whats-on/family-kids-news/bonfire-night-2026-yorkshires-biggest-34659274</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>离 Huddersfield 约 10 公里，比市内的活动规模大</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>第2名</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="n"/>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>University of Chester</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>The Lord Mayor's Spooktacular Fireworks（切斯特赛马场万圣节烟花）</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Chester Racecourse, Watergate Square, Chester CH1 2LY</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>31 Oct 2026（周六）</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(烟花/万圣节)</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>赛马场官方主办，年年举办的市长烟花会，今年提前到万圣节并改成万圣节主题（Chester Standard、Chester Online 报道）</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.chester-races.com/whats-on/the-lord-mayors-spooctacular-fireworks/ ; https://chesteronline.co.uk/chester-fireworks-bonfire-night/</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>市中心赛马场，有游乐设施、踩高跷、火舞表演；是切斯特窗口期内唯一确认的大活动</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>第1名</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="n"/>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="P73" s="2" t="inlineStr">
         <is>
           <t>未完成</t>
         </is>
@@ -6181,7 +6649,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
     </row>
@@ -6769,7 +7237,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第7轮 已搜/无结果</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
@@ -6777,7 +7245,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>计划：第7轮 西北（曼城/兰卡/切斯特）</t>
+          <t>Preston 窗口期内没找到确认过的活动：圣诞亮灯的"Sat 22 Nov"是 2025 年的日期，而且不在窗口内；Guild Hall 还在关闭中；53 Degrees 只找到 10/10 的演出，不在窗口内</t>
         </is>
       </c>
     </row>
@@ -6794,13 +7262,17 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>顺带匹配（没专门搜）</t>
+          <t>第7轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>未达 3–5 条：搜到的 Lancaster 酒吧巡游和 Woman in Black 都是美国宾州 Lancaster 的，没收录</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6815,15 +7287,15 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>第7轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>计划：第7轮 西北（曼城/兰卡/切斯特）</t>
+          <t>未达 3–5 条：圣诞市集 11/18 才开，不在窗口内</t>
         </is>
       </c>
     </row>
@@ -6865,15 +7337,15 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>顺带匹配（没专门搜）</t>
+          <t>第7轮 已搜/有结果</t>
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>都是女性向活动，Manchester 还没专门搜</t>
+          <t>包含第1轮的 3 条女性向活动；Project Halloween（Fatsoma）用了模板宣传语，没收录</t>
         </is>
       </c>
     </row>
@@ -7334,7 +7806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7608,10 +8080,34 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>没收录（模板宣传语）</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Project Halloween（Fatsoma，Manchester / Newcastle 两地）："Biggest Halloween Event / 10,000 People"这类宣传语在多个城市的页面上一字不差，按 skill 规则不当作热度依据；也没有其他独立来源</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>社群空缺</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>University of Lancashire（Preston）：窗口期内没找到确认过的活动，下轮可以试试兰开夏郡范围或 Blackpool</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>窗口提醒</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>BFI 伦敦电影节只有 15–18 Oct 在窗口内；Frieze 在 15–18 Oct，要推得早</t>
         </is>

</xml_diff>

<commit_message>
Close Oct–Nov digest at round 9; mark remaining communities as not searched
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_10.15-11.15.xlsx
+++ b/data/UK_Events_TrackB_10.15-11.15.xlsx
@@ -8005,7 +8005,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -8013,7 +8013,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8055,7 +8055,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -8063,7 +8063,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批；另外该社群本来就缺可靠的带日期信源</t>
+          <t>本期到第 9 轮结束；该社群本来就缺可靠的带日期信源</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8126,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8201,7 +8201,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
@@ -8209,7 +8209,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8272,7 +8272,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
@@ -8280,7 +8280,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
@@ -8305,7 +8305,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
@@ -8372,7 +8372,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8485,7 +8485,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8510,7 +8510,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>计划：第12轮起按兴趣分批</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8735,7 +8735,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
@@ -8743,7 +8743,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>计划：第10轮 中部其余学校</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -8852,7 +8852,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
@@ -8860,7 +8860,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>计划：第10轮 中部其余学校</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -9252,7 +9252,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D53" s="2" t="n">
@@ -9260,7 +9260,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>计划：第11轮 约克+赫尔</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -9352,7 +9352,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D57" s="2" t="n">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>计划：第11轮 约克+赫尔</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>
@@ -9377,7 +9377,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>未搜（留给后续轮次）</t>
+          <t>未搜（用户决定本期不搜）</t>
         </is>
       </c>
       <c r="D58" s="2" t="n">
@@ -9385,7 +9385,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>计划：第10轮 中部其余学校</t>
+          <t>本期到第 9 轮结束</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit Oct–Nov digest and record lessons + output format in skill
Fixes found in the audit: Skindred Glasgow split out of Core. festival (not
in its lineup), Durham Jazz Festival is its second edition, fireworks
nights removed from Live Music Crew, St Fagans price and Skindred
Birmingham ticketing source added.

Skill now documents verification lessons from this run, the cloud
environment limits, EPIC.LAN as an esports source, and the per-community
post-block Excel output format.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_10.15-11.15.xlsx
+++ b/data/UK_Events_TrackB_10.15-11.15.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Track B 30天活动'!$A$1:$O$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'社群覆盖清单'!$A$1:$E$66</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核实与缺口'!$A$1:$B$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核实与缺口'!$A$1:$B$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1201,11 +1201,10 @@
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: MUSIC 👇
-🎆 Ally Pally Fireworks &amp; Drone Festival, London — fireworks, drones and an Eats Everything DJ set, 7–8 Nov.
-🎇 Battersea Park Fireworks, London — fireworks plus a Rudimental DJ set, 7–8 Nov.
 🎃 Skindred Halloween Special, Alexandra Palace — with Alien Ant Farm, Spineshank &amp; Orgy, 31 Oct.
 🎧 Ben Hemsley Halloween Day Rave, Gateshead Stadium — house &amp; trance all day, 2,400+ going (18+), 31 Oct.
-🤘 Core. Festival, Glasgow — heavy music weekend incl. Skindred at the Barrowland, 13–15 Nov.
+🤘 Core. Festival, Glasgow — a heavy-music weekend with Pig Destroyer, Eyehategod &amp; more, 13–15 Nov.
+🎸 Skindred, Barrowland Ballroom, Glasgow — the "You Got This" tour hits a legendary venue, 13 Nov.
 🎸 Pop Mutations x Tiny Changes, Glasgow — an indie weekender across four grassroots venues, 13–14 Nov.
 🤘 Skindred, O2 Academy Birmingham — a rock night on Halloween eve, 30 Oct.
 🎤 Reverend and The Makers, Northumbria SU — a big indie gig right on campus, 14 Nov.
@@ -1214,7 +1213,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
+          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1229,12 +1228,12 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
+          <t>31 Oct 2026（周六）18:30</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐节)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="I10" s="9" t="inlineStr">
@@ -1244,17 +1243,17 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
         </is>
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
         </is>
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -1279,12 +1278,12 @@
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1294,12 +1293,12 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>年轻人娱乐(Club/电子)</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
@@ -1309,22 +1308,22 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
         </is>
       </c>
       <c r="K11" s="8" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
         </is>
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
         <is>
-          <t>UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London；St Mary's University, Twickenham</t>
+          <t>Newcastle university / Newcastle university 2 / Northumbria university</t>
         </is>
       </c>
       <c r="N11" s="8" t="inlineStr">
@@ -1344,52 +1343,52 @@
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
+          <t>Core. 重型音乐节（Pig Destroyer / Eyehategod / Wormrot / Raging Speedhorn 等）</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>Glasgow 多个场地（具体场地看官网和 What's On Glasgow）</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:30</t>
+          <t>13–15 Nov 2026</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>高热度</t>
+          <t>年轻人娱乐(Live Music/金属)</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>中热度</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
+          <t>What's On Glasgow 收录，号称"苏格兰最新的重型音乐节"，今年第二届；阵容里有 Pig Destroyer、Eyehategod 等国际乐队</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
+          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://corepresents.seetickets.com/search/all</t>
         </is>
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
+          <t>金属、硬核爱好者的周末；多个场馆可以串场</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
         <is>
-          <t>UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London</t>
+          <t>Glasgow City College / Glasgow Caledonian University / University of Strathclyde</t>
         </is>
       </c>
       <c r="N12" s="8" t="inlineStr">
@@ -1409,12 +1408,12 @@
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Ben Hemsley 万圣节日场 Rave（with Ewan McVicar）</t>
+          <t>Skindred "You Got This" 巡演 格拉斯哥站</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Gateshead International Stadium, Neilson Road, Gateshead NE10 0EF</t>
+          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -1424,37 +1423,37 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）13:30–23:00，16:00 后停止入场</t>
+          <t>13 Nov 2026（周五）19:00 开门</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Club/电子)</t>
-        </is>
-      </c>
-      <c r="I13" s="9" t="inlineStr">
-        <is>
-          <t>高热度</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>中热度</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>Skiddle 显示"hot seller"、2,448+ 人标记参加（平台实时数字）；机库场地可容纳 6,000 人</t>
+          <t>全英巡演的格拉斯哥站，Visit Glasgow 有收录；和 Core. 音乐节同一个周末，但不属于 Core. 阵容</t>
         </is>
       </c>
       <c r="K13" s="8" t="inlineStr">
         <is>
-          <t>https://www.skiddle.com/whats-on/Gateshead/Gateshead-Stadium/ ; https://www.skiddle.com/artists/Ben-Hemsley-123570182/</t>
+          <t>https://www.visitglasgow.com/events/skindred-13112026-139289 ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>万圣节当天东北部最大的 house / trance 活动之一；限 18 岁以上；地铁可直达</t>
+          <t>Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
         <is>
-          <t>Newcastle university / Newcastle university 2 / Northumbria university</t>
+          <t>Glasgow City College / Glasgow Caledonian University / University of Strathclyde</t>
         </is>
       </c>
       <c r="N13" s="8" t="inlineStr">
@@ -1474,12 +1473,12 @@
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
+          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
+          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1489,12 +1488,12 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
+          <t>13–14 Nov 2026</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/金属)</t>
+          <t>年轻人娱乐(Live Music/独立音乐)</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -1504,17 +1503,17 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
+          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
+          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
+          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -1539,27 +1538,27 @@
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Pop Mutations x Tiny Changes 小型音乐周末</t>
+          <t>Skindred "You Got This" 巡演 伯明翰站</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
+          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>13–14 Nov 2026</t>
+          <t>30 Oct 2026（周五）</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立音乐)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
@@ -1569,22 +1568,22 @@
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>Clash 杂志、VisitScotland 报道；阵容有 Kathryn Joseph、Rozi Plain、The Pastels、Billy Nomates；和心理健康慈善机构 Tiny Changes 合办</t>
+          <t>NME、Kerrang! 报道的全英巡演；See Tickets、Live Nation 正规售票；嘉宾 Alien Ant Farm、Spineshank</t>
         </is>
       </c>
       <c r="K15" s="8" t="inlineStr">
         <is>
-          <t>https://www.clashmusic.com/live/pop-mutations-x-tiny-changes-confirm-intimate-glasgow-weekender ; https://www.popmutations.com/events/pop-mutations-x-tiny-changes</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/o2-academy-birmingham/3619857 ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>独立、小众音乐爱好者的首选，都在市中心小场馆，氛围好，票价通常不高</t>
+          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
         <is>
-          <t>Glasgow City College / Glasgow Caledonian University / University of Strathclyde</t>
+          <t>BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life</t>
         </is>
       </c>
       <c r="N15" s="8" t="inlineStr">
@@ -1604,12 +1603,12 @@
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Skindred "You Got This" 巡演 伯明翰站</t>
+          <t>Reverend and The Makers 演唱会</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>O2 Academy Birmingham, 16–18 Horsefair, Bristol Street, Birmingham B1 1DB</t>
+          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1619,12 +1618,12 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>30 Oct 2026（周五）</t>
+          <t>14 Nov 2026（周六）19:00 开门</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
+          <t>年轻人娱乐(Live Music/独立摇滚)</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
@@ -1634,22 +1633,22 @@
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
+          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
         </is>
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
+          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>万圣节前夜的摇滚场，O2 Academy 就在市中心，BCU 和 SCCB 过去都方便</t>
+          <t>就在 Northumbria 学生会里，在校生走路就到</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
-          <t>BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life</t>
+          <t>Newcastle university / Newcastle university 2 / Northumbria university</t>
         </is>
       </c>
       <c r="N16" s="8" t="inlineStr">
@@ -1669,12 +1668,12 @@
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Reverend and The Makers 演唱会</t>
+          <t>Embrace 30 周年巡演（嘉宾：The Rolling People / The Bunny Suit）</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Northumbria Students' Union, 2 Sandyford Road, Newcastle upon Tyne NE1 8SB</t>
+          <t>O2 Academy Leeds, 55 Cookridge Street, Leeds LS2 3AW</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1684,12 +1683,12 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）19:00 开门</t>
+          <t>13 Nov 2026（周五）19:00</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/独立摇滚)</t>
+          <t>年轻人娱乐(Live Music/英伦摇滚)</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr">
@@ -1699,22 +1698,22 @@
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>SJM Concerts 主办，Ticketmaster / Songkick / Bandsintown 都有正式票务页；成熟乐队巡演</t>
+          <t>Live Nation / Academy Music Group 正式售票；乐队 30 周年新专辑巡演</t>
         </is>
       </c>
       <c r="K17" s="8" t="inlineStr">
         <is>
-          <t>https://www.songkick.com/concerts/43167629-reverend-and-the-makers-at-northumbria-students-union ; https://www.ents24.com/newcastle-upon-tyne-events/northumbria-university-students-union/reverend-and-the-makers/7473947</t>
+          <t>https://www.academymusicgroup.com/o2academyleeds/events/embrace-tickets-ae136632 ; https://www.gigsandtours.com/event/embrace/o2-academy-leeds/3605026</t>
         </is>
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>就在 Northumbria 学生会里，在校生走路就到</t>
+          <t>票价约 £37.70；场馆离 Leeds 大学、Leeds Beckett 都近</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
         <is>
-          <t>Newcastle university / Newcastle university 2 / Northumbria university</t>
+          <t>Leeds Uni Student Hub / Leeds University group 2</t>
         </is>
       </c>
       <c r="N17" s="8" t="inlineStr">
@@ -1729,82 +1728,17 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Embrace 30 周年巡演（嘉宾：The Rolling People / The Bunny Suit）</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>O2 Academy Leeds, 55 Cookridge Street, Leeds LS2 3AW</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>13 Nov 2026（周五）19:00</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(Live Music/英伦摇滚)</t>
-        </is>
-      </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>中热度</t>
-        </is>
-      </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>Live Nation / Academy Music Group 正式售票；乐队 30 周年新专辑巡演</t>
-        </is>
-      </c>
-      <c r="K18" s="8" t="inlineStr">
-        <is>
-          <t>https://www.academymusicgroup.com/o2academyleeds/events/embrace-tickets-ae136632 ; https://www.gigsandtours.com/event/embrace/o2-academy-leeds/3605026</t>
-        </is>
-      </c>
-      <c r="L18" s="8" t="inlineStr">
-        <is>
-          <t>票价约 £37.70；场馆离 Leeds 大学、Leeds Beckett 都近</t>
-        </is>
-      </c>
-      <c r="M18" s="8" t="inlineStr">
-        <is>
-          <t>Leeds Uni Student Hub / Leeds University group 2</t>
-        </is>
-      </c>
-      <c r="N18" s="8" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O18" s="8" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Page Turners Club</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>待制作：Page Turners Club.png</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: BOOKS &amp; STORIES 👇
@@ -1812,29 +1746,94 @@
 📚 Off the Shelf Festival of Words, Sheffield — talks, readings and screenings, to 25 Oct.</t>
         </is>
       </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>21–31 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>兴趣类(文学/讲故事)</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
+        </is>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>Heriot-Watt University / University of Edinburgh Freshers 2026</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="7" t="n"/>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Scottish International Storytelling Festival 2026（主题：Bird &amp; Beast）</t>
+          <t>Off the Shelf Festival of Words 2026</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Scottish Storytelling Centre, 43–45 High Street, Edinburgh EH1 1SR（主场馆 Netherbow Theatre）</t>
+          <t>Sheffield（市内多个场地）</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>21–31 Oct 2026</t>
+          <t>9–25 Oct 2026（窗口内为 15–25 Oct）</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>兴趣类(文学/讲故事)</t>
+          <t>兴趣类(文学/讲座)</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
@@ -1844,22 +1843,22 @@
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>年年举办的国际讲故事节，Edinburgh Festival City 和 Forever Edinburgh 官方都有收录；合作场地有 Royal Botanic Garden、National Library of Scotland</t>
+          <t>谢菲尔德官方旅游网站列为"headline event"；年年举办的大型文学节，有数百场活动</t>
         </is>
       </c>
       <c r="K19" s="8" t="inlineStr">
         <is>
-          <t>https://www.sisf.org.uk/ ; https://www.edinburghfestivalcity.com/festivals/scottish-international-storytelling-festival ; https://theqr.co.uk/2026/09/15/scottish-storytelling-festival-2026-returns-with-bird-beast/</t>
+          <t>https://www.welcometosheffield.co.uk/content/events/off-the-shelf-festival-of-words-2026/</t>
         </is>
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>文学、苏格兰文化爱好者会喜欢；在 Royal Mile 上，很多场次价格不高</t>
+          <t>有讲座、朗读、放映，很多场次免费或便宜；由谢菲尔德大学参与主办</t>
         </is>
       </c>
       <c r="M19" s="8" t="inlineStr">
         <is>
-          <t>Heriot-Watt University / University of Edinburgh Freshers 2026</t>
+          <t>Sheffield Hallam University / University of Sheffield</t>
         </is>
       </c>
       <c r="N19" s="8" t="inlineStr">
@@ -1874,82 +1873,17 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Off the Shelf Festival of Words 2026</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Sheffield（市内多个场地）</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>city_only</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>9–25 Oct 2026（窗口内为 15–25 Oct）</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>兴趣类(文学/讲座)</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>中热度</t>
-        </is>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>谢菲尔德官方旅游网站列为"headline event"；年年举办的大型文学节，有数百场活动</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="inlineStr">
-        <is>
-          <t>https://www.welcometosheffield.co.uk/content/events/off-the-shelf-festival-of-words-2026/</t>
-        </is>
-      </c>
-      <c r="L20" s="8" t="inlineStr">
-        <is>
-          <t>有讲座、朗读、放映，很多场次免费或便宜；由谢菲尔德大学参与主办</t>
-        </is>
-      </c>
-      <c r="M20" s="8" t="inlineStr">
-        <is>
-          <t>Sheffield Hallam University / University of Sheffield</t>
-        </is>
-      </c>
-      <c r="N20" s="8" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O20" s="8" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Reel Talk Club</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>待制作：Reel Talk Club.png</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: FILM 👇
@@ -1960,24 +1894,89 @@
 🎞️ Edinburgh Short Film Festival, Edinburgh — bite-size screenings for film lovers, 6–22 Nov.</t>
         </is>
       </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>电影/媒体</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London</t>
+        </is>
+      </c>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O20" s="8" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="7" t="n"/>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
+          <t>Leeds International Film Festival（第 40 届）</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
+          <t>Hyde Park Picture House, 73 Brudenell Road, Leeds LS6 1JD / Everyman Leeds 等多个影院</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
+          <t>29 Oct – 15 Nov 2026（有来源写 5–22 Nov；主流来源和官方节目时间表都写 29 Oct 开始）</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -1992,22 +1991,22 @@
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
+          <t>第 40 届，英国历史最悠久的电影节之一；10/1 节目上线、10/8 单片开票（YEP 报道）</t>
         </is>
       </c>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
+          <t>https://www.leedsfilm.com/liff-2026-6ftb ; https://www.yorkshireeveningpost.co.uk/whats-on/arts-and-entertainment/leeds-international-film-festival-2026-opening-films-liff-40th-9021020</t>
         </is>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
+          <t>Hyde Park Picture House 就在 Leeds 大学学生区旁边；几乎整个窗口期都有放映</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
         <is>
-          <t>UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London</t>
+          <t>Leeds Uni Student Hub / Leeds University group 2</t>
         </is>
       </c>
       <c r="N21" s="8" t="inlineStr">
@@ -2027,52 +2026,52 @@
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Leeds International Film Festival（第 40 届）</t>
+          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Hyde Park Picture House, 73 Brudenell Road, Leeds LS6 1JD / Everyman Leeds 等多个影院</t>
+          <t>Islington Mill, James Street, Salford</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>29 Oct – 15 Nov 2026（有来源写 5–22 Nov；主流来源和官方节目时间表都写 29 Oct 开始）</t>
+          <t>31 Oct 2026（周六）18:00–24:00</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>高热度</t>
+          <t>电影/媒体 + 社交类(女性)</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>中热度</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>第 40 届，英国历史最悠久的电影节之一；10/1 节目上线、10/8 单片开票（YEP 报道）</t>
+          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
         </is>
       </c>
       <c r="K22" s="8" t="inlineStr">
         <is>
-          <t>https://www.leedsfilm.com/liff-2026-6ftb ; https://www.yorkshireeveningpost.co.uk/whats-on/arts-and-entertainment/leeds-international-film-festival-2026-opening-films-liff-40th-9021020</t>
+          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
         </is>
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>Hyde Park Picture House 就在 Leeds 大学学生区旁边；几乎整个窗口期都有放映</t>
+          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
         <is>
-          <t>Leeds Uni Student Hub / Leeds University group 2</t>
+          <t>Girls' Corner；The University of Manchester</t>
         </is>
       </c>
       <c r="N22" s="8" t="inlineStr">
@@ -2092,27 +2091,27 @@
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Girl Gang MCR：The Craft 30 周年沉浸式放映</t>
+          <t>Iris Prize LGBTQ+ Film Festival 20 周年</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Islington Mill, James Street, Salford</t>
+          <t>Cardiff（多个场地）</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）18:00–24:00</t>
+          <t>12–18 Oct 2026（窗口内为 15–18 Oct；18 Oct 颁奖）</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>电影/媒体 + 社交类(女性)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
@@ -2122,22 +2121,22 @@
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>票务页显示"1/3 Sold"（真实售票信号）；主办方两次获 Film Society of the Year "Best Single Event"</t>
+          <t>第 20 届，Visit Cardiff、Visit Wales 官方收录；Iris Prize 是有影响力的 LGBTQ+ 短片奖</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr">
         <is>
-          <t>https://www.tickettailor.com/events/girlgangmcr/2344142 ; https://girlgangmcr.com/previous-projects/immersive-screenings/</t>
+          <t>https://irisprize.org/ ; https://www.visitcardiff.com/events/iris-prize/</t>
         </is>
       </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>万圣节当晚的女巫主题放映，带 disco 和手工环节，女生结伴去很合适；注意 Girl Gang 受众年龄偏宽（16–80）</t>
+          <t>窗口内有 Best British Day、20 周年庆典、颁奖夜；要推得早</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
         <is>
-          <t>Girls' Corner；The University of Manchester</t>
+          <t>University of Cardiff / Cardiff Metropolitan University</t>
         </is>
       </c>
       <c r="N23" s="8" t="inlineStr">
@@ -2157,12 +2156,12 @@
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Iris Prize LGBTQ+ Film Festival 20 周年</t>
+          <t>Edinburgh Short Film Festival（第 16 届）</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Cardiff（多个场地）</t>
+          <t>Edinburgh（多个场地）</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -2172,7 +2171,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>12–18 Oct 2026（窗口内为 15–18 Oct；18 Oct 颁奖）</t>
+          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -2180,29 +2179,29 @@
           <t>电影/媒体</t>
         </is>
       </c>
-      <c r="I24" s="10" t="inlineStr">
-        <is>
-          <t>中热度</t>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>第 20 届，Visit Cardiff、Visit Wales 官方收录；Iris Prize 是有影响力的 LGBTQ+ 短片奖</t>
+          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
         </is>
       </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>https://irisprize.org/ ; https://www.visitcardiff.com/events/iris-prize/</t>
+          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
         </is>
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>窗口内有 Best British Day、20 周年庆典、颁奖夜；要推得早</t>
+          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
         <is>
-          <t>University of Cardiff / Cardiff Metropolitan University</t>
+          <t>Heriot-Watt University / University of Edinburgh Freshers 2026</t>
         </is>
       </c>
       <c r="N24" s="8" t="inlineStr">
@@ -2217,240 +2216,175 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n"/>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Edinburgh Short Film Festival（第 16 届）</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>Edinburgh（多个场地）</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>city_only</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>6–22 Nov 2026（窗口内为 6–15 Nov）</t>
-        </is>
-      </c>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>电影/媒体</t>
-        </is>
-      </c>
-      <c r="I25" s="11" t="inlineStr">
-        <is>
-          <t>潜在价值</t>
-        </is>
-      </c>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>已办到第 16 届，在 FilmFreeway / Festhome 正规征片；没搜到售票数据</t>
-        </is>
-      </c>
-      <c r="K25" s="8" t="inlineStr">
-        <is>
-          <t>https://filmfreeway.com/EdinburghShortFilmFestival ; https://www.awn.com/event/edinburgh-short-film-festival-2026</t>
-        </is>
-      </c>
-      <c r="L25" s="8" t="inlineStr">
-        <is>
-          <t>短片放映门槛低，适合电影爱好者和传媒专业学生；具体场地和场次要看官网</t>
-        </is>
-      </c>
-      <c r="M25" s="8" t="inlineStr">
-        <is>
-          <t>Heriot-Watt University / University of Edinburgh Freshers 2026</t>
-        </is>
-      </c>
-      <c r="N25" s="8" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O25" s="8" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Snack Finds &amp; Picks</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>待制作：Snack Finds &amp; Picks.png</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: FESTIVE FOOD MARKETS 👇
 🎄 Frankfurt Christmas Market, Birmingham — German food &amp; mulled wine by New Street, from 5 Nov.</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Birmingham's Frankfurt Christmas Market 2026</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G26" s="8" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr">
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>本地生活类(集市/美食)</t>
         </is>
       </c>
-      <c r="I26" s="9" t="inlineStr">
+      <c r="I25" s="9" t="inlineStr">
         <is>
           <t>高热度</t>
         </is>
       </c>
-      <c r="J26" s="8" t="inlineStr">
+      <c r="J25" s="8" t="inlineStr">
         <is>
           <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
         </is>
       </c>
-      <c r="K26" s="8" t="inlineStr">
+      <c r="K25" s="8" t="inlineStr">
         <is>
           <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
         </is>
       </c>
-      <c r="L26" s="8" t="inlineStr">
+      <c r="L25" s="8" t="inlineStr">
         <is>
           <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
         </is>
       </c>
-      <c r="M26" s="8" t="inlineStr">
+      <c r="M25" s="8" t="inlineStr">
         <is>
           <t>UK Food Lovers；BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life</t>
         </is>
       </c>
-      <c r="N26" s="8" t="inlineStr">
+      <c r="N25" s="8" t="inlineStr">
         <is>
           <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
         </is>
       </c>
-      <c r="O26" s="8" t="inlineStr">
+      <c r="O25" s="8" t="inlineStr">
         <is>
           <t>未完成</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Swim Wave Tribe</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>待制作：Swim Wave Tribe.png</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: WILD SWIMMING 👇
 🏊 Capernwray Lake Swim, Carnforth — a late-season open-water swim (cold-water experience needed), 31 Oct.</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Capernwray 湖泊公开水域游泳（Lake Swim）</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G27" s="8" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>31 Oct 2026</t>
         </is>
       </c>
-      <c r="H27" s="8" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>运动户外(游泳)</t>
         </is>
       </c>
-      <c r="I27" s="11" t="inlineStr">
+      <c r="I26" s="11" t="inlineStr">
         <is>
           <t>潜在价值</t>
         </is>
       </c>
-      <c r="J27" s="8" t="inlineStr">
+      <c r="J26" s="8" t="inlineStr">
         <is>
           <t>仅见于 Outdoor Swimmer 杂志活动日历；主办方未核实（疑为 T2 Events，他们在该场地办过比赛）；无报名数据</t>
         </is>
       </c>
-      <c r="K27" s="8" t="inlineStr">
+      <c r="K26" s="8" t="inlineStr">
         <is>
           <t>https://outdoorswimmer.com/events/ ; https://www.t2.events/our-events/capernwray-open-water-swim/</t>
         </is>
       </c>
-      <c r="L27" s="8" t="inlineStr">
+      <c r="L26" s="8" t="inlineStr">
         <is>
           <t>窗口内极少数的户外游泳活动，10 月底水温很低，只适合有冷水经验的人；离 Lancaster 大学约 10 公里</t>
         </is>
       </c>
-      <c r="M27" s="8" t="inlineStr">
+      <c r="M26" s="8" t="inlineStr">
         <is>
           <t>University of Lancaster</t>
         </is>
       </c>
-      <c r="N27" s="8" t="inlineStr">
+      <c r="N26" s="8" t="inlineStr">
         <is>
           <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
         </is>
       </c>
-      <c r="O27" s="8" t="inlineStr">
+      <c r="O26" s="8" t="inlineStr">
         <is>
           <t>未完成</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>UK Food Lovers</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>待制作：UK Food Lovers.png</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: FESTIVE FOOD MARKETS 👇
@@ -2458,14 +2392,79 @@
 🎄 Manchester Christmas Markets, Manchester city centre — the markets are back, free to wander, from 6 Nov.</t>
         </is>
       </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>venue_only</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>本地生活类(集市/美食)</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="inlineStr">
+        <is>
+          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+        </is>
+      </c>
+      <c r="L27" s="8" t="inlineStr">
+        <is>
+          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+        </is>
+      </c>
+      <c r="M27" s="8" t="inlineStr">
+        <is>
+          <t>Snack Finds &amp; Picks；BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life</t>
+        </is>
+      </c>
+      <c r="N27" s="8" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O27" s="8" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="7" t="n"/>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Birmingham's Frankfurt Christmas Market 2026</t>
+          <t>Manchester Christmas Markets 2026</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Victoria Square &amp; New Street（Corporation Street 至 Bullring 段）, Birmingham city centre</t>
+          <t>Albert Square / Cathedral Gardens / Exchange Square 等，Manchester city centre</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -2475,7 +2474,7 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>5 Nov – 24 Dec 2026（窗口内为 5–15 Nov；8 Nov 纪念日星期天 13:00 开）</t>
+          <t>6 Nov – 22 Dec 2026（Albert Square、Cathedral Gardens 开到 3 Jan 2027；窗口内为 6–15 Nov）</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
@@ -2490,22 +2489,22 @@
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>伯明翰市议会官方公布日期；年年举办，号称德国、奥地利以外最大的正宗德式圣诞市集（主办方说法）</t>
+          <t>年年举办的全英知名圣诞市集，The Manc 报道了 2026 年开市日期和新增点位</t>
         </is>
       </c>
       <c r="K28" s="8" t="inlineStr">
         <is>
-          <t>https://www.birmingham.gov.uk/news/article/1841/birminghams_frankfurt_christmas_market_dates_confirmed ; https://thebfcm.co.uk/ ; https://www.centralbid.co.uk/events/birminghams-frankfurt-christmas-market-2026/</t>
+          <t>https://themanc.com/news/manchester-christmas-markets-2026-opening-date-announced-including-new-spots/ ; https://www.visitmanchester.com/whats-on/whats-on-this-christmas-in-manchester/</t>
         </is>
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>免费入场，就在 New Street 站旁，吃喝逛一站搞定</t>
+          <t>免费入场，市中心多个点位，逛吃一条龙</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
         <is>
-          <t>Snack Finds &amp; Picks；BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life</t>
+          <t>The University of Manchester</t>
         </is>
       </c>
       <c r="N28" s="8" t="inlineStr">
@@ -2520,161 +2519,96 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Manchester Christmas Markets 2026</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Albert Square / Cathedral Gardens / Exchange Square 等，Manchester city centre</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>venue_only</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>6 Nov – 22 Dec 2026（Albert Square、Cathedral Gardens 开到 3 Jan 2027；窗口内为 6–15 Nov）</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>本地生活类(集市/美食)</t>
-        </is>
-      </c>
-      <c r="I29" s="9" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>年年举办的全英知名圣诞市集，The Manc 报道了 2026 年开市日期和新增点位</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="inlineStr">
-        <is>
-          <t>https://themanc.com/news/manchester-christmas-markets-2026-opening-date-announced-including-new-spots/ ; https://www.visitmanchester.com/whats-on/whats-on-this-christmas-in-manchester/</t>
-        </is>
-      </c>
-      <c r="L29" s="8" t="inlineStr">
-        <is>
-          <t>免费入场，市中心多个点位，逛吃一条龙</t>
-        </is>
-      </c>
-      <c r="M29" s="8" t="inlineStr">
-        <is>
-          <t>The University of Manchester</t>
-        </is>
-      </c>
-      <c r="N29" s="8" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O29" s="8" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Valorant Riot Crew</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>待制作：Valorant Riot Crew.png</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: VALORANT &amp; LAN 👇
 🎯 EPIC49 LAN, Kettering — 4 days of LAN with a VALORANT tournament (BYOC ticket needed), 29 Oct–1 Nov.</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>EPIC49 LAN Party（含 CS2 / VALORANT / StarCraft II / osu! 锦标赛）</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>Kettering Leisure Village, Kettering, Northamptonshire</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>venue_only</t>
         </is>
       </c>
-      <c r="G30" s="8" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>29 Oct 16:00 – 1 Nov 16:00 2026（锦标赛在 30 Oct – 1 Nov）</t>
         </is>
       </c>
-      <c r="H30" s="8" t="inlineStr">
+      <c r="H29" s="8" t="inlineStr">
         <is>
           <t>年轻人娱乐(电竞/LAN)</t>
         </is>
       </c>
-      <c r="I30" s="9" t="inlineStr">
+      <c r="I29" s="9" t="inlineStr">
         <is>
           <t>高热度</t>
         </is>
       </c>
-      <c r="J30" s="8" t="inlineStr">
+      <c r="J29" s="8" t="inlineStr">
         <is>
           <t>英国老牌 LAN 系列，已办到第 49 届，每年两届；这届 700 个电脑位；官网有 EPIC49 专页，赛事项目包括 CS2 和 VALORANT</t>
         </is>
       </c>
-      <c r="K30" s="8" t="inlineStr">
+      <c r="K29" s="8" t="inlineStr">
         <is>
           <t>https://www.epiclan.co.uk/epic49 ; https://www.yorkshirepudd.co.uk/epic49-kettering-lan/ ; https://esportsinsider.com/2025/07/epic-lan-unveils-dates-for-2026-events</t>
         </is>
       </c>
-      <c r="L30" s="8" t="inlineStr">
+      <c r="L29" s="8" t="inlineStr">
         <is>
           <t>自带电脑参加 4 天 LAN；报比赛必须买 BYOC 票，而且一张票只能报一个项目；万圣节夜有社区派对；票价没核实</t>
         </is>
       </c>
-      <c r="M30" s="8" t="inlineStr">
+      <c r="M29" s="8" t="inlineStr">
         <is>
           <t>The Gaming Corner；CS2 Frag Hub</t>
         </is>
       </c>
-      <c r="N30" s="8" t="inlineStr">
+      <c r="N29" s="8" t="inlineStr">
         <is>
           <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
         </is>
       </c>
-      <c r="O30" s="8" t="inlineStr">
+      <c r="O29" s="8" t="inlineStr">
         <is>
           <t>未完成</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>待制作：UCL Hub.png</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: LONDON &amp; CAMPUS 👇
@@ -2687,14 +2621,79 @@
 🎃 Skindred Halloween Special, Alexandra Palace — with Alien Ant Farm, Spineshank &amp; Orgy, 31 Oct.</t>
         </is>
       </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>MCM Comic Con London（October 2026）</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>23–25 Oct 2026</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>兴趣类(游戏/动漫/流行文化)</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
+        </is>
+      </c>
+      <c r="K30" s="8" t="inlineStr">
+        <is>
+          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
+        </is>
+      </c>
+      <c r="L30" s="8" t="inlineStr">
+        <is>
+          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
+        </is>
+      </c>
+      <c r="M30" s="8" t="inlineStr">
+        <is>
+          <t>The Gaming Corner</t>
+        </is>
+      </c>
+      <c r="N30" s="8" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O30" s="8" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n"/>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="7" t="n"/>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>MCM Comic Con London（October 2026）</t>
+          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>ExCeL London, 1 Western Gateway, Royal Victoria Dock, London E16 1XL</t>
+          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -2704,12 +2703,12 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>23–25 Oct 2026</t>
+          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>兴趣类(游戏/动漫/流行文化)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="I31" s="9" t="inlineStr">
@@ -2719,22 +2718,22 @@
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t>英国最大流行文化展之一，一年两届长期举办；官方已公布 Critical Role 为首批嘉宾</t>
+          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
         </is>
       </c>
       <c r="K31" s="8" t="inlineStr">
         <is>
-          <t>https://www.mcmcomiccon.com/london/en-us/tickets.html ; https://www.excel.london/whats-on/mcm-comic-con-2026 ; https://www.mcmcomiccon.com/global/en-us/blog/gaming/critical-role-guests-mcm-london-october-2026.html</t>
+          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
         </is>
       </c>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>游戏、动漫、cosplay 一站式，年轻人浓度高；ExCeL 在东伦敦，QMUL 过去最方便</t>
+          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
         </is>
       </c>
       <c r="M31" s="8" t="inlineStr">
         <is>
-          <t>The Gaming Corner</t>
+          <t>Reel Talk Club</t>
         </is>
       </c>
       <c r="N31" s="8" t="inlineStr">
@@ -2754,27 +2753,27 @@
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>BFI London Film Festival 第 70 届（最后几天 + 闭幕）</t>
+          <t>Frieze London &amp; Frieze Masters 2026</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>BFI Southbank, Belvedere Road, London SE1 8XT（闭幕式：Royal Festival Hall, Southbank Centre）</t>
+          <t>The Regent's Park, London</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>7–18 Oct 2026（窗口内为 15–18 Oct；闭幕 18 Oct）</t>
+          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>电影/媒体</t>
+          <t>兴趣类(艺术/展览)</t>
         </is>
       </c>
       <c r="I32" s="9" t="inlineStr">
@@ -2784,22 +2783,22 @@
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
-          <t>第 70 届，英国最重要的电影节之一；闭幕片 The Debut（Jesse Eisenberg）英国首映</t>
+          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
         </is>
       </c>
       <c r="K32" s="8" t="inlineStr">
         <is>
-          <t>https://whatson.bfi.org.uk/lff/Online/default.asp ; https://en.wikipedia.org/wiki/2026_BFI_London_Film_Festival</t>
+          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
         </is>
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>大量首映场，有不少普通票价场次；KCL 就在隔壁。窗口只覆盖最后 4 天，要推得早</t>
+          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
         <is>
-          <t>Reel Talk Club</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N32" s="8" t="inlineStr">
@@ -2819,27 +2818,27 @@
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Frieze London &amp; Frieze Masters 2026</t>
+          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>The Regent's Park, London</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>15–18 Oct 2026（公众开放；14 Oct 仅限邀请）</t>
+          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>兴趣类(艺术/展览)</t>
+          <t>年轻人娱乐(烟花/音乐节)</t>
         </is>
       </c>
       <c r="I33" s="9" t="inlineStr">
@@ -2849,17 +2848,17 @@
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>国际一线艺术博览会，每年固定在 Regent's Park 举办</t>
+          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>https://www.frieze.com/fairs/frieze-london-frieze-masters/visitor-information ; https://www.royalparks.org.uk/events/frieze-london-frieze-masters</t>
+          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>艺术生必去；⚠️票价偏高，只能网上买、不能再次入场，推之前查一下有没有学生票</t>
+          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
         </is>
       </c>
       <c r="M33" s="8" t="inlineStr">
@@ -2884,12 +2883,12 @@
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Alexandra Palace Fireworks &amp; Drone Festival</t>
+          <t>Battersea Park Fireworks 2026</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
+          <t>Battersea Park, London SW11 4NJ</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -2899,12 +2898,12 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:00 烟花）/ 8 Nov 2026（周日，18:00 烟花）</t>
+          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐节)</t>
+          <t>年轻人娱乐(烟花/音乐)</t>
         </is>
       </c>
       <c r="I34" s="9" t="inlineStr">
@@ -2914,22 +2913,22 @@
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>伦敦最大的篝火夜活动之一，年年办；Time Out 有专文；周六由 Eats Everything 做 DJ 压轴</t>
+          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>https://www.alexandrapalace.com/whats-on/fireworks-drone-festival/ ; https://www.timeout.com/london/news/alexandra-palace-fireworks-drone-show-2026-details-revealed-091026</t>
+          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
         </is>
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>从 £10.50（早鸟）/ £18 起；周六是成人派对氛围（DJ + 德国啤酒节），适合学生</t>
+          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
         </is>
       </c>
       <c r="M34" s="8" t="inlineStr">
         <is>
-          <t>Live Music Crew</t>
+          <t>St Mary's University, Twickenham</t>
         </is>
       </c>
       <c r="N34" s="8" t="inlineStr">
@@ -2949,27 +2948,27 @@
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Battersea Park Fireworks 2026</t>
+          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Battersea Park, London SW11 4NJ</t>
+          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>7 Nov（周六，20:30 烟花）/ 8 Nov 2026（周日，19:00 烟花）</t>
+          <t>14 Nov 2026（周六）11:00–15:30</t>
         </is>
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/音乐)</t>
+          <t>本地生活类(城市传统活动)</t>
         </is>
       </c>
       <c r="I35" s="9" t="inlineStr">
@@ -2979,22 +2978,22 @@
       </c>
       <c r="J35" s="8" t="inlineStr">
         <is>
-          <t>Wandsworth Council 主办，年年举办；当地媒体称预计再次售罄；周六 Rudimental DJ set</t>
+          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
         </is>
       </c>
       <c r="K35" s="8" t="inlineStr">
         <is>
-          <t>https://www.batterseaparkfireworks.com/ ; https://www.london-now.co.uk/news/26529624.battersea-park-fireworks-2026-tickets-sale-week/</t>
+          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
         </is>
       </c>
       <c r="L35" s="8" t="inlineStr">
         <is>
-          <t>RCA Battersea 校区就在旁边；有 happy hour（游乐设施半价、饮品 £5），学生友好</t>
+          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
         </is>
       </c>
       <c r="M35" s="8" t="inlineStr">
         <is>
-          <t>Live Music Crew；St Mary's University, Twickenham</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N35" s="8" t="inlineStr">
@@ -3014,27 +3013,27 @@
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Lord Mayor's Show 2026（伦敦金融城市长巡游）</t>
+          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
+          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>14 Nov 2026（周六）11:00–15:30</t>
+          <t>31 Oct 2026（周六）18:30</t>
         </is>
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>本地生活类(城市传统活动)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="I36" s="9" t="inlineStr">
@@ -3044,22 +3043,22 @@
       </c>
       <c r="J36" s="8" t="inlineStr">
         <is>
-          <t>数百年历史的年度巡游，官方确认 2026 年日期</t>
+          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
         </is>
       </c>
       <c r="K36" s="8" t="inlineStr">
         <is>
-          <t>https://www.lordmayorsshow.london/ ; https://londonist.com/london/things-to-do/a-guide-to-the-lord-mayor-s-show</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
         </is>
       </c>
       <c r="L36" s="8" t="inlineStr">
         <is>
-          <t>免费、在市中心，留学生能体验很"英国"的传统活动；LSE/KCL 走路就到</t>
+          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
         </is>
       </c>
       <c r="M36" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="N36" s="8" t="inlineStr">
@@ -3074,82 +3073,17 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n"/>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="7" t="n"/>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Skindred 万圣节专场（嘉宾：Alien Ant Farm / Spineshank / Orgy）</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Alexandra Palace, Alexandra Palace Way, London N22 7AY</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G37" s="8" t="inlineStr">
-        <is>
-          <t>31 Oct 2026（周六）18:30</t>
-        </is>
-      </c>
-      <c r="H37" s="8" t="inlineStr">
-        <is>
-          <t>年轻人娱乐(Live Music/摇滚)</t>
-        </is>
-      </c>
-      <c r="I37" s="9" t="inlineStr">
-        <is>
-          <t>高热度</t>
-        </is>
-      </c>
-      <c r="J37" s="8" t="inlineStr">
-        <is>
-          <t>NME、Kerrang! 专门报道的巡演压轴场；在 See Tickets 正规售票；四支乐队同台</t>
-        </is>
-      </c>
-      <c r="K37" s="8" t="inlineStr">
-        <is>
-          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/alexandra-palace/3619860 ; https://www.nme.com/news/music/skindred-announce-2026-uk-and-ireland-tour-with-alien-ant-farm-including-halloween-alexandra-palace-gig-3936573</t>
-        </is>
-      </c>
-      <c r="L37" s="8" t="inlineStr">
-        <is>
-          <t>万圣节夜的 nu-metal 怀旧大场，Ally Pally 场馆有气势</t>
-        </is>
-      </c>
-      <c r="M37" s="8" t="inlineStr">
-        <is>
-          <t>Live Music Crew</t>
-        </is>
-      </c>
-      <c r="N37" s="8" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O37" s="8" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>University of St Andrews</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>待制作：University of St Andrews.png</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: ST ANDREWS 👇
@@ -3159,14 +3093,79 @@
 🎞️ Byre Thursday Films, St Andrews — easy study-break screenings, 29 Oct / 5 &amp; 12 Nov.</t>
         </is>
       </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Alan Carr 单口喜剧巡演 @ Byre Theatre</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>The Byre Theatre, Abbey Street, St Andrews KY16 9LA</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>20 Oct 2026（周二）</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(喜剧)</t>
+        </is>
+      </c>
+      <c r="I37" s="10" t="inlineStr">
+        <is>
+          <t>中热度</t>
+        </is>
+      </c>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>知名喜剧人巡演场；Byre 是 St Andrews 大学主办的剧院，官方活动日历有列出；小剧场，座位少</t>
+        </is>
+      </c>
+      <c r="K37" s="8" t="inlineStr">
+        <is>
+          <t>https://byretheatre.com/upcoming/ ; https://events.st-andrews.ac.uk/event-location/byre/</t>
+        </is>
+      </c>
+      <c r="L37" s="8" t="inlineStr">
+        <is>
+          <t>在小镇能看到一线喜剧人很难得，就在校园边上；座位有限，要早买</t>
+        </is>
+      </c>
+      <c r="M37" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N37" s="8" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O37" s="8" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n"/>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="7" t="n"/>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Alan Carr 单口喜剧巡演 @ Byre Theatre</t>
+          <t>Knockhill Live-Action &amp; Fireworks Spectacular（赛车表演 + 篝火烟花）</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>The Byre Theatre, Abbey Street, St Andrews KY16 9LA</t>
+          <t>Knockhill Racing Circuit, Dunfermline, Fife KY12 9TF</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -3176,12 +3175,12 @@
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>20 Oct 2026（周二）</t>
+          <t>7 Nov 2026（周六）13:00 开门，14:00 赛道表演，约 17:30 放烟花</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(喜剧)</t>
+          <t>年轻人娱乐(烟花/赛车) + 一日游</t>
         </is>
       </c>
       <c r="I38" s="10" t="inlineStr">
@@ -3191,22 +3190,22 @@
       </c>
       <c r="J38" s="8" t="inlineStr">
         <is>
-          <t>知名喜剧人巡演场；Byre 是 St Andrews 大学主办的剧院，官方活动日历有列出；小剧场，座位少</t>
+          <t>苏格兰国家赛车场官方主办，年年举办；烟花由 Edinburgh 21CC Fireworks 制作；What's On Fife 收录</t>
         </is>
       </c>
       <c r="K38" s="8" t="inlineStr">
         <is>
-          <t>https://byretheatre.com/upcoming/ ; https://events.st-andrews.ac.uk/event-location/byre/</t>
+          <t>https://www.knockhill.com/events/fixture-Live-Action-amp-Fireworks-Spectacular-id917 ; https://www.whatsonfife.co.uk/event/078801-live-action-and-fireworks-spectacular-at-knockhill</t>
         </is>
       </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
-          <t>在小镇能看到一线喜剧人很难得，就在校园边上；座位有限，要早买</t>
+          <t>赛车漂移表演 + 烟花，很特别；离 Stirling 约 35 公里、离 St Andrews 约 50 公里，适合组团开车去</t>
         </is>
       </c>
       <c r="M38" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Day Trip Buddies；University of Stirling</t>
         </is>
       </c>
       <c r="N38" s="8" t="inlineStr">
@@ -3226,12 +3225,12 @@
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Knockhill Live-Action &amp; Fireworks Spectacular（赛车表演 + 篝火烟花）</t>
+          <t>Rich Hall 单口喜剧 @ Byre Theatre</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Knockhill Racing Circuit, Dunfermline, Fife KY12 9TF</t>
+          <t>The Byre Theatre, Abbey Street, St Andrews KY16 9LA</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -3241,37 +3240,37 @@
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>7 Nov 2026（周六）13:00 开门，14:00 赛道表演，约 17:30 放烟花</t>
+          <t>23 Oct 2026（周五）</t>
         </is>
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(烟花/赛车) + 一日游</t>
-        </is>
-      </c>
-      <c r="I39" s="10" t="inlineStr">
-        <is>
-          <t>中热度</t>
+          <t>年轻人娱乐(喜剧)</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>潜在价值</t>
         </is>
       </c>
       <c r="J39" s="8" t="inlineStr">
         <is>
-          <t>苏格兰国家赛车场官方主办，年年举办；烟花由 Edinburgh 21CC Fireworks 制作；What's On Fife 收录</t>
+          <t>Byre Theatre 官方节目单有列出；没有售票数据</t>
         </is>
       </c>
       <c r="K39" s="8" t="inlineStr">
         <is>
-          <t>https://www.knockhill.com/events/fixture-Live-Action-amp-Fireworks-Spectacular-id917 ; https://www.whatsonfife.co.uk/event/078801-live-action-and-fireworks-spectacular-at-knockhill</t>
+          <t>https://byretheatre.com/upcoming/</t>
         </is>
       </c>
       <c r="L39" s="8" t="inlineStr">
         <is>
-          <t>赛车漂移表演 + 烟花，很特别；离 Stirling 约 35 公里、离 St Andrews 约 50 公里，适合组团开车去</t>
+          <t>周五晚上的喜剧场，就在校园边上</t>
         </is>
       </c>
       <c r="M39" s="8" t="inlineStr">
         <is>
-          <t>Day Trip Buddies；University of Stirling</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N39" s="8" t="inlineStr">
@@ -3291,7 +3290,7 @@
       <c r="C40" s="7" t="n"/>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Rich Hall 单口喜剧 @ Byre Theatre</t>
+          <t>Byre Theatre 周四电影放映</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -3306,12 +3305,12 @@
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>23 Oct 2026（周五）</t>
+          <t>29 Oct / 5 Nov / 12 Nov 2026（都是周四）</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(喜剧)</t>
+          <t>电影/媒体</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
@@ -3321,17 +3320,17 @@
       </c>
       <c r="J40" s="8" t="inlineStr">
         <is>
-          <t>Byre Theatre 官方节目单有列出；没有售票数据</t>
+          <t>大学剧院固定的放映场，官方节目单有列出</t>
         </is>
       </c>
       <c r="K40" s="8" t="inlineStr">
         <is>
-          <t>https://byretheatre.com/upcoming/</t>
+          <t>https://byretheatre.com/upcoming/film/</t>
         </is>
       </c>
       <c r="L40" s="8" t="inlineStr">
         <is>
-          <t>周五晚上的喜剧场，就在校园边上</t>
+          <t>便宜又方便的学习间隙放松，片单看官网</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
@@ -3351,138 +3350,139 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n"/>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="7" t="n"/>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Byre Theatre 周四电影放映</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>The Byre Theatre, Abbey Street, St Andrews KY16 9LA</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="G41" s="8" t="inlineStr">
-        <is>
-          <t>29 Oct / 5 Nov / 12 Nov 2026（都是周四）</t>
-        </is>
-      </c>
-      <c r="H41" s="8" t="inlineStr">
-        <is>
-          <t>电影/媒体</t>
-        </is>
-      </c>
-      <c r="I41" s="11" t="inlineStr">
-        <is>
-          <t>潜在价值</t>
-        </is>
-      </c>
-      <c r="J41" s="8" t="inlineStr">
-        <is>
-          <t>大学剧院固定的放映场，官方节目单有列出</t>
-        </is>
-      </c>
-      <c r="K41" s="8" t="inlineStr">
-        <is>
-          <t>https://byretheatre.com/upcoming/film/</t>
-        </is>
-      </c>
-      <c r="L41" s="8" t="inlineStr">
-        <is>
-          <t>便宜又方便的学习间隙放松，片单看官网</t>
-        </is>
-      </c>
-      <c r="M41" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N41" s="8" t="inlineStr">
-        <is>
-          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
-        </is>
-      </c>
-      <c r="O41" s="8" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>Glasgow City College / Glasgow Caledonian University / University of Strathclyde</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>待制作：Glasgow City College.png</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: GLASGOW NIGHTS 👇
 🧟 GlasGLOW: Zombie Zoo, Glasgow Botanic Gardens — Glasgow's biggest Halloween light trail, late Oct–1 Nov.
-🤘 Core. Festival, Glasgow — heavy music weekend incl. Skindred at the Barrowland, 13–15 Nov.
+🤘 Core. Festival, Glasgow — a heavy-music weekend with Pig Destroyer, Eyehategod &amp; more, 13–15 Nov.
+🎸 Skindred, Barrowland Ballroom, Glasgow — the "You Got This" tour hits a legendary venue, 13 Nov.
 🎸 Pop Mutations x Tiny Changes, Glasgow — an indie weekender across four grassroots venues, 13–14 Nov.</t>
         </is>
       </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>itison GlasGLOW 2026：Zombie Zoo 万圣节灯光夜游</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Glasgow Botanic Gardens, 730 Great Western Road, Glasgow G12 0UE</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>⚠️起始日两种说法：16 Oct 或 24 Oct 开始，1–2 Nov 结束（24 Oct–1 Nov 两种说法都覆盖）</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>年轻人娱乐(沉浸式/万圣节)</t>
+        </is>
+      </c>
+      <c r="I41" s="9" t="inlineStr">
+        <is>
+          <t>高热度</t>
+        </is>
+      </c>
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>第 8 年举办；自称英国最大的万圣节活动；往年曾因需求大加售数千张票（Scottish Daily Express 报道）</t>
+        </is>
+      </c>
+      <c r="K41" s="8" t="inlineStr">
+        <is>
+          <t>https://www.itison.com/glasglow ; https://www.glasgowworld.com/news/glasglow-botanic-gardens-dates-5290284 ; https://www.scottishdailyexpress.co.uk/news/scottish-news/glasglow-botanic-gardens-thousands-extra-30877210</t>
+        </is>
+      </c>
+      <c r="L41" s="8" t="inlineStr">
+        <is>
+          <t>格拉斯哥万圣节季最火的项目，60 分钟沉浸式僵尸主题路线；要分时段买票，热门时段会卖完</t>
+        </is>
+      </c>
+      <c r="M41" s="8" t="inlineStr">
+        <is>
+          <t>University of West of Scotland</t>
+        </is>
+      </c>
+      <c r="N41" s="8" t="inlineStr">
+        <is>
+          <t>未取图：云端环境出站被拦（WebFetch EGRESS_BLOCKED），需在本地 Claude Code 补</t>
+        </is>
+      </c>
+      <c r="O41" s="8" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n"/>
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="7" t="n"/>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>itison GlasGLOW 2026：Zombie Zoo 万圣节灯光夜游</t>
+          <t>Core. 重型音乐节（Pig Destroyer / Eyehategod / Wormrot / Raging Speedhorn 等）</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Glasgow Botanic Gardens, 730 Great Western Road, Glasgow G12 0UE</t>
+          <t>Glasgow 多个场地（具体场地看官网和 What's On Glasgow）</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>city_only</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>⚠️起始日两种说法：16 Oct 或 24 Oct 开始，1–2 Nov 结束（24 Oct–1 Nov 两种说法都覆盖）</t>
+          <t>13–15 Nov 2026</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(沉浸式/万圣节)</t>
-        </is>
-      </c>
-      <c r="I42" s="9" t="inlineStr">
-        <is>
-          <t>高热度</t>
+          <t>年轻人娱乐(Live Music/金属)</t>
+        </is>
+      </c>
+      <c r="I42" s="10" t="inlineStr">
+        <is>
+          <t>中热度</t>
         </is>
       </c>
       <c r="J42" s="8" t="inlineStr">
         <is>
-          <t>第 8 年举办；自称英国最大的万圣节活动；往年曾因需求大加售数千张票（Scottish Daily Express 报道）</t>
+          <t>What's On Glasgow 收录，号称"苏格兰最新的重型音乐节"，今年第二届；阵容里有 Pig Destroyer、Eyehategod 等国际乐队</t>
         </is>
       </c>
       <c r="K42" s="8" t="inlineStr">
         <is>
-          <t>https://www.itison.com/glasglow ; https://www.glasgowworld.com/news/glasglow-botanic-gardens-dates-5290284 ; https://www.scottishdailyexpress.co.uk/news/scottish-news/glasglow-botanic-gardens-thousands-extra-30877210</t>
+          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://corepresents.seetickets.com/search/all</t>
         </is>
       </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>格拉斯哥万圣节季最火的项目，60 分钟沉浸式僵尸主题路线；要分时段买票，热门时段会卖完</t>
+          <t>金属、硬核爱好者的周末；多个场馆可以串场</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
-          <t>University of West of Scotland</t>
+          <t>Live Music Crew</t>
         </is>
       </c>
       <c r="N42" s="8" t="inlineStr">
@@ -3502,27 +3502,27 @@
       <c r="C43" s="7" t="n"/>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Core. 重型音乐节（含 Skindred @ Barrowland）</t>
+          <t>Skindred "You Got This" 巡演 格拉斯哥站</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT（Skindred 场）；其余场次分布在格拉斯哥多个场地</t>
+          <t>Barrowland Ballroom, 244 Gallowgate, Glasgow G4 0TT</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>13–15 Nov 2026（Skindred：13 Nov 周五 19:00 开门）</t>
+          <t>13 Nov 2026（周五）19:00 开门</t>
         </is>
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>年轻人娱乐(Live Music/金属)</t>
+          <t>年轻人娱乐(Live Music/摇滚)</t>
         </is>
       </c>
       <c r="I43" s="10" t="inlineStr">
@@ -3532,17 +3532,17 @@
       </c>
       <c r="J43" s="8" t="inlineStr">
         <is>
-          <t>What's On Glasgow 收录的"苏格兰最新重型音乐节"，今年第二届；Skindred 是正在英国巡演的成熟乐队，Barrowland 场有独立票务页</t>
+          <t>全英巡演的格拉斯哥站，Visit Glasgow 有收录；和 Core. 音乐节同一个周末，但不属于 Core. 阵容</t>
         </is>
       </c>
       <c r="K43" s="8" t="inlineStr">
         <is>
-          <t>https://www.whatsonglasgow.co.uk/event/118210-core./ ; https://www.visitglasgow.com/events/skindred-13112026-139289</t>
+          <t>https://www.visitglasgow.com/events/skindred-13112026-139289 ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>金属、摇滚爱好者的周末；Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
+          <t>Barrowland 是格拉斯哥的传奇场馆；14 岁以上可入场</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
@@ -4375,12 +4375,12 @@
       </c>
       <c r="J55" s="8" t="inlineStr">
         <is>
-          <t>NME、Kerrang! 报道的全英巡演；成熟乐队，有官方巡演日程</t>
+          <t>NME、Kerrang! 报道的全英巡演；See Tickets、Live Nation 正规售票；嘉宾 Alien Ant Farm、Spineshank</t>
         </is>
       </c>
       <c r="K55" s="8" t="inlineStr">
         <is>
-          <t>https://www.hitthelights.co.uk/tour-news/2026/skindred-uk-tour-dates/ ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
+          <t>https://www.seetickets.com/event/skindred-you-got-this-tour/o2-academy-birmingham/3619857 ; https://www.kerrang.com/skindred-2026-uk-ireland-headline-tour-london-alexandra-palace-alien-ant-farm-spineshank-nu-metal</t>
         </is>
       </c>
       <c r="L55" s="8" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="M60" s="8" t="inlineStr">
         <is>
-          <t>Live Music Crew；UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London</t>
+          <t>UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London</t>
         </is>
       </c>
       <c r="N60" s="8" t="inlineStr">
@@ -5997,7 +5997,7 @@
       </c>
       <c r="J78" s="8" t="inlineStr">
         <is>
-          <t>新办的爵士节（Visit County Durham 报道"新创办"），UK Jazz News 有收录；还没有售票数据</t>
+          <t>2025 年创办，今年第二届；UK Jazz News、Visit County Durham 都有报道；还没有售票数据</t>
         </is>
       </c>
       <c r="K78" s="8" t="inlineStr">
@@ -6609,7 +6609,7 @@
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: CARDIFF 👇
 ⛸️ Cardiff's Winter Wonderland, Cardiff Castle — ice skating in a castle, from 12 Nov.
-🔥 St Fagans Halloween Nights, Cardiff — Welsh folklore and a Wicker Man burning each night, 29–31 Oct.
+🔥 St Fagans Halloween Nights, Cardiff — Welsh folklore and a Wicker Man burning each night, £16, 29–31 Oct.
 🏉 Wales v Japan, Principality Stadium — Nations Championship rugby, 7 Nov.
 🏉 Wales v New Zealand, Principality Stadium — the big one against the All Blacks, 14 Nov.
 🎄 Cardiff Christmas Market, Cardiff city centre — plus a new Victorian market on Queen St (12–15 Nov), from 12 Nov.
@@ -6723,7 +6723,7 @@
       </c>
       <c r="L88" s="8" t="inlineStr">
         <is>
-          <t>威尔士民俗 + 万圣节，还有鬼屋 disco 和游乐场；必须提前买票</t>
+          <t>票价 £16；威尔士民俗 + 万圣节，还有鬼屋 disco 和游乐场；必须提前买票</t>
         </is>
       </c>
       <c r="M88" s="8" t="inlineStr">
@@ -7217,79 +7217,79 @@
   <autoFilter ref="A1:O95"/>
   <mergeCells count="75">
     <mergeCell ref="B53:B55"/>
-    <mergeCell ref="A21:A25"/>
+    <mergeCell ref="B27:B28"/>
     <mergeCell ref="A57:A59"/>
-    <mergeCell ref="C21:C25"/>
+    <mergeCell ref="B18:B19"/>
     <mergeCell ref="C57:C59"/>
     <mergeCell ref="C73:C76"/>
     <mergeCell ref="A60:A63"/>
     <mergeCell ref="A45:A46"/>
     <mergeCell ref="B77:B78"/>
-    <mergeCell ref="C31:C37"/>
+    <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A20:A24"/>
+    <mergeCell ref="B2:B3"/>
     <mergeCell ref="C45:C46"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="A47:A49"/>
     <mergeCell ref="A67:A72"/>
     <mergeCell ref="B84:B86"/>
     <mergeCell ref="B82:B83"/>
-    <mergeCell ref="B10:B18"/>
+    <mergeCell ref="C41:C44"/>
+    <mergeCell ref="A10:A17"/>
+    <mergeCell ref="A79:A81"/>
     <mergeCell ref="A93:A95"/>
     <mergeCell ref="A53:A55"/>
+    <mergeCell ref="A27:A28"/>
     <mergeCell ref="C7:C9"/>
     <mergeCell ref="C53:C55"/>
     <mergeCell ref="A87:A92"/>
     <mergeCell ref="B73:B76"/>
+    <mergeCell ref="B20:B24"/>
+    <mergeCell ref="A41:A44"/>
     <mergeCell ref="B7:B9"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B47:B49"/>
-    <mergeCell ref="A79:A81"/>
+    <mergeCell ref="A37:A40"/>
+    <mergeCell ref="C10:C17"/>
     <mergeCell ref="C2:C3"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A10:A18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C42:C44"/>
+    <mergeCell ref="A18:A19"/>
     <mergeCell ref="B50:B52"/>
+    <mergeCell ref="B67:B72"/>
+    <mergeCell ref="B30:B36"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="B93:B95"/>
     <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B67:B72"/>
     <mergeCell ref="B60:B63"/>
-    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="A73:A76"/>
     <mergeCell ref="A84:A86"/>
     <mergeCell ref="C84:C86"/>
+    <mergeCell ref="C27:C28"/>
     <mergeCell ref="C60:C63"/>
     <mergeCell ref="B64:B65"/>
     <mergeCell ref="C82:C83"/>
+    <mergeCell ref="B37:B40"/>
     <mergeCell ref="B87:B92"/>
-    <mergeCell ref="A31:A37"/>
     <mergeCell ref="A77:A78"/>
-    <mergeCell ref="B93:B95"/>
+    <mergeCell ref="B10:B17"/>
+    <mergeCell ref="A50:A52"/>
     <mergeCell ref="C79:C81"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="A19:A20"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B31:B37"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="A30:A36"/>
+    <mergeCell ref="C50:C52"/>
     <mergeCell ref="B45:B46"/>
-    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="C30:C36"/>
+    <mergeCell ref="B41:B44"/>
     <mergeCell ref="C67:C72"/>
     <mergeCell ref="C93:C95"/>
     <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B21:B25"/>
     <mergeCell ref="B57:B59"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="C20:C24"/>
     <mergeCell ref="C47:C49"/>
-    <mergeCell ref="C28:C29"/>
     <mergeCell ref="A64:A65"/>
     <mergeCell ref="C77:C78"/>
     <mergeCell ref="C64:C65"/>
     <mergeCell ref="C87:C92"/>
+    <mergeCell ref="C37:C40"/>
     <mergeCell ref="A82:A83"/>
-    <mergeCell ref="A73:A76"/>
-    <mergeCell ref="C10:C18"/>
+    <mergeCell ref="C18:C19"/>
     <mergeCell ref="C5:C6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7673,11 +7673,11 @@
         </is>
       </c>
       <c r="D11" s="14" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>都来自城市轮顺带（烟花节 DJ、Skindred 巡演、格拉斯哥音乐节）；还没专门做全国演出轮</t>
+          <t>都来自城市轮顺带（巡演、音乐节、club 活动）；烟花节虽有 DJ，但不算演出，没放进这个群</t>
         </is>
       </c>
     </row>
@@ -9040,7 +9040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9350,17 +9350,53 @@
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
+          <t>已更正</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Core. 音乐节：之前写成"含 Skindred"，其实 Skindred 格拉斯哥站（11/13 Barrowland）是独立巡演，现在拆成两条</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>已更正</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Durham Jazz Festival：之前写"新办"，实际 2025 年创办，今年第二届</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>已更正</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Live Music Crew：去掉了 Ally Pally、Battersea 两个烟花节（有 DJ 但主体是烟花，和 Valorant 群推 CS 内容是同一类错误）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
           <t>窗口提醒</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>BFI 伦敦电影节只有 15–18 Oct 在窗口内；Frieze 在 15–18 Oct，要推得早</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B26"/>
+  <autoFilter ref="A1:B29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Tighten event addresses in Oct–Nov digest; add address rule to skill
Researched venues and postcodes for vague entries (multi-venue festivals
now list main venues, trails and parades list routes or hubs), corrected
the Briarlands Farm location and the Season of the Witch start date, and
logged the three venues that remain unpublished.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_10.15-11.15.xlsx
+++ b/data/UK_Events_TrackB_10.15-11.15.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Track B 30天活动'!$A$1:$O$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'社群覆盖清单'!$A$1:$E$66</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核实与缺口'!$A$1:$B$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核实与缺口'!$A$1:$B$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -632,12 +632,12 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Kettering Leisure Village, Kettering, Northamptonshire</t>
+          <t>Arena Sports, Kettering Leisure Village, Thurston Drive, Kettering NN15 6PB</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
@@ -776,12 +776,12 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Kettering Leisure Village, Kettering, Northamptonshire</t>
+          <t>Arena Sports, Kettering Leisure Village, Thurston Drive, Kettering NN15 6PB</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
@@ -856,12 +856,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal TF11 8LE</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -991,7 +991,7 @@
           <t>🔍 Event Radar (UK) — what's worth doing this month.
 This month: GIRLS' NIGHTS OUT 👇
 🔮 The Craft 30th Anniversary Screening, Salford — an immersive witchy Halloween movie night by Girl Gang, 31 Oct.
-🧹 Season of the Witch, Manchester — Girl Gang's craft nights &amp; witchy events, 4 Oct–22 Nov.
+🧹 Season of the Witch, Manchester — Girl Gang's craft nights &amp; witchy events, to 22 Nov.
 💬 Lonely Girls Club Meet-up, Manchester — a solo-friendly night to make new friends, £8.95, 27 Oct.</t>
         </is>
       </c>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Islington Mill, James Street, Salford</t>
+          <t>Islington Mill, James Street, Salford M3 5HW</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -1067,17 +1067,17 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Manchester 多个场地</t>
+          <t>Manchester 多个场地：Craft &amp; Coven 手工夜在 Cloudwater Taproom；其余场次（含 Pendle 徒步）场地和日期要看 girlgangmcr.com</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
+          <t>22 Sep – 22 Nov 2026（窗口内为 15 Oct – 15 Nov；单场日期见官网）</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Manchester（场地待公布）</t>
+          <t>Manchester（⚠️具体场地报名后才公布，官网没公开）</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1348,12 +1348,12 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Glasgow 多个场地（具体场地看官网和 What's On Glasgow）</t>
+          <t>Glasgow 多个场地：The Art School（20 Scott Street）、Nice N Sleazy（421 Sauchiehall Street）、Garnethill Multicultural Centre、Woodside Hall（11/15 Pig Destroyer 场）</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
+          <t>Glasgow 4 家场馆：The Old Hairdressers（Renfield Lane）、Stereo（Renfield Lane）、Mono（King's Court）、The Glad Café（Pollokshaws Road）</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1818,12 +1818,12 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Sheffield（市内多个场地）</t>
+          <t>Sheffield 多个场地：Montgomery Theatre（27 Surrey Street）、Lyceum Theatre、Firth Hall（University of Sheffield）、Millennium Gallery 等</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Islington Mill, James Street, Salford</t>
+          <t>Islington Mill, James Street, Salford M3 5HW</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -2096,12 +2096,12 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Cardiff（多个场地）</t>
+          <t>Cineworld Cardiff, Mary Ann Street, Cardiff CF10 2EN（主场馆）</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -2161,12 +2161,12 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Edinburgh（多个场地）</t>
+          <t>Filmhouse, 88 Lothian Road, Edinburgh EH3 9BZ / Summerhall, 1 Summerhall, Edinburgh EH9 1PL</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -2319,12 +2319,12 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
+          <t>Capernwray Diving Centre, Jackdaw Quarry, Capernwray Road, Over Kellet, Carnforth LA6 1AD</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -2543,12 +2543,12 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Kettering Leisure Village, Kettering, Northamptonshire</t>
+          <t>Arena Sports, Kettering Leisure Village, Thurston Drive, Kettering NN15 6PB</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>The Regent's Park, London</t>
+          <t>The Regent's Park, London NW1（Frieze London 和 Frieze Masters 两个帐篷都在园内，入口以官网为准）</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>City of London，从 Mansion House 出发（全程约 3 英里）</t>
+          <t>City of London：Mansion House 出发 → Royal Courts of Justice（Strand）→ 返回，沿途都能看</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -3442,12 +3442,12 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Glasgow 多个场地（具体场地看官网和 What's On Glasgow）</t>
+          <t>Glasgow 多个场地：The Art School（20 Scott Street）、Nice N Sleazy（421 Sauchiehall Street）、Garnethill Multicultural Centre、Woodside Hall（11/15 Pig Destroyer 场）</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>The Old Hairdressers / Mono / The Glad Café / Stereo（格拉斯哥 4 家独立场馆）</t>
+          <t>Glasgow 4 家场馆：The Old Hairdressers（Renfield Lane）、Stereo（Renfield Lane）、Mono（King's Court）、The Glad Café（Pollokshaws Road）</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -3717,12 +3717,12 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Paisley town centre（游行路线经过 Mill Street）</t>
+          <t>Paisley town centre：游行走 Smithhills St → Gauze St → Mill St → Bridge St → Cotton St → St Mirren Brae → Causeyside St → Orchard St；街头表演在 County Square，舞台在 Bridge Street 停车场</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
@@ -3928,12 +3928,12 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Edinburgh（多个场地）</t>
+          <t>Filmhouse, 88 Lothian Road, Edinburgh EH3 9BZ / Summerhall, 1 Summerhall, Edinburgh EH9 1PL</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
@@ -4074,12 +4074,12 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Briarlands Farm, Stirling（Cambusbarron / Craigforth 一带，具体地址见官网）</t>
+          <t>Briarlands Farm, Blairdrummond, Stirling FK9 4UP</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
@@ -4429,12 +4429,12 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Weston Park, Weston-under-Lizard, Shifnal, Shropshire</t>
+          <t>Weston Park, Weston-under-Lizard, Shifnal TF11 8LE</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
@@ -4510,12 +4510,12 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Sheffield（市内多个场地）</t>
+          <t>Sheffield 多个场地：Montgomery Theatre（27 Surrey Street）、Lyceum Theatre、Firth Hall（University of Sheffield）、Millennium Gallery 等</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr">
@@ -4997,12 +4997,12 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>Lancaster city centre（历史建筑和街区）</t>
+          <t>Lancaster city centre：Market Square、Dalton Square、The Storey Gardens、Lancaster Castle、Quay Meadow 等（完整地图见 lightuplancaster.co.uk）</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
@@ -5062,12 +5062,12 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Capernwray Dive Centre, Capernwray, Carnforth, Lancashire</t>
+          <t>Capernwray Diving Centre, Jackdaw Quarry, Capernwray Road, Over Kellet, Carnforth LA6 1AD</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G65" s="8" t="inlineStr">
@@ -5214,7 +5214,7 @@
 🎆 Free Council Fireworks, Platt Fields, Fallowfield — lantern parade + fireworks, completely free, 7 Nov.
 🎧 The Warehouse Project Halloween: NeXup, Depot Mayfield — house &amp; tech house till 4am (18+), 31 Oct.
 🔮 The Craft 30th Anniversary Screening, Salford — an immersive witchy Halloween movie night by Girl Gang, 31 Oct.
-🧹 Season of the Witch, Manchester — Girl Gang's craft nights &amp; witchy events, 4 Oct–22 Nov.
+🧹 Season of the Witch, Manchester — Girl Gang's craft nights &amp; witchy events, to 22 Nov.
 💬 Lonely Girls Club Meet-up, Manchester — a solo-friendly night to make new friends, £8.95, 27 Oct.</t>
         </is>
       </c>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Islington Mill, James Street, Salford</t>
+          <t>Islington Mill, James Street, Salford M3 5HW</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
@@ -5485,17 +5485,17 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>Manchester 多个场地</t>
+          <t>Manchester 多个场地：Craft &amp; Coven 手工夜在 Cloudwater Taproom；其余场次（含 Pendle 徒步）场地和日期要看 girlgangmcr.com</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>4 Oct – 22 Nov 2026（单场日期见官网）</t>
+          <t>22 Sep – 22 Nov 2026（窗口内为 15 Oct – 15 Nov；单场日期见官网）</t>
         </is>
       </c>
       <c r="H71" s="8" t="inlineStr">
@@ -5550,7 +5550,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>Manchester（场地待公布）</t>
+          <t>Manchester（⚠️具体场地报名后才公布，官网没公开）</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
+          <t>Beamish Museum, Beamish, County Durham DH9 0RG</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
@@ -5907,7 +5907,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>Beamish Museum, Regional Museums Store, Beamish, County Durham DH9 0RG</t>
+          <t>Beamish Museum, Beamish, County Durham DH9 0RG</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
@@ -5972,7 +5972,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>Gala Theatre / Redhills (Durham Miners' Hall) / Sir Thomas Allen Assembly Rooms 等，Durham</t>
+          <t>Gala Theatre &amp; Gala Studio（Millennium Place, Durham）/ Redhills (Durham Miners' Hall) / Sir Thomas Allen Assembly Rooms / Old Cinema Launderette（Gilesgate）等</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
@@ -6053,17 +6053,17 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Leeds city centre（40 多处装置，Briggate 等）</t>
+          <t>Leeds city centre：信息点在 Millennium Square；主要区域有 Briggate、Town Hall、Corn Exchange、Civic Hall、South Bank（Royal Armouries 一带）</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>venue_only</t>
         </is>
       </c>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t>28–29 Oct 2026（周三、周四）18:00–21:30</t>
+          <t>28–29 Oct 2026（周三、周四）18:00 起（结束时间有 21:30 和 22:00 两种说法）</t>
         </is>
       </c>
       <c r="H79" s="8" t="inlineStr">
@@ -6263,12 +6263,12 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>DRAM Centre, Dalton, Huddersfield（与 Moldgreen ARLFC 合办）</t>
+          <t>DRAM Sport &amp; Community Centre, Ridgeway, Dalton, Huddersfield HD5 9QJ</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
@@ -6328,12 +6328,12 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>Mirfield Showground, Mirfield, West Yorkshire</t>
+          <t>Mirfield Showground, Huddersfield Road, Mirfield WF14 9NE</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>venue_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G83" s="8" t="inlineStr">
@@ -6539,7 +6539,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>Stoke-on-Trent City Centre（Hanley）</t>
+          <t>Hanley city centre, Stoke-on-Trent（City Centre BID 主办；⚠️具体街区官方没写）</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr">
@@ -6549,7 +6549,7 @@
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>31 Oct 2026（周六）10:00 起</t>
+          <t>31 Oct 2026（周六）10:00 起（Facebook 活动页写的日期）</t>
         </is>
       </c>
       <c r="H86" s="8" t="inlineStr">
@@ -6948,12 +6948,12 @@
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>Cardiff（多个场地）</t>
+          <t>Cineworld Cardiff, Mary Ann Street, Cardiff CF10 2EN（主场馆）</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>city_only</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="G92" s="8" t="inlineStr">
@@ -7029,7 +7029,7 @@
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>The Lemon Tree / Cowdray Hall / King's Pavilion 等，Aberdeen &amp; Aberdeenshire</t>
+          <t>Aberdeen &amp; Aberdeenshire 多个场地：The Lemon Tree（5 West North Street, AB24 5AT）、Cowdray Hall、King's Pavilion、Aberdeen Art Gallery、Maritime Museum、Anatomy Rooms，另有一场在前核掩体</t>
         </is>
       </c>
       <c r="F93" s="5" t="inlineStr">
@@ -7159,7 +7159,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>Aberdeen Beach / Beach Boulevard 一带（往年因海滩施工改在 North Pier 燃放）</t>
+          <t>Aberdeen Beach Esplanade 南段观看；往年烟花从 Port of Aberdeen North Pier 尽头燃放（⚠️2026 年的安排还没公布）</t>
         </is>
       </c>
       <c r="F95" s="5" t="inlineStr">
@@ -9040,7 +9040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9386,17 +9386,53 @@
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
+          <t>已更正</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Briarlands Farm：之前写"Cambusbarron / Craigforth 一带"是猜的，实际在 Blairdrummond, FK9 4UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>已更正</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Girl Gang Season of the Witch：整季其实从 22 Sep 开始，不是 4 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>地址未明</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Lonely Girls Club 10/27：场地报名后才公布；Stoke 万圣节街头派对：只知道在 Hanley 市中心；Aberdeen 烟花：2026 年燃放点还没公布</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
           <t>窗口提醒</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>BFI 伦敦电影节只有 15–18 Oct 在窗口内；Frieze 在 15–18 Oct，要推得早</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B29"/>
+  <autoFilter ref="A1:B32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Size post-block rows so the full 发布文案 is visible
Excel does not auto-fit merged cells, so blocks showed only the first
line or two of the post copy. Row heights are now computed from the
wrapped text; the rule is recorded in the skill's output format.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_10.15-11.15.xlsx
+++ b/data/UK_Events_TrackB_10.15-11.15.xlsx
@@ -606,7 +606,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>The Gaming Corner</t>
@@ -686,7 +686,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="5" t="n"/>
       <c r="B3" s="6" t="n"/>
       <c r="C3" s="7" t="n"/>
@@ -751,7 +751,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>CS2 Frag Hub</t>
@@ -830,7 +830,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Day Trip Buddies</t>
@@ -910,7 +910,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="5" t="n"/>
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="7" t="n"/>
@@ -975,7 +975,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="58" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Girls' Corner</t>
@@ -1056,7 +1056,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="58" customHeight="1">
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="7" t="n"/>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="58" customHeight="1">
       <c r="A9" s="5" t="n"/>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="7" t="n"/>
@@ -1186,7 +1186,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="85" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Live Music Crew</t>
@@ -1272,7 +1272,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="58" customHeight="1">
       <c r="A11" s="5" t="n"/>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="7" t="n"/>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="71.5" customHeight="1">
       <c r="A12" s="5" t="n"/>
       <c r="B12" s="6" t="n"/>
       <c r="C12" s="7" t="n"/>
@@ -1402,7 +1402,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="71.5" customHeight="1">
       <c r="A13" s="5" t="n"/>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="7" t="n"/>
@@ -1467,7 +1467,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="58" customHeight="1">
       <c r="A14" s="5" t="n"/>
       <c r="B14" s="6" t="n"/>
       <c r="C14" s="7" t="n"/>
@@ -1532,7 +1532,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="71.5" customHeight="1">
       <c r="A15" s="5" t="n"/>
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="7" t="n"/>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="71.5" customHeight="1">
       <c r="A16" s="5" t="n"/>
       <c r="B16" s="6" t="n"/>
       <c r="C16" s="7" t="n"/>
@@ -1662,7 +1662,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="58" customHeight="1">
       <c r="A17" s="5" t="n"/>
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="7" t="n"/>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="71.5" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Page Turners Club</t>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="58" customHeight="1">
       <c r="A19" s="5" t="n"/>
       <c r="B19" s="6" t="n"/>
       <c r="C19" s="7" t="n"/>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="71.5" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Reel Talk Club</t>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="71.5" customHeight="1">
       <c r="A21" s="5" t="n"/>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="7" t="n"/>
@@ -2020,7 +2020,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="58" customHeight="1">
       <c r="A22" s="5" t="n"/>
       <c r="B22" s="6" t="n"/>
       <c r="C22" s="7" t="n"/>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="58" customHeight="1">
       <c r="A23" s="5" t="n"/>
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="7" t="n"/>
@@ -2150,7 +2150,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="58" customHeight="1">
       <c r="A24" s="5" t="n"/>
       <c r="B24" s="6" t="n"/>
       <c r="C24" s="7" t="n"/>
@@ -2215,7 +2215,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="71.5" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Snack Finds &amp; Picks</t>
@@ -2294,7 +2294,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="73.5" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Swim Wave Tribe</t>
@@ -2373,7 +2373,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="71.5" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>UK Food Lovers</t>
@@ -2453,7 +2453,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="71.5" customHeight="1">
       <c r="A28" s="5" t="n"/>
       <c r="B28" s="6" t="n"/>
       <c r="C28" s="7" t="n"/>
@@ -2518,7 +2518,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="60" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Valorant Riot Crew</t>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="71.5" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>UCL Hub / IC Collective / Royal College of Art / King's College London / London School of Economics / Queen Mary University of London</t>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="58" customHeight="1">
       <c r="A31" s="5" t="n"/>
       <c r="B31" s="6" t="n"/>
       <c r="C31" s="7" t="n"/>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="58" customHeight="1">
       <c r="A32" s="5" t="n"/>
       <c r="B32" s="6" t="n"/>
       <c r="C32" s="7" t="n"/>
@@ -2812,7 +2812,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="58" customHeight="1">
       <c r="A33" s="5" t="n"/>
       <c r="B33" s="6" t="n"/>
       <c r="C33" s="7" t="n"/>
@@ -2877,7 +2877,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="58" customHeight="1">
       <c r="A34" s="5" t="n"/>
       <c r="B34" s="6" t="n"/>
       <c r="C34" s="7" t="n"/>
@@ -2942,7 +2942,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="58" customHeight="1">
       <c r="A35" s="5" t="n"/>
       <c r="B35" s="6" t="n"/>
       <c r="C35" s="7" t="n"/>
@@ -3007,7 +3007,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="85" customHeight="1">
       <c r="A36" s="5" t="n"/>
       <c r="B36" s="6" t="n"/>
       <c r="C36" s="7" t="n"/>
@@ -3072,7 +3072,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="58" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
           <t>University of St Andrews</t>
@@ -3154,7 +3154,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="71.5" customHeight="1">
       <c r="A38" s="5" t="n"/>
       <c r="B38" s="6" t="n"/>
       <c r="C38" s="7" t="n"/>
@@ -3219,7 +3219,7 @@
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="58" customHeight="1">
       <c r="A39" s="5" t="n"/>
       <c r="B39" s="6" t="n"/>
       <c r="C39" s="7" t="n"/>
@@ -3284,7 +3284,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="58" customHeight="1">
       <c r="A40" s="5" t="n"/>
       <c r="B40" s="6" t="n"/>
       <c r="C40" s="7" t="n"/>
@@ -3349,7 +3349,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="71.5" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
           <t>Glasgow City College / Glasgow Caledonian University / University of Strathclyde</t>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="71.5" customHeight="1">
       <c r="A42" s="5" t="n"/>
       <c r="B42" s="6" t="n"/>
       <c r="C42" s="7" t="n"/>
@@ -3496,7 +3496,7 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="71.5" customHeight="1">
       <c r="A43" s="5" t="n"/>
       <c r="B43" s="6" t="n"/>
       <c r="C43" s="7" t="n"/>
@@ -3561,7 +3561,7 @@
         </is>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="58" customHeight="1">
       <c r="A44" s="5" t="n"/>
       <c r="B44" s="6" t="n"/>
       <c r="C44" s="7" t="n"/>
@@ -3626,7 +3626,7 @@
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="71.5" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
           <t>University of West of Scotland</t>
@@ -3706,7 +3706,7 @@
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="71.5" customHeight="1">
       <c r="A46" s="5" t="n"/>
       <c r="B46" s="6" t="n"/>
       <c r="C46" s="7" t="n"/>
@@ -3771,7 +3771,7 @@
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="58" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
           <t>Heriot-Watt University / University of Edinburgh Freshers 2026</t>
@@ -3852,7 +3852,7 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="71.5" customHeight="1">
       <c r="A48" s="5" t="n"/>
       <c r="B48" s="6" t="n"/>
       <c r="C48" s="7" t="n"/>
@@ -3917,7 +3917,7 @@
         </is>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="58" customHeight="1">
       <c r="A49" s="5" t="n"/>
       <c r="B49" s="6" t="n"/>
       <c r="C49" s="7" t="n"/>
@@ -3982,7 +3982,7 @@
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="71.5" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
         <is>
           <t>University of Stirling</t>
@@ -4063,7 +4063,7 @@
         </is>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="58" customHeight="1">
       <c r="A51" s="5" t="n"/>
       <c r="B51" s="6" t="n"/>
       <c r="C51" s="7" t="n"/>
@@ -4128,7 +4128,7 @@
         </is>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="58" customHeight="1">
       <c r="A52" s="5" t="n"/>
       <c r="B52" s="6" t="n"/>
       <c r="C52" s="7" t="n"/>
@@ -4193,7 +4193,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="71.5" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
           <t>BCU Fresher Hub 2026 / Aston Fresher Hub 2026 / SCCB| Birmingham Student Life</t>
@@ -4274,7 +4274,7 @@
         </is>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="58" customHeight="1">
       <c r="A54" s="5" t="n"/>
       <c r="B54" s="6" t="n"/>
       <c r="C54" s="7" t="n"/>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="71.5" customHeight="1">
       <c r="A55" s="5" t="n"/>
       <c r="B55" s="6" t="n"/>
       <c r="C55" s="7" t="n"/>
@@ -4404,7 +4404,7 @@
         </is>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="60" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
           <t>Wolverhampton Freshers Hub 2026 / Harper Adams Campus Life</t>
@@ -4483,7 +4483,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="58" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
           <t>Sheffield Hallam University / University of Sheffield</t>
@@ -4564,7 +4564,7 @@
         </is>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="58" customHeight="1">
       <c r="A58" s="5" t="n"/>
       <c r="B58" s="6" t="n"/>
       <c r="C58" s="7" t="n"/>
@@ -4629,7 +4629,7 @@
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="58" customHeight="1">
       <c r="A59" s="5" t="n"/>
       <c r="B59" s="6" t="n"/>
       <c r="C59" s="7" t="n"/>
@@ -4694,7 +4694,7 @@
         </is>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="71.5" customHeight="1">
       <c r="A60" s="5" t="inlineStr">
         <is>
           <t>St Mary's University, Twickenham</t>
@@ -4776,7 +4776,7 @@
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="58" customHeight="1">
       <c r="A61" s="5" t="n"/>
       <c r="B61" s="6" t="n"/>
       <c r="C61" s="7" t="n"/>
@@ -4841,7 +4841,7 @@
         </is>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="58" customHeight="1">
       <c r="A62" s="5" t="n"/>
       <c r="B62" s="6" t="n"/>
       <c r="C62" s="7" t="n"/>
@@ -4906,7 +4906,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="58" customHeight="1">
       <c r="A63" s="5" t="n"/>
       <c r="B63" s="6" t="n"/>
       <c r="C63" s="7" t="n"/>
@@ -4971,7 +4971,7 @@
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="71.5" customHeight="1">
       <c r="A64" s="5" t="inlineStr">
         <is>
           <t>University of Lancaster</t>
@@ -5051,7 +5051,7 @@
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="58" customHeight="1">
       <c r="A65" s="5" t="n"/>
       <c r="B65" s="6" t="n"/>
       <c r="C65" s="7" t="n"/>
@@ -5116,7 +5116,7 @@
         </is>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="73.5" customHeight="1">
       <c r="A66" s="5" t="inlineStr">
         <is>
           <t>University of Chester</t>
@@ -5195,7 +5195,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="71.5" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
           <t>The University of Manchester</t>
@@ -5279,7 +5279,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="58" customHeight="1">
       <c r="A68" s="5" t="n"/>
       <c r="B68" s="6" t="n"/>
       <c r="C68" s="7" t="n"/>
@@ -5344,7 +5344,7 @@
         </is>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="58" customHeight="1">
       <c r="A69" s="5" t="n"/>
       <c r="B69" s="6" t="n"/>
       <c r="C69" s="7" t="n"/>
@@ -5409,7 +5409,7 @@
         </is>
       </c>
     </row>
-    <row r="70">
+    <row r="70" ht="58" customHeight="1">
       <c r="A70" s="5" t="n"/>
       <c r="B70" s="6" t="n"/>
       <c r="C70" s="7" t="n"/>
@@ -5474,7 +5474,7 @@
         </is>
       </c>
     </row>
-    <row r="71">
+    <row r="71" ht="58" customHeight="1">
       <c r="A71" s="5" t="n"/>
       <c r="B71" s="6" t="n"/>
       <c r="C71" s="7" t="n"/>
@@ -5539,7 +5539,7 @@
         </is>
       </c>
     </row>
-    <row r="72">
+    <row r="72" ht="58" customHeight="1">
       <c r="A72" s="5" t="n"/>
       <c r="B72" s="6" t="n"/>
       <c r="C72" s="7" t="n"/>
@@ -5604,7 +5604,7 @@
         </is>
       </c>
     </row>
-    <row r="73">
+    <row r="73" ht="58" customHeight="1">
       <c r="A73" s="5" t="inlineStr">
         <is>
           <t>Newcastle university / Newcastle university 2 / Northumbria university</t>
@@ -5686,7 +5686,7 @@
         </is>
       </c>
     </row>
-    <row r="74">
+    <row r="74" ht="58" customHeight="1">
       <c r="A74" s="5" t="n"/>
       <c r="B74" s="6" t="n"/>
       <c r="C74" s="7" t="n"/>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
     </row>
-    <row r="75">
+    <row r="75" ht="58" customHeight="1">
       <c r="A75" s="5" t="n"/>
       <c r="B75" s="6" t="n"/>
       <c r="C75" s="7" t="n"/>
@@ -5816,7 +5816,7 @@
         </is>
       </c>
     </row>
-    <row r="76">
+    <row r="76" ht="71.5" customHeight="1">
       <c r="A76" s="5" t="n"/>
       <c r="B76" s="6" t="n"/>
       <c r="C76" s="7" t="n"/>
@@ -5881,7 +5881,7 @@
         </is>
       </c>
     </row>
-    <row r="77">
+    <row r="77" ht="58" customHeight="1">
       <c r="A77" s="5" t="inlineStr">
         <is>
           <t>Durham university</t>
@@ -5961,7 +5961,7 @@
         </is>
       </c>
     </row>
-    <row r="78">
+    <row r="78" ht="71.5" customHeight="1">
       <c r="A78" s="5" t="n"/>
       <c r="B78" s="6" t="n"/>
       <c r="C78" s="7" t="n"/>
@@ -6026,7 +6026,7 @@
         </is>
       </c>
     </row>
-    <row r="79">
+    <row r="79" ht="85" customHeight="1">
       <c r="A79" s="5" t="inlineStr">
         <is>
           <t>Leeds Uni Student Hub / Leeds University group 2</t>
@@ -6107,7 +6107,7 @@
         </is>
       </c>
     </row>
-    <row r="80">
+    <row r="80" ht="71.5" customHeight="1">
       <c r="A80" s="5" t="n"/>
       <c r="B80" s="6" t="n"/>
       <c r="C80" s="7" t="n"/>
@@ -6172,7 +6172,7 @@
         </is>
       </c>
     </row>
-    <row r="81">
+    <row r="81" ht="58" customHeight="1">
       <c r="A81" s="5" t="n"/>
       <c r="B81" s="6" t="n"/>
       <c r="C81" s="7" t="n"/>
@@ -6237,7 +6237,7 @@
         </is>
       </c>
     </row>
-    <row r="82">
+    <row r="82" ht="58" customHeight="1">
       <c r="A82" s="5" t="inlineStr">
         <is>
           <t>Huddersfield Uni Student Hub</t>
@@ -6317,7 +6317,7 @@
         </is>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="58" customHeight="1">
       <c r="A83" s="5" t="n"/>
       <c r="B83" s="6" t="n"/>
       <c r="C83" s="7" t="n"/>
@@ -6382,7 +6382,7 @@
         </is>
       </c>
     </row>
-    <row r="84">
+    <row r="84" ht="58" customHeight="1">
       <c r="A84" s="5" t="inlineStr">
         <is>
           <t>Staffs Student Life | Stoke / Keele Campus Life</t>
@@ -6463,7 +6463,7 @@
         </is>
       </c>
     </row>
-    <row r="85">
+    <row r="85" ht="58" customHeight="1">
       <c r="A85" s="5" t="n"/>
       <c r="B85" s="6" t="n"/>
       <c r="C85" s="7" t="n"/>
@@ -6528,7 +6528,7 @@
         </is>
       </c>
     </row>
-    <row r="86">
+    <row r="86" ht="58" customHeight="1">
       <c r="A86" s="5" t="n"/>
       <c r="B86" s="6" t="n"/>
       <c r="C86" s="7" t="n"/>
@@ -6593,7 +6593,7 @@
         </is>
       </c>
     </row>
-    <row r="87">
+    <row r="87" ht="58" customHeight="1">
       <c r="A87" s="5" t="inlineStr">
         <is>
           <t>University of Cardiff / Cardiff Metropolitan University</t>
@@ -6677,7 +6677,7 @@
         </is>
       </c>
     </row>
-    <row r="88">
+    <row r="88" ht="58" customHeight="1">
       <c r="A88" s="5" t="n"/>
       <c r="B88" s="6" t="n"/>
       <c r="C88" s="7" t="n"/>
@@ -6742,7 +6742,7 @@
         </is>
       </c>
     </row>
-    <row r="89">
+    <row r="89" ht="71.5" customHeight="1">
       <c r="A89" s="5" t="n"/>
       <c r="B89" s="6" t="n"/>
       <c r="C89" s="7" t="n"/>
@@ -6807,7 +6807,7 @@
         </is>
       </c>
     </row>
-    <row r="90">
+    <row r="90" ht="58" customHeight="1">
       <c r="A90" s="5" t="n"/>
       <c r="B90" s="6" t="n"/>
       <c r="C90" s="7" t="n"/>
@@ -6872,7 +6872,7 @@
         </is>
       </c>
     </row>
-    <row r="91">
+    <row r="91" ht="58" customHeight="1">
       <c r="A91" s="5" t="n"/>
       <c r="B91" s="6" t="n"/>
       <c r="C91" s="7" t="n"/>
@@ -6937,7 +6937,7 @@
         </is>
       </c>
     </row>
-    <row r="92">
+    <row r="92" ht="58" customHeight="1">
       <c r="A92" s="5" t="n"/>
       <c r="B92" s="6" t="n"/>
       <c r="C92" s="7" t="n"/>
@@ -7002,7 +7002,7 @@
         </is>
       </c>
     </row>
-    <row r="93">
+    <row r="93" ht="71.5" customHeight="1">
       <c r="A93" s="5" t="inlineStr">
         <is>
           <t>University of Aberdeen Freshers 2026</t>
@@ -7083,7 +7083,7 @@
         </is>
       </c>
     </row>
-    <row r="94">
+    <row r="94" ht="71.5" customHeight="1">
       <c r="A94" s="5" t="n"/>
       <c r="B94" s="6" t="n"/>
       <c r="C94" s="7" t="n"/>
@@ -7148,7 +7148,7 @@
         </is>
       </c>
     </row>
-    <row r="95">
+    <row r="95" ht="58" customHeight="1">
       <c r="A95" s="5" t="n"/>
       <c r="B95" s="6" t="n"/>
       <c r="C95" s="7" t="n"/>

</xml_diff>

<commit_message>
Fix venue addresses found in postcode audit; tighten skill address rule
hmv Empire Coventry is 22 Hertford Street CV1 1LF and WWT Slimbridge is
Bowditch GL2 7BT (both had been written from memory). Add verified
postcodes for Martin Mere, Lido Ponty and Utilita Arena Cardiff; drop an
unverified Summerhall postcode. Every other venue postcode in the
November digest was checked against official or multiple sources.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015EcMbQsiuHSK5T5ZfDf7k5
</commit_message>
<xml_diff>
--- a/data/UK_Events_TrackB_10.15-11.15.xlsx
+++ b/data/UK_Events_TrackB_10.15-11.15.xlsx
@@ -2161,7 +2161,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Filmhouse, 88 Lothian Road, Edinburgh EH3 9BZ / Summerhall, 1 Summerhall, Edinburgh EH9 1PL</t>
+          <t>Filmhouse, 88 Lothian Road, Edinburgh EH3 9BZ / Summerhall, Edinburgh</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Filmhouse, 88 Lothian Road, Edinburgh EH3 9BZ / Summerhall, 1 Summerhall, Edinburgh EH9 1PL</t>
+          <t>Filmhouse, 88 Lothian Road, Edinburgh EH3 9BZ / Summerhall, Edinburgh</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">

</xml_diff>